<commit_message>
Simplify Dashboard: 2 charts (Profit After Tax + Cumulative Cash), remove Total Revenue KPI
- KEY METRICS: keep Cumulative Cash and Profit After Tax, remove Total Revenue row
- Charts: replace 3 original charts with Profit After Tax and Cumulative Cash (3 scenarios each)
- Rename Net Result → Profit After Tax
- Sheet protection preserved (password: 2027)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -353,70 +353,38 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
+          <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1800" b="1" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
+              <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:rPr>
-              <a:t>Total Revenue (10-Year)</a:t>
+              <a:t>Profit After Tax (10-Year)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
     </title>
     <plotArea>
       <lineChart>
         <grouping val="standard"/>
-        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <strRef>
-              <f>"Base"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Base</v>
-                </pt>
-              </strCache>
-            </strRef>
+            <v>Base</v>
           </tx>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="4a7ebb"/>
-            </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="28000">
               <a:solidFill>
-                <a:srgbClr val="4a7ebb"/>
+                <a:srgbClr val="1F4E79"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
-              <a:round/>
             </a:ln>
           </spPr>
           <marker>
@@ -428,121 +396,19 @@
             </spPr>
           </marker>
           <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
             <showCatName val="0"/>
             <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
           </dLbls>
           <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
+            <numRef>
+              <f>'Dashboard'!$B$11:$K$11</f>
+            </numRef>
           </cat>
           <val>
             <numRef>
-              <f>Dashboard!$B$15:$K$15</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>152310.75</v>
-                </pt>
-                <pt idx="1">
-                  <v>201895.25</v>
-                </pt>
-                <pt idx="2">
-                  <v>244282.79</v>
-                </pt>
-                <pt idx="3">
-                  <v>291142.5388</v>
-                </pt>
-                <pt idx="4">
-                  <v>326552.765456</v>
-                </pt>
-                <pt idx="5">
-                  <v>349118.08528032</v>
-                </pt>
-                <pt idx="6">
-                  <v>364729.275681734</v>
-                </pt>
-                <pt idx="7">
-                  <v>388930.420639009</v>
-                </pt>
-                <pt idx="8">
-                  <v>414018.103513176</v>
-                </pt>
-                <pt idx="9">
-                  <v>440041.551205681</v>
-                </pt>
-              </numCache>
+              <f>'Dashboard'!$B$19:$K$19</f>
             </numRef>
           </val>
           <smooth val="1"/>
@@ -551,26 +417,156 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <strRef>
-              <f>"Downside"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Downside</v>
-                </pt>
-              </strCache>
-            </strRef>
+            <v>Downside</v>
           </tx>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="be4b48"/>
-            </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="20000">
               <a:solidFill>
-                <a:srgbClr val="be4b48"/>
+                <a:srgbClr val="C62828"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$B$11:$K$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$31:$K$31</f>
+            </numRef>
+          </val>
+          <smooth val="1"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Upside</v>
+          </tx>
+          <spPr>
+            <a:ln w="20000">
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$B$11:$K$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$43:$K$43</f>
+            </numRef>
+          </val>
+          <smooth val="1"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>CHF</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crossesAt val="0"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumulative Cash (10-Year)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Base</v>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
-              <a:round/>
             </a:ln>
           </spPr>
           <marker>
@@ -582,149 +578,35 @@
             </spPr>
           </marker>
           <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
             <showCatName val="0"/>
             <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
           </dLbls>
           <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
+            <numRef>
+              <f>'Dashboard'!$B$11:$K$11</f>
+            </numRef>
           </cat>
           <val>
             <numRef>
-              <f>Dashboard!$B$27:$K$27</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>116467</v>
-                </pt>
-                <pt idx="1">
-                  <v>149172</v>
-                </pt>
-                <pt idx="2">
-                  <v>177669.68</v>
-                </pt>
-                <pt idx="3">
-                  <v>210520.38</v>
-                </pt>
-                <pt idx="4">
-                  <v>235761.720304</v>
-                </pt>
-                <pt idx="5">
-                  <v>253331.39832224</v>
-                </pt>
-                <pt idx="6">
-                  <v>263665.281245331</v>
-                </pt>
-                <pt idx="7">
-                  <v>282291.27602515</v>
-                </pt>
-                <pt idx="8">
-                  <v>301488.847290762</v>
-                </pt>
-                <pt idx="9">
-                  <v>321289.10616093</v>
-                </pt>
-              </numCache>
+              <f>'Dashboard'!$B$20:$K$20</f>
             </numRef>
           </val>
           <smooth val="1"/>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="1"/>
+          <order val="1"/>
           <tx>
-            <strRef>
-              <f>"Upside"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Upside</v>
-                </pt>
-              </strCache>
-            </strRef>
+            <v>Downside</v>
           </tx>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="98b855"/>
-            </a:solidFill>
-            <a:ln w="47520">
+            <a:ln w="20000">
               <a:solidFill>
-                <a:srgbClr val="98b855"/>
+                <a:srgbClr val="C62828"/>
               </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
+              <a:prstDash val="dash"/>
             </a:ln>
           </spPr>
           <marker>
@@ -735,1116 +617,30 @@
               </a:ln>
             </spPr>
           </marker>
-          <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
-          </dLbls>
           <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
+            <numRef>
+              <f>'Dashboard'!$B$11:$K$11</f>
+            </numRef>
           </cat>
           <val>
             <numRef>
-              <f>Dashboard!$B$39:$K$39</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>161610.75</v>
-                </pt>
-                <pt idx="1">
-                  <v>218945.25</v>
-                </pt>
-                <pt idx="2">
-                  <v>267532.79</v>
-                </pt>
-                <pt idx="3">
-                  <v>320592.5388</v>
-                </pt>
-                <pt idx="4">
-                  <v>360652.765456</v>
-                </pt>
-                <pt idx="5">
-                  <v>385264.08528032</v>
-                </pt>
-                <pt idx="6">
-                  <v>403044.035681734</v>
-                </pt>
-                <pt idx="7">
-                  <v>429544.06623901</v>
-                </pt>
-                <pt idx="8">
-                  <v>457068.567849176</v>
-                </pt>
-                <pt idx="9">
-                  <v>485675.043401841</v>
-                </pt>
-              </numCache>
+              <f>'Dashboard'!$B$32:$K$32</f>
             </numRef>
           </val>
           <smooth val="1"/>
-        </ser>
-        <hiLowLines>
-          <spPr>
-            <a:ln w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </hiLowLines>
-        <marker val="0"/>
-        <axId val="85242700"/>
-        <axId val="44893475"/>
-      </lineChart>
-      <catAx>
-        <axId val="85242700"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr rot="0"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>Year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-          <overlay val="0"/>
-          <spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </title>
-        <numFmt formatCode="0" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:ln w="9360">
-            <a:solidFill>
-              <a:srgbClr val="878787"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-          </a:p>
-        </txPr>
-        <crossAx val="44893475"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="0"/>
-      </catAx>
-      <valAx>
-        <axId val="44893475"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr rot="-5400000"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>CHF</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-          <overlay val="0"/>
-          <spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </title>
-        <numFmt formatCode="#,##0" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:ln w="9360">
-            <a:solidFill>
-              <a:srgbClr val="878787"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-          </a:p>
-        </txPr>
-        <crossAx val="85242700"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-      <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:t/>
-          </a:r>
-        </a:p>
-      </txPr>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:solidFill>
-      <a:srgbClr val="ffffff"/>
-    </a:solidFill>
-    <a:ln w="9360">
-      <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-      <a:round/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1800" b="1" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:rPr>
-              <a:t>EBIT (10-Year)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <varyColors val="0"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>"Base"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Base</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="4f81bd"/>
-            </a:solidFill>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="f9f9f9"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="0"/>
-          <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
-          </dLbls>
-          <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Dashboard!$B$17:$K$17</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>-1314.13500000001</v>
-                </pt>
-                <pt idx="1">
-                  <v>32337.71845</v>
-                </pt>
-                <pt idx="2">
-                  <v>58472.3875035</v>
-                </pt>
-                <pt idx="3">
-                  <v>47740.8210486051</v>
-                </pt>
-                <pt idx="4">
-                  <v>56202.0032716632</v>
-                </pt>
-                <pt idx="5">
-                  <v>68640.13657583699</v>
-                </pt>
-                <pt idx="6">
-                  <v>57612.3905784282</v>
-                </pt>
-                <pt idx="7">
-                  <v>69635.4957555821</v>
-                </pt>
-                <pt idx="8">
-                  <v>80977.1620012691</v>
-                </pt>
-                <pt idx="9">
-                  <v>92656.13608696189</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>"Downside"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Downside</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="c0504d"/>
-            </a:solidFill>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="f9f9f9"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="0"/>
-          <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
-          </dLbls>
-          <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Dashboard!$B$29:$K$29</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>-60201.61775</v>
-                </pt>
-                <pt idx="1">
-                  <v>-45819.1612825</v>
-                </pt>
-                <pt idx="2">
-                  <v>-36012.282870975</v>
-                </pt>
-                <pt idx="3">
-                  <v>-69391.5954141042</v>
-                </pt>
-                <pt idx="4">
-                  <v>-75141.6562079873</v>
-                </pt>
-                <pt idx="5">
-                  <v>-69218.24268791539</v>
-                </pt>
-                <pt idx="6">
-                  <v>-89519.136623471</v>
-                </pt>
-                <pt idx="7">
-                  <v>-84897.8875907913</v>
-                </pt>
-                <pt idx="8">
-                  <v>-81508.2354479307</v>
-                </pt>
-                <pt idx="9">
-                  <v>-78204.1212255961</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
         </ser>
         <ser>
           <idx val="2"/>
           <order val="2"/>
           <tx>
-            <strRef>
-              <f>"Upside"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Upside</v>
-                </pt>
-              </strCache>
-            </strRef>
+            <v>Upside</v>
           </tx>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="9bbb59"/>
-            </a:solidFill>
-            <a:ln w="9360">
+            <a:ln w="20000">
               <a:solidFill>
-                <a:srgbClr val="f9f9f9"/>
+                <a:srgbClr val="2E7D32"/>
               </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="0"/>
-          <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
-          </dLbls>
-          <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Dashboard!$B$41:$K$41</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>15667.10925</v>
-                </pt>
-                <pt idx="1">
-                  <v>57865.5950275</v>
-                </pt>
-                <pt idx="2">
-                  <v>91012.907628325</v>
-                </pt>
-                <pt idx="3">
-                  <v>89360.9069361748</v>
-                </pt>
-                <pt idx="4">
-                  <v>103819.54138088</v>
-                </pt>
-                <pt idx="5">
-                  <v>118810.034011061</v>
-                </pt>
-                <pt idx="6">
-                  <v>111282.994833593</v>
-                </pt>
-                <pt idx="7">
-                  <v>126213.887599754</v>
-                </pt>
-                <pt idx="8">
-                  <v>140679.673412864</v>
-                </pt>
-                <pt idx="9">
-                  <v>155658.899039058</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <overlap val="0"/>
-        <axId val="40041692"/>
-        <axId val="9810824"/>
-      </barChart>
-      <catAx>
-        <axId val="40041692"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr rot="0"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>Year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-          <overlay val="0"/>
-          <spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </title>
-        <numFmt formatCode="0" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:ln w="9360">
-            <a:solidFill>
-              <a:srgbClr val="878787"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-          </a:p>
-        </txPr>
-        <crossAx val="9810824"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="0"/>
-      </catAx>
-      <valAx>
-        <axId val="9810824"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr rot="-5400000"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>CHF</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-          <overlay val="0"/>
-          <spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </title>
-        <numFmt formatCode="#,##0" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:ln w="9360">
-            <a:solidFill>
-              <a:srgbClr val="878787"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-          </a:p>
-        </txPr>
-        <crossAx val="40041692"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-      <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:t/>
-          </a:r>
-        </a:p>
-      </txPr>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:solidFill>
-      <a:srgbClr val="ffffff"/>
-    </a:solidFill>
-    <a:ln w="9360">
-      <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-      <a:round/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1800" b="1" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr sz="1800" b="1" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:rPr>
-              <a:t>Cumulative Cash (10-Year)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <varyColors val="0"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>"Base"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Base</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="4a7ebb"/>
-            </a:solidFill>
-            <a:ln w="47520">
-              <a:solidFill>
-                <a:srgbClr val="4a7ebb"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
+              <a:prstDash val="dash"/>
             </a:ln>
           </spPr>
           <marker>
@@ -1855,656 +651,67 @@
               </a:ln>
             </spPr>
           </marker>
-          <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
-          </dLbls>
           <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
+            <numRef>
+              <f>'Dashboard'!$B$11:$K$11</f>
+            </numRef>
           </cat>
           <val>
             <numRef>
-              <f>Dashboard!$B$20:$K$20</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>18685.865</v>
-                </pt>
-                <pt idx="1">
-                  <v>46936.09583792</v>
-                </pt>
-                <pt idx="2">
-                  <v>98017.5735609776</v>
-                </pt>
-                <pt idx="3">
-                  <v>139723.954829039</v>
-                </pt>
-                <pt idx="4">
-                  <v>188822.024887164</v>
-                </pt>
-                <pt idx="5">
-                  <v>248786.048199815</v>
-                </pt>
-                <pt idx="6">
-                  <v>299116.23260913</v>
-                </pt>
-                <pt idx="7">
-                  <v>359949.801701207</v>
-                </pt>
-                <pt idx="8">
-                  <v>430691.450425515</v>
-                </pt>
-                <pt idx="9">
-                  <v>511635.850911085</v>
-                </pt>
-              </numCache>
+              <f>'Dashboard'!$B$44:$K$44</f>
             </numRef>
           </val>
           <smooth val="1"/>
         </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>"Downside"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Downside</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="be4b48"/>
-            </a:solidFill>
-            <a:ln w="47520">
-              <a:solidFill>
-                <a:srgbClr val="be4b48"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
-          </dLbls>
-          <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Dashboard!$B$32:$K$32</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>-40201.61775</v>
-                </pt>
-                <pt idx="1">
-                  <v>-86020.7790325</v>
-                </pt>
-                <pt idx="2">
-                  <v>-122033.061903475</v>
-                </pt>
-                <pt idx="3">
-                  <v>-191424.657317579</v>
-                </pt>
-                <pt idx="4">
-                  <v>-266566.313525567</v>
-                </pt>
-                <pt idx="5">
-                  <v>-335784.556213482</v>
-                </pt>
-                <pt idx="6">
-                  <v>-425303.692836953</v>
-                </pt>
-                <pt idx="7">
-                  <v>-510201.580427744</v>
-                </pt>
-                <pt idx="8">
-                  <v>-591709.8158756749</v>
-                </pt>
-                <pt idx="9">
-                  <v>-669913.937101271</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-          <smooth val="1"/>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>"Upside"</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Upside</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="98b855"/>
-            </a:solidFill>
-            <a:ln w="47520">
-              <a:solidFill>
-                <a:srgbClr val="98b855"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <dLbls>
-            <txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                    <a:latin typeface="Arial"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showLeaderLines val="1"/>
-          </dLbls>
-          <cat>
-            <multiLvlStrRef>
-              <multiLvlStrCache>
-                <lvl>
-                  <pt idx="0">
-                    <v>2036</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2035</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2034</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2033</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2032</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2031</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2030</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2029</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2028</v>
-                  </pt>
-                </lvl>
-                <lvl>
-                  <pt idx="0">
-                    <v>2027</v>
-                  </pt>
-                </lvl>
-              </multiLvlStrCache>
-              <f>Dashboard!$B$11:$K$11</f>
-            </multiLvlStrRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Dashboard!$B$44:$K$44</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="10"/>
-                <pt idx="0">
-                  <v>33686.7866408</v>
-                </pt>
-                <pt idx="1">
-                  <v>84238.17045682399</v>
-                </pt>
-                <pt idx="2">
-                  <v>163747.046560929</v>
-                </pt>
-                <pt idx="3">
-                  <v>241812.734860371</v>
-                </pt>
-                <pt idx="4">
-                  <v>332509.486210708</v>
-                </pt>
-                <pt idx="5">
-                  <v>436301.931922771</v>
-                </pt>
-                <pt idx="6">
-                  <v>533518.756209398</v>
-                </pt>
-                <pt idx="7">
-                  <v>643779.208416543</v>
-                </pt>
-                <pt idx="8">
-                  <v>766676.971110021</v>
-                </pt>
-                <pt idx="9">
-                  <v>902660.585310542</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-          <smooth val="1"/>
-        </ser>
-        <hiLowLines>
-          <spPr>
-            <a:ln w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </hiLowLines>
-        <marker val="0"/>
-        <axId val="30039530"/>
-        <axId val="32954427"/>
+        <axId val="10"/>
+        <axId val="100"/>
       </lineChart>
       <catAx>
-        <axId val="30039530"/>
+        <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="0"/>
-              <a:lstStyle/>
+              <a:bodyPr/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
+                  <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>Year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-          <overlay val="0"/>
-          <spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </title>
-        <numFmt formatCode="0" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:ln w="9360">
-            <a:solidFill>
-              <a:srgbClr val="878787"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-          </a:p>
-        </txPr>
-        <crossAx val="32954427"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="0"/>
-      </catAx>
-      <valAx>
-        <axId val="32954427"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln w="9360">
-              <a:solidFill>
-                <a:srgbClr val="878787"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr rot="-5400000"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr sz="1000" b="1" strike="noStrike" spc="-1">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
                   <a:t>CHF</a:t>
                 </a:r>
               </a:p>
             </rich>
           </tx>
-          <overlay val="0"/>
-          <spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
         </title>
-        <numFmt formatCode="#,##0" sourceLinked="1"/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:ln w="9360">
-            <a:solidFill>
-              <a:srgbClr val="878787"/>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t/>
-            </a:r>
-          </a:p>
-        </txPr>
-        <crossAx val="30039530"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
+        <crossAx val="10"/>
+        <crossesAt val="0"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-      <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:t/>
-          </a:r>
-        </a:p>
-      </txPr>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
-  <spPr>
-    <a:solidFill>
-      <a:srgbClr val="ffffff"/>
-    </a:solidFill>
-    <a:ln w="9360">
-      <a:solidFill>
-        <a:srgbClr val="d9d9d9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-      <a:round/>
-    </a:ln>
-  </spPr>
 </chartSpace>
 </file>
 
@@ -2635,19 +842,14 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
+  <oneCellAnchor>
     <from>
       <col>12</col>
       <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>160560</rowOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>29</col>
-      <colOff>403920</colOff>
-      <row>30</row>
-      <rowOff>35640</rowOff>
-    </to>
+    <ext cx="7200000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -2661,20 +863,15 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
+  </oneCellAnchor>
+  <oneCellAnchor>
     <from>
       <col>12</col>
       <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>160560</rowOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>29</col>
-      <colOff>403920</colOff>
-      <row>46</row>
-      <rowOff>35640</rowOff>
-    </to>
+    <ext cx="7200000" cy="4320000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -2688,34 +885,7 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>12</col>
-      <colOff>0</colOff>
-      <row>33</row>
-      <rowOff>160920</rowOff>
-    </from>
-    <to>
-      <col>29</col>
-      <colOff>403920</colOff>
-      <row>62</row>
-      <rowOff>36000</rowOff>
-    </to>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="3" name="Chart 3"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </twoCellAnchor>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -2985,23 +1155,10 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="20">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>10-Year Total Revenue (CHF)</t>
-        </is>
-      </c>
-      <c r="B6" s="25">
-        <f>SUM(B27:K27)</f>
-        <v/>
-      </c>
-      <c r="C6" s="25">
-        <f>SUM(B15:K15)</f>
-        <v/>
-      </c>
-      <c r="D6" s="25">
-        <f>SUM(B39:K39)</f>
-        <v/>
-      </c>
+      <c r="A6" s="24" t="n"/>
+      <c r="B6" s="25" t="n"/>
+      <c r="C6" s="25" t="n"/>
+      <c r="D6" s="25" t="n"/>
     </row>
     <row r="7"/>
     <row r="8"/>

</xml_diff>

<commit_message>
Simplify charts: remove gridlines, data labels, reference lines
Clean line charts with just the 3 scenario lines and legend.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -364,7 +364,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Profit After Tax (10-Year)</a:t>
+              <a:t>Profit After Tax</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -380,7 +380,7 @@
             <v>Base</v>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="1F4E79"/>
               </a:solidFill>
@@ -395,12 +395,6 @@
               </a:ln>
             </spPr>
           </marker>
-          <dLbls>
-            <numFmt formatCode="#,##0"/>
-            <showVal val="1"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-          </dLbls>
           <cat>
             <numRef>
               <f>'Dashboard'!$B$11:$K$11</f>
@@ -411,7 +405,6 @@
               <f>'Dashboard'!$B$19:$K$19</f>
             </numRef>
           </val>
-          <smooth val="1"/>
         </ser>
         <ser>
           <idx val="1"/>
@@ -420,7 +413,7 @@
             <v>Downside</v>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="C62828"/>
               </a:solidFill>
@@ -445,7 +438,6 @@
               <f>'Dashboard'!$B$31:$K$31</f>
             </numRef>
           </val>
-          <smooth val="1"/>
         </ser>
         <ser>
           <idx val="2"/>
@@ -454,7 +446,7 @@
             <v>Upside</v>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -479,7 +471,6 @@
               <f>'Dashboard'!$B$43:$K$43</f>
             </numRef>
           </val>
-          <smooth val="1"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -501,27 +492,10 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>CHF</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crossesAt val="0"/>
       </valAx>
     </plotArea>
     <legend>
@@ -546,7 +520,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Cumulative Cash (10-Year)</a:t>
+              <a:t>Cumulative Cash</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -562,7 +536,7 @@
             <v>Base</v>
           </tx>
           <spPr>
-            <a:ln w="28000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="1F4E79"/>
               </a:solidFill>
@@ -577,12 +551,6 @@
               </a:ln>
             </spPr>
           </marker>
-          <dLbls>
-            <numFmt formatCode="#,##0"/>
-            <showVal val="1"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-          </dLbls>
           <cat>
             <numRef>
               <f>'Dashboard'!$B$11:$K$11</f>
@@ -593,7 +561,6 @@
               <f>'Dashboard'!$B$20:$K$20</f>
             </numRef>
           </val>
-          <smooth val="1"/>
         </ser>
         <ser>
           <idx val="1"/>
@@ -602,7 +569,7 @@
             <v>Downside</v>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="C62828"/>
               </a:solidFill>
@@ -627,7 +594,6 @@
               <f>'Dashboard'!$B$32:$K$32</f>
             </numRef>
           </val>
-          <smooth val="1"/>
         </ser>
         <ser>
           <idx val="2"/>
@@ -636,7 +602,7 @@
             <v>Upside</v>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln w="25000">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -661,7 +627,6 @@
               <f>'Dashboard'!$B$44:$K$44</f>
             </numRef>
           </val>
-          <smooth val="1"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -683,27 +648,10 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>CHF</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crossesAt val="0"/>
       </valAx>
     </plotArea>
     <legend>

</xml_diff>

<commit_message>
Standard business line charts with gridlines, data labels, titles
- Horizontal gridlines, Y-axis label (CHF), chart titles
- Data labels on all 3 scenario lines
- Base: solid thick navy, Downside/Upside: thin dashed red/green

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -364,7 +364,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Profit After Tax</a:t>
+              <a:t>Profit After Tax (CHF)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -380,7 +380,7 @@
             <v>Base</v>
           </tx>
           <spPr>
-            <a:ln w="25000">
+            <a:ln w="28000">
               <a:solidFill>
                 <a:srgbClr val="1F4E79"/>
               </a:solidFill>
@@ -395,6 +395,12 @@
               </a:ln>
             </spPr>
           </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Dashboard'!$B$11:$K$11</f>
@@ -413,7 +419,7 @@
             <v>Downside</v>
           </tx>
           <spPr>
-            <a:ln w="25000">
+            <a:ln w="18000">
               <a:solidFill>
                 <a:srgbClr val="C62828"/>
               </a:solidFill>
@@ -428,6 +434,12 @@
               </a:ln>
             </spPr>
           </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Dashboard'!$B$11:$K$11</f>
@@ -446,7 +458,7 @@
             <v>Upside</v>
           </tx>
           <spPr>
-            <a:ln w="25000">
+            <a:ln w="18000">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -461,6 +473,12 @@
               </a:ln>
             </spPr>
           </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Dashboard'!$B$11:$K$11</f>
@@ -492,6 +510,22 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>CHF</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -520,7 +554,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Cumulative Cash</a:t>
+              <a:t>Cumulative Cash (CHF)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -536,7 +570,7 @@
             <v>Base</v>
           </tx>
           <spPr>
-            <a:ln w="25000">
+            <a:ln w="28000">
               <a:solidFill>
                 <a:srgbClr val="1F4E79"/>
               </a:solidFill>
@@ -551,6 +585,12 @@
               </a:ln>
             </spPr>
           </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Dashboard'!$B$11:$K$11</f>
@@ -569,7 +609,7 @@
             <v>Downside</v>
           </tx>
           <spPr>
-            <a:ln w="25000">
+            <a:ln w="18000">
               <a:solidFill>
                 <a:srgbClr val="C62828"/>
               </a:solidFill>
@@ -584,6 +624,12 @@
               </a:ln>
             </spPr>
           </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Dashboard'!$B$11:$K$11</f>
@@ -602,7 +648,7 @@
             <v>Upside</v>
           </tx>
           <spPr>
-            <a:ln w="25000">
+            <a:ln w="18000">
               <a:solidFill>
                 <a:srgbClr val="2E7D32"/>
               </a:solidFill>
@@ -617,6 +663,12 @@
               </a:ln>
             </spPr>
           </marker>
+          <dLbls>
+            <numFmt formatCode="#,##0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Dashboard'!$B$11:$K$11</f>
@@ -648,6 +700,22 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>CHF</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -797,7 +865,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="4320000"/>
+    <ext cx="7920000" cy="4680000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -819,7 +887,7 @@
       <row>16</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="4320000"/>
+    <ext cx="7920000" cy="4680000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>

</xml_diff>

<commit_message>
Restructure Revenue sheet: Bar/F&B breakdown, MODEL ASSUMPTIONS header
- Rename "GLOBAL REVENUE VARIABLES" to "MODEL ASSUMPTIONS" with distinct
  visual style (gray background + navy text vs blue section headers)
- Restructure Bar/F&B section into 5 sub-blocks per Business Plan:
  Friday Night Coffee+Drinks, Saturday Day Drinks, Saturday Day Food,
  Saturday Night Drinks, Sunday Coffee
- All guest count, per-person spend, and share rate cells are yellow
  (editable) with share rates at 0%
- Add Excel comments on share rate cells noting potential profit-margin basis
- Dinner section: 0 CHF with yellow cells for future control
- Update P&L cross-references to match new Revenue row layout
- Sheet protection preserved (password: 2027)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -106,8 +106,28 @@
       <family val="2"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -130,6 +150,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E2F3"/>
+        <bgColor rgb="FFD9E2F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -159,7 +191,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -268,6 +300,9 @@
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
@@ -276,6 +311,63 @@
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -735,6 +827,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Unknown Author</author>
+    <author>Model Note</author>
   </authors>
   <commentList>
     <comment ref="B6" authorId="0" shapeId="0">
@@ -790,14 +883,29 @@
         <t>BP states Phase 3 as 30/35/35/40. Adjusted to 30/35/40/45 assuming the 35k repeat was unintentional.</t>
       </text>
     </comment>
-    <comment ref="B82" authorId="0" shapeId="0">
+    <comment ref="B70" authorId="1" shapeId="0">
       <text>
-        <t>100% Aura revenue (self-operated by GRÜEZI). Related costs are included in Sunday Program cost line.</t>
+        <t>Share rate may be based on profit margin, not gross revenue. Adjust when contract terms are confirmed.</t>
       </text>
     </comment>
-    <comment ref="B89" authorId="0" shapeId="0">
+    <comment ref="B76" authorId="1" shapeId="0">
       <text>
-        <t>Currently set to 0. Can be used to model dinner revenue if a share agreement is negotiated with the restaurant. Enter a flat CHF amount per year.</t>
+        <t>Share rate may be based on profit margin, not gross revenue. Adjust when contract terms are confirmed.</t>
+      </text>
+    </comment>
+    <comment ref="B82" authorId="1" shapeId="0">
+      <text>
+        <t>Share rate may be based on profit margin, not gross revenue. Adjust when contract terms are confirmed.</t>
+      </text>
+    </comment>
+    <comment ref="B88" authorId="1" shapeId="0">
+      <text>
+        <t>Share rate may be based on profit margin, not gross revenue. Adjust when contract terms are confirmed.</t>
+      </text>
+    </comment>
+    <comment ref="B94" authorId="1" shapeId="0">
+      <text>
+        <t>Share rate may be based on profit margin, not gross revenue. Adjust when contract terms are confirmed.</t>
       </text>
     </comment>
   </commentList>
@@ -2754,7 +2862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="42" customWidth="1" style="19" min="1" max="1"/>
@@ -2770,9 +2878,9 @@
     </row>
     <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="20">
-      <c r="A3" s="22" t="inlineStr">
-        <is>
-          <t>GLOBAL REVENUE VARIABLES</t>
+      <c r="A3" s="36" t="inlineStr">
+        <is>
+          <t>MODEL ASSUMPTIONS</t>
         </is>
       </c>
       <c r="B3" s="22" t="n"/>
@@ -2792,7 +2900,7 @@
           <t>Total Guest Count</t>
         </is>
       </c>
-      <c r="B4" s="36" t="n">
+      <c r="B4" s="37" t="n">
         <v>280</v>
       </c>
     </row>
@@ -2802,7 +2910,7 @@
           <t>Total Ticket Count</t>
         </is>
       </c>
-      <c r="B5" s="36" t="n">
+      <c r="B5" s="37" t="n">
         <v>250</v>
       </c>
     </row>
@@ -2882,7 +2990,7 @@
           <t>Summer Start Year</t>
         </is>
       </c>
-      <c r="B13" s="37" t="n">
+      <c r="B13" s="38" t="n">
         <v>2027</v>
       </c>
     </row>
@@ -2955,7 +3063,7 @@
           <t xml:space="preserve">  Drop 1 Unit Price</t>
         </is>
       </c>
-      <c r="B22" s="36" t="n">
+      <c r="B22" s="37" t="n">
         <v>210</v>
       </c>
     </row>
@@ -2965,7 +3073,7 @@
           <t xml:space="preserve">  Drop 2 Unit Price</t>
         </is>
       </c>
-      <c r="B23" s="36" t="n">
+      <c r="B23" s="37" t="n">
         <v>250</v>
       </c>
     </row>
@@ -2975,7 +3083,7 @@
           <t xml:space="preserve">  Drop 3 Unit Price</t>
         </is>
       </c>
-      <c r="B24" s="36" t="n">
+      <c r="B24" s="37" t="n">
         <v>290</v>
       </c>
     </row>
@@ -3596,19 +3704,19 @@
           <t xml:space="preserve">  Presenting Partner — Price</t>
         </is>
       </c>
-      <c r="B44" s="36" t="n">
+      <c r="B44" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="C44" s="36" t="n">
+      <c r="C44" s="37" t="n">
         <v>50000</v>
       </c>
-      <c r="D44" s="36" t="n">
+      <c r="D44" s="37" t="n">
         <v>50000</v>
       </c>
-      <c r="E44" s="36" t="n">
+      <c r="E44" s="37" t="n">
         <v>50000</v>
       </c>
-      <c r="F44" s="36" t="n">
+      <c r="F44" s="37" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3618,19 +3726,19 @@
           <t xml:space="preserve">  Presenting Partner — Count</t>
         </is>
       </c>
-      <c r="B45" s="36" t="n">
+      <c r="B45" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="C45" s="36" t="n">
+      <c r="C45" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="36" t="n">
+      <c r="D45" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="E45" s="36" t="n">
+      <c r="E45" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="F45" s="36" t="n">
+      <c r="F45" s="37" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3668,19 +3776,19 @@
           <t xml:space="preserve">  Partner — Price</t>
         </is>
       </c>
-      <c r="B48" s="36" t="n">
+      <c r="B48" s="37" t="n">
         <v>15000</v>
       </c>
-      <c r="C48" s="36" t="n">
+      <c r="C48" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="D48" s="36" t="n">
+      <c r="D48" s="37" t="n">
         <v>15000</v>
       </c>
-      <c r="E48" s="36" t="n">
+      <c r="E48" s="37" t="n">
         <v>15000</v>
       </c>
-      <c r="F48" s="36" t="n">
+      <c r="F48" s="37" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -3690,19 +3798,19 @@
           <t xml:space="preserve">  Partner — Count</t>
         </is>
       </c>
-      <c r="B49" s="36" t="n">
+      <c r="B49" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="C49" s="36" t="n">
+      <c r="C49" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="D49" s="36" t="n">
+      <c r="D49" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="E49" s="36" t="n">
+      <c r="E49" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="F49" s="36" t="n">
+      <c r="F49" s="37" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3740,19 +3848,19 @@
           <t xml:space="preserve">  Supporting Partner — Price</t>
         </is>
       </c>
-      <c r="B52" s="36" t="n">
+      <c r="B52" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="C52" s="36" t="n">
+      <c r="C52" s="37" t="n">
         <v>5000</v>
       </c>
-      <c r="D52" s="36" t="n">
+      <c r="D52" s="37" t="n">
         <v>5000</v>
       </c>
-      <c r="E52" s="36" t="n">
+      <c r="E52" s="37" t="n">
         <v>5000</v>
       </c>
-      <c r="F52" s="36" t="n">
+      <c r="F52" s="37" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -3762,19 +3870,19 @@
           <t xml:space="preserve">  Supporting Partner — Count</t>
         </is>
       </c>
-      <c r="B53" s="36" t="n">
+      <c r="B53" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="C53" s="36" t="n">
+      <c r="C53" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="D53" s="36" t="n">
+      <c r="D53" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="E53" s="36" t="n">
+      <c r="E53" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="F53" s="36" t="n">
+      <c r="F53" s="37" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3917,34 +4025,34 @@
           <t>ASA Contribution (manual input)</t>
         </is>
       </c>
-      <c r="B61" s="36" t="n">
+      <c r="B61" s="37" t="n">
         <v>10000</v>
       </c>
-      <c r="C61" s="36" t="n">
+      <c r="C61" s="37" t="n">
         <v>12500</v>
       </c>
-      <c r="D61" s="36" t="n">
+      <c r="D61" s="37" t="n">
         <v>15000</v>
       </c>
-      <c r="E61" s="36" t="n">
+      <c r="E61" s="37" t="n">
         <v>20000</v>
       </c>
-      <c r="F61" s="36" t="n">
+      <c r="F61" s="37" t="n">
         <v>25000</v>
       </c>
-      <c r="G61" s="36" t="n">
+      <c r="G61" s="37" t="n">
         <v>30000</v>
       </c>
-      <c r="H61" s="36" t="n">
+      <c r="H61" s="37" t="n">
         <v>30000</v>
       </c>
-      <c r="I61" s="36" t="n">
+      <c r="I61" s="37" t="n">
         <v>35000</v>
       </c>
-      <c r="J61" s="36" t="n">
+      <c r="J61" s="37" t="n">
         <v>40000</v>
       </c>
-      <c r="K61" s="36" t="n">
+      <c r="K61" s="37" t="n">
         <v>45000</v>
       </c>
     </row>
@@ -3957,826 +4065,1330 @@
     </row>
     <row r="63"/>
     <row r="64" ht="15" customHeight="1" s="20">
-      <c r="A64" s="22" t="inlineStr">
+      <c r="A64" s="39" t="inlineStr">
         <is>
           <t>SECTION 4: BAR / F&amp;B REVENUE</t>
         </is>
       </c>
-      <c r="B64" s="22" t="n"/>
-      <c r="C64" s="22" t="n"/>
-      <c r="D64" s="22" t="n"/>
-      <c r="E64" s="22" t="n"/>
-      <c r="F64" s="22" t="n"/>
-      <c r="G64" s="22" t="n"/>
-      <c r="H64" s="22" t="n"/>
-      <c r="I64" s="22" t="n"/>
-      <c r="J64" s="22" t="n"/>
-      <c r="K64" s="22" t="n"/>
+      <c r="B64" s="40" t="n"/>
+      <c r="C64" s="40" t="n"/>
+      <c r="D64" s="40" t="n"/>
+      <c r="E64" s="40" t="n"/>
+      <c r="F64" s="40" t="n"/>
+      <c r="G64" s="40" t="n"/>
+      <c r="H64" s="40" t="n"/>
+      <c r="I64" s="40" t="n"/>
+      <c r="J64" s="40" t="n"/>
+      <c r="K64" s="40" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="20">
-      <c r="A65" s="33" t="inlineStr">
+      <c r="A65" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">  Share rates are currently set to 0%. Aura does not take a share of bar/food revenue. If a share agreement is negotiated, change the share rate.</t>
         </is>
       </c>
-    </row>
-    <row r="66"/>
+      <c r="B65" s="42" t="n"/>
+      <c r="C65" s="42" t="n"/>
+      <c r="D65" s="42" t="n"/>
+      <c r="E65" s="42" t="n"/>
+      <c r="F65" s="42" t="n"/>
+      <c r="G65" s="42" t="n"/>
+      <c r="H65" s="42" t="n"/>
+      <c r="I65" s="42" t="n"/>
+      <c r="J65" s="42" t="n"/>
+      <c r="K65" s="42" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="42" t="n"/>
+      <c r="B66" s="42" t="n"/>
+      <c r="C66" s="42" t="n"/>
+      <c r="D66" s="42" t="n"/>
+      <c r="E66" s="42" t="n"/>
+      <c r="F66" s="42" t="n"/>
+      <c r="G66" s="42" t="n"/>
+      <c r="H66" s="42" t="n"/>
+      <c r="I66" s="42" t="n"/>
+      <c r="J66" s="42" t="n"/>
+      <c r="K66" s="42" t="n"/>
+    </row>
     <row r="67" ht="15" customHeight="1" s="20">
-      <c r="A67" s="27" t="n"/>
-      <c r="B67" s="28" t="n">
+      <c r="A67" s="40" t="n"/>
+      <c r="B67" s="43" t="n">
         <v>2027</v>
       </c>
-      <c r="C67" s="28" t="n">
+      <c r="C67" s="43" t="n">
         <v>2028</v>
       </c>
-      <c r="D67" s="28" t="n">
+      <c r="D67" s="43" t="n">
         <v>2029</v>
       </c>
-      <c r="E67" s="28" t="n">
+      <c r="E67" s="43" t="n">
         <v>2030</v>
       </c>
-      <c r="F67" s="28" t="n">
+      <c r="F67" s="43" t="n">
         <v>2031</v>
       </c>
-      <c r="G67" s="28" t="n">
+      <c r="G67" s="43" t="n">
         <v>2032</v>
       </c>
-      <c r="H67" s="28" t="n">
+      <c r="H67" s="43" t="n">
         <v>2033</v>
       </c>
-      <c r="I67" s="28" t="n">
+      <c r="I67" s="43" t="n">
         <v>2034</v>
       </c>
-      <c r="J67" s="28" t="n">
+      <c r="J67" s="43" t="n">
         <v>2035</v>
       </c>
-      <c r="K67" s="28" t="n">
+      <c r="K67" s="43" t="n">
         <v>2036</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="20">
-      <c r="A68" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Friday Coffee/Drinks — Guest Count</t>
-        </is>
-      </c>
-      <c r="B68" s="36" t="n">
+      <c r="A68" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Friday Night: Coffee + Drinks — Guest Count</t>
+        </is>
+      </c>
+      <c r="B68" s="45" t="n">
         <v>150</v>
       </c>
+      <c r="C68" s="42" t="n"/>
+      <c r="D68" s="42" t="n"/>
+      <c r="E68" s="42" t="n"/>
+      <c r="F68" s="42" t="n"/>
+      <c r="G68" s="42" t="n"/>
+      <c r="H68" s="42" t="n"/>
+      <c r="I68" s="42" t="n"/>
+      <c r="J68" s="42" t="n"/>
+      <c r="K68" s="42" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="20">
-      <c r="A69" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Friday Coffee/Drinks — Per-person Spend</t>
-        </is>
-      </c>
-      <c r="B69" s="36" t="n">
-        <v>15</v>
-      </c>
+      <c r="A69" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Friday Night: Coffee + Drinks — Per-person Spend</t>
+        </is>
+      </c>
+      <c r="B69" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="C69" s="42" t="n"/>
+      <c r="D69" s="42" t="n"/>
+      <c r="E69" s="42" t="n"/>
+      <c r="F69" s="42" t="n"/>
+      <c r="G69" s="42" t="n"/>
+      <c r="H69" s="42" t="n"/>
+      <c r="I69" s="42" t="n"/>
+      <c r="J69" s="42" t="n"/>
+      <c r="K69" s="42" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="20">
-      <c r="A70" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Friday Coffee/Drinks — Share Rate</t>
-        </is>
-      </c>
-      <c r="B70" s="34" t="n">
+      <c r="A70" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Friday Night: Coffee + Drinks — Share Rate</t>
+        </is>
+      </c>
+      <c r="B70" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="C70" s="42" t="n"/>
+      <c r="D70" s="42" t="n"/>
+      <c r="E70" s="42" t="n"/>
+      <c r="F70" s="42" t="n"/>
+      <c r="G70" s="42" t="n"/>
+      <c r="H70" s="42" t="n"/>
+      <c r="I70" s="42" t="n"/>
+      <c r="J70" s="42" t="n"/>
+      <c r="K70" s="42" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" s="20">
-      <c r="A71" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Friday Coffee/Drinks — Est. Total Sales (reference)</t>
-        </is>
-      </c>
-      <c r="B71" s="29">
+      <c r="A71" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Friday Night: Coffee + Drinks — Est. Total Sales (reference)</t>
+        </is>
+      </c>
+      <c r="B71" s="47">
         <f>B68*B69</f>
         <v/>
       </c>
-      <c r="C71" s="29">
+      <c r="C71" s="47">
         <f>B71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="D71" s="29">
+      <c r="D71" s="47">
         <f>C71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="E71" s="29">
+      <c r="E71" s="47">
         <f>D71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="F71" s="29">
+      <c r="F71" s="47">
         <f>E71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="G71" s="29">
+      <c r="G71" s="47">
         <f>F71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="H71" s="29">
+      <c r="H71" s="47">
         <f>G71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="I71" s="29">
+      <c r="I71" s="47">
         <f>H71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="J71" s="29">
+      <c r="J71" s="47">
         <f>I71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="K71" s="29">
+      <c r="K71" s="47">
         <f>J71*(1+$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="20">
-      <c r="A72" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Friday Coffee/Drinks — Aura Revenue</t>
-        </is>
-      </c>
-      <c r="B72" s="29">
-        <f>B71*B70</f>
-        <v/>
-      </c>
-      <c r="C72" s="29">
+      <c r="A72" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Friday Night: Coffee + Drinks — Aura Revenue</t>
+        </is>
+      </c>
+      <c r="B72" s="47">
+        <f>B71*$B70</f>
+        <v/>
+      </c>
+      <c r="C72" s="47">
         <f>C71*$B70</f>
         <v/>
       </c>
-      <c r="D72" s="29">
+      <c r="D72" s="47">
         <f>D71*$B70</f>
         <v/>
       </c>
-      <c r="E72" s="29">
+      <c r="E72" s="47">
         <f>E71*$B70</f>
         <v/>
       </c>
-      <c r="F72" s="29">
+      <c r="F72" s="47">
         <f>F71*$B70</f>
         <v/>
       </c>
-      <c r="G72" s="29">
+      <c r="G72" s="47">
         <f>G71*$B70</f>
         <v/>
       </c>
-      <c r="H72" s="29">
+      <c r="H72" s="47">
         <f>H71*$B70</f>
         <v/>
       </c>
-      <c r="I72" s="29">
+      <c r="I72" s="47">
         <f>I71*$B70</f>
         <v/>
       </c>
-      <c r="J72" s="29">
+      <c r="J72" s="47">
         <f>J71*$B70</f>
         <v/>
       </c>
-      <c r="K72" s="29">
+      <c r="K72" s="47">
         <f>K71*$B70</f>
         <v/>
       </c>
     </row>
-    <row r="73"/>
+    <row r="73">
+      <c r="A73" s="42" t="n"/>
+      <c r="B73" s="42" t="n"/>
+      <c r="C73" s="42" t="n"/>
+      <c r="D73" s="42" t="n"/>
+      <c r="E73" s="42" t="n"/>
+      <c r="F73" s="42" t="n"/>
+      <c r="G73" s="42" t="n"/>
+      <c r="H73" s="42" t="n"/>
+      <c r="I73" s="42" t="n"/>
+      <c r="J73" s="42" t="n"/>
+      <c r="K73" s="42" t="n"/>
+    </row>
     <row r="74" ht="15" customHeight="1" s="20">
-      <c r="A74" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Saturday Day+Night — Guest Count</t>
-        </is>
-      </c>
-      <c r="B74" s="36" t="n">
+      <c r="A74" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Drinks — Guest Count</t>
+        </is>
+      </c>
+      <c r="B74" s="45" t="n">
         <v>280</v>
       </c>
+      <c r="C74" s="42" t="n"/>
+      <c r="D74" s="42" t="n"/>
+      <c r="E74" s="42" t="n"/>
+      <c r="F74" s="42" t="n"/>
+      <c r="G74" s="42" t="n"/>
+      <c r="H74" s="42" t="n"/>
+      <c r="I74" s="42" t="n"/>
+      <c r="J74" s="42" t="n"/>
+      <c r="K74" s="42" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" s="20">
-      <c r="A75" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Saturday Day+Night — Per-person Spend</t>
-        </is>
-      </c>
-      <c r="B75" s="36" t="n">
-        <v>65</v>
-      </c>
+      <c r="A75" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Drinks — Per-person Spend</t>
+        </is>
+      </c>
+      <c r="B75" s="45" t="n">
+        <v>20</v>
+      </c>
+      <c r="C75" s="42" t="n"/>
+      <c r="D75" s="42" t="n"/>
+      <c r="E75" s="42" t="n"/>
+      <c r="F75" s="42" t="n"/>
+      <c r="G75" s="42" t="n"/>
+      <c r="H75" s="42" t="n"/>
+      <c r="I75" s="42" t="n"/>
+      <c r="J75" s="42" t="n"/>
+      <c r="K75" s="42" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1" s="20">
-      <c r="A76" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Saturday Day+Night — Share Rate</t>
-        </is>
-      </c>
-      <c r="B76" s="34" t="n">
+      <c r="A76" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Drinks — Share Rate</t>
+        </is>
+      </c>
+      <c r="B76" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="C76" s="42" t="n"/>
+      <c r="D76" s="42" t="n"/>
+      <c r="E76" s="42" t="n"/>
+      <c r="F76" s="42" t="n"/>
+      <c r="G76" s="42" t="n"/>
+      <c r="H76" s="42" t="n"/>
+      <c r="I76" s="42" t="n"/>
+      <c r="J76" s="42" t="n"/>
+      <c r="K76" s="42" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" s="20">
-      <c r="A77" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Saturday Day+Night — Est. Total Sales (reference)</t>
-        </is>
-      </c>
-      <c r="B77" s="29">
+      <c r="A77" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Drinks — Est. Total Sales (reference)</t>
+        </is>
+      </c>
+      <c r="B77" s="47">
         <f>B74*B75</f>
         <v/>
       </c>
-      <c r="C77" s="29">
+      <c r="C77" s="47">
         <f>B77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="D77" s="29">
+      <c r="D77" s="47">
         <f>C77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="E77" s="29">
+      <c r="E77" s="47">
         <f>D77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="F77" s="29">
+      <c r="F77" s="47">
         <f>E77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="G77" s="29">
+      <c r="G77" s="47">
         <f>F77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="H77" s="29">
+      <c r="H77" s="47">
         <f>G77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="I77" s="29">
+      <c r="I77" s="47">
         <f>H77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="J77" s="29">
+      <c r="J77" s="47">
         <f>I77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="K77" s="29">
+      <c r="K77" s="47">
         <f>J77*(1+$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="20">
-      <c r="A78" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Saturday Day+Night — Aura Revenue</t>
-        </is>
-      </c>
-      <c r="B78" s="29">
-        <f>B77*B76</f>
-        <v/>
-      </c>
-      <c r="C78" s="29">
+      <c r="A78" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Drinks — Aura Revenue</t>
+        </is>
+      </c>
+      <c r="B78" s="47">
+        <f>B77*$B76</f>
+        <v/>
+      </c>
+      <c r="C78" s="47">
         <f>C77*$B76</f>
         <v/>
       </c>
-      <c r="D78" s="29">
+      <c r="D78" s="47">
         <f>D77*$B76</f>
         <v/>
       </c>
-      <c r="E78" s="29">
+      <c r="E78" s="47">
         <f>E77*$B76</f>
         <v/>
       </c>
-      <c r="F78" s="29">
+      <c r="F78" s="47">
         <f>F77*$B76</f>
         <v/>
       </c>
-      <c r="G78" s="29">
+      <c r="G78" s="47">
         <f>G77*$B76</f>
         <v/>
       </c>
-      <c r="H78" s="29">
+      <c r="H78" s="47">
         <f>H77*$B76</f>
         <v/>
       </c>
-      <c r="I78" s="29">
+      <c r="I78" s="47">
         <f>I77*$B76</f>
         <v/>
       </c>
-      <c r="J78" s="29">
+      <c r="J78" s="47">
         <f>J77*$B76</f>
         <v/>
       </c>
-      <c r="K78" s="29">
+      <c r="K78" s="47">
         <f>K77*$B76</f>
         <v/>
       </c>
     </row>
-    <row r="79"/>
+    <row r="79">
+      <c r="A79" s="42" t="n"/>
+      <c r="B79" s="42" t="n"/>
+      <c r="C79" s="42" t="n"/>
+      <c r="D79" s="42" t="n"/>
+      <c r="E79" s="42" t="n"/>
+      <c r="F79" s="42" t="n"/>
+      <c r="G79" s="42" t="n"/>
+      <c r="H79" s="42" t="n"/>
+      <c r="I79" s="42" t="n"/>
+      <c r="J79" s="42" t="n"/>
+      <c r="K79" s="42" t="n"/>
+    </row>
     <row r="80" ht="15" customHeight="1" s="20">
-      <c r="A80" s="24" t="inlineStr">
+      <c r="A80" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Food — Guest Count</t>
+        </is>
+      </c>
+      <c r="B80" s="45" t="n">
+        <v>280</v>
+      </c>
+      <c r="C80" s="42" t="n"/>
+      <c r="D80" s="42" t="n"/>
+      <c r="E80" s="42" t="n"/>
+      <c r="F80" s="42" t="n"/>
+      <c r="G80" s="42" t="n"/>
+      <c r="H80" s="42" t="n"/>
+      <c r="I80" s="42" t="n"/>
+      <c r="J80" s="42" t="n"/>
+      <c r="K80" s="42" t="n"/>
+    </row>
+    <row r="81" ht="15" customHeight="1" s="20">
+      <c r="A81" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Food — Per-person Spend</t>
+        </is>
+      </c>
+      <c r="B81" s="45" t="n">
+        <v>50</v>
+      </c>
+      <c r="C81" s="42" t="n"/>
+      <c r="D81" s="42" t="n"/>
+      <c r="E81" s="42" t="n"/>
+      <c r="F81" s="42" t="n"/>
+      <c r="G81" s="42" t="n"/>
+      <c r="H81" s="42" t="n"/>
+      <c r="I81" s="42" t="n"/>
+      <c r="J81" s="42" t="n"/>
+      <c r="K81" s="42" t="n"/>
+    </row>
+    <row r="82" ht="15" customHeight="1" s="20">
+      <c r="A82" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Food — Share Rate</t>
+        </is>
+      </c>
+      <c r="B82" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" s="42" t="n"/>
+      <c r="D82" s="42" t="n"/>
+      <c r="E82" s="42" t="n"/>
+      <c r="F82" s="42" t="n"/>
+      <c r="G82" s="42" t="n"/>
+      <c r="H82" s="42" t="n"/>
+      <c r="I82" s="42" t="n"/>
+      <c r="J82" s="42" t="n"/>
+      <c r="K82" s="42" t="n"/>
+    </row>
+    <row r="83" ht="15" customHeight="1" s="20">
+      <c r="A83" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Food — Est. Total Sales (reference)</t>
+        </is>
+      </c>
+      <c r="B83" s="47">
+        <f>B80*B81</f>
+        <v/>
+      </c>
+      <c r="C83" s="47">
+        <f>B83*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="D83" s="47">
+        <f>C83*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="E83" s="47">
+        <f>D83*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="F83" s="47">
+        <f>E83*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="G83" s="47">
+        <f>F83*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="H83" s="47">
+        <f>G83*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="I83" s="47">
+        <f>H83*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="J83" s="47">
+        <f>I83*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="K83" s="47">
+        <f>J83*(1+$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Day: Food — Aura Revenue</t>
+        </is>
+      </c>
+      <c r="B84" s="42">
+        <f>B83*$B82</f>
+        <v/>
+      </c>
+      <c r="C84" s="42">
+        <f>C83*$B82</f>
+        <v/>
+      </c>
+      <c r="D84" s="42">
+        <f>D83*$B82</f>
+        <v/>
+      </c>
+      <c r="E84" s="42">
+        <f>E83*$B82</f>
+        <v/>
+      </c>
+      <c r="F84" s="42">
+        <f>F83*$B82</f>
+        <v/>
+      </c>
+      <c r="G84" s="42">
+        <f>G83*$B82</f>
+        <v/>
+      </c>
+      <c r="H84" s="42">
+        <f>H83*$B82</f>
+        <v/>
+      </c>
+      <c r="I84" s="42">
+        <f>I83*$B82</f>
+        <v/>
+      </c>
+      <c r="J84" s="42">
+        <f>J83*$B82</f>
+        <v/>
+      </c>
+      <c r="K84" s="42">
+        <f>K83*$B82</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1" s="20">
+      <c r="A85" s="40" t="n"/>
+      <c r="B85" s="49" t="n"/>
+      <c r="C85" s="49" t="n"/>
+      <c r="D85" s="49" t="n"/>
+      <c r="E85" s="49" t="n"/>
+      <c r="F85" s="49" t="n"/>
+      <c r="G85" s="49" t="n"/>
+      <c r="H85" s="49" t="n"/>
+      <c r="I85" s="49" t="n"/>
+      <c r="J85" s="49" t="n"/>
+      <c r="K85" s="49" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Night: Drinks — Guest Count</t>
+        </is>
+      </c>
+      <c r="B86" s="50" t="n">
+        <v>150</v>
+      </c>
+      <c r="C86" s="42" t="n"/>
+      <c r="D86" s="42" t="n"/>
+      <c r="E86" s="42" t="n"/>
+      <c r="F86" s="42" t="n"/>
+      <c r="G86" s="42" t="n"/>
+      <c r="H86" s="42" t="n"/>
+      <c r="I86" s="42" t="n"/>
+      <c r="J86" s="42" t="n"/>
+      <c r="K86" s="42" t="n"/>
+    </row>
+    <row r="87" ht="15" customHeight="1" s="20">
+      <c r="A87" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Night: Drinks — Per-person Spend</t>
+        </is>
+      </c>
+      <c r="B87" s="51" t="n">
+        <v>50</v>
+      </c>
+      <c r="C87" s="40" t="n"/>
+      <c r="D87" s="40" t="n"/>
+      <c r="E87" s="40" t="n"/>
+      <c r="F87" s="40" t="n"/>
+      <c r="G87" s="40" t="n"/>
+      <c r="H87" s="40" t="n"/>
+      <c r="I87" s="40" t="n"/>
+      <c r="J87" s="40" t="n"/>
+      <c r="K87" s="40" t="n"/>
+    </row>
+    <row r="88" ht="15" customHeight="1" s="20">
+      <c r="A88" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Night: Drinks — Share Rate</t>
+        </is>
+      </c>
+      <c r="B88" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="C88" s="53" t="n"/>
+      <c r="D88" s="53" t="n"/>
+      <c r="E88" s="53" t="n"/>
+      <c r="F88" s="53" t="n"/>
+      <c r="G88" s="53" t="n"/>
+      <c r="H88" s="53" t="n"/>
+      <c r="I88" s="53" t="n"/>
+      <c r="J88" s="53" t="n"/>
+      <c r="K88" s="53" t="n"/>
+    </row>
+    <row r="89" ht="15" customHeight="1" s="20">
+      <c r="A89" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Night: Drinks — Est. Total Sales (reference)</t>
+        </is>
+      </c>
+      <c r="B89" s="47">
+        <f>B86*B87</f>
+        <v/>
+      </c>
+      <c r="C89" s="47">
+        <f>B89*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="D89" s="47">
+        <f>C89*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="E89" s="47">
+        <f>D89*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="F89" s="47">
+        <f>E89*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="G89" s="47">
+        <f>F89*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="H89" s="47">
+        <f>G89*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="I89" s="47">
+        <f>H89*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="J89" s="47">
+        <f>I89*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="K89" s="47">
+        <f>J89*(1+$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" ht="15" customHeight="1" s="20">
+      <c r="A90" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Saturday Night: Drinks — Aura Revenue</t>
+        </is>
+      </c>
+      <c r="B90" s="42">
+        <f>B89*$B88</f>
+        <v/>
+      </c>
+      <c r="C90" s="42">
+        <f>C89*$B88</f>
+        <v/>
+      </c>
+      <c r="D90" s="42">
+        <f>D89*$B88</f>
+        <v/>
+      </c>
+      <c r="E90" s="42">
+        <f>E89*$B88</f>
+        <v/>
+      </c>
+      <c r="F90" s="42">
+        <f>F89*$B88</f>
+        <v/>
+      </c>
+      <c r="G90" s="42">
+        <f>G89*$B88</f>
+        <v/>
+      </c>
+      <c r="H90" s="42">
+        <f>H89*$B88</f>
+        <v/>
+      </c>
+      <c r="I90" s="42">
+        <f>I89*$B88</f>
+        <v/>
+      </c>
+      <c r="J90" s="42">
+        <f>J89*$B88</f>
+        <v/>
+      </c>
+      <c r="K90" s="42">
+        <f>K89*$B88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="42" t="n"/>
+      <c r="B91" s="42" t="n"/>
+      <c r="C91" s="42" t="n"/>
+      <c r="D91" s="42" t="n"/>
+      <c r="E91" s="42" t="n"/>
+      <c r="F91" s="42" t="n"/>
+      <c r="G91" s="42" t="n"/>
+      <c r="H91" s="42" t="n"/>
+      <c r="I91" s="42" t="n"/>
+      <c r="J91" s="42" t="n"/>
+      <c r="K91" s="42" t="n"/>
+    </row>
+    <row r="92" ht="15" customHeight="1" s="20">
+      <c r="A92" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sunday Coffee — Guest Count</t>
         </is>
       </c>
-      <c r="B80" s="36" t="n">
+      <c r="B92" s="51" t="n">
         <v>80</v>
       </c>
-    </row>
-    <row r="81" ht="15" customHeight="1" s="20">
-      <c r="A81" s="24" t="inlineStr">
+      <c r="C92" s="40" t="n"/>
+      <c r="D92" s="40" t="n"/>
+      <c r="E92" s="40" t="n"/>
+      <c r="F92" s="40" t="n"/>
+      <c r="G92" s="40" t="n"/>
+      <c r="H92" s="40" t="n"/>
+      <c r="I92" s="40" t="n"/>
+      <c r="J92" s="40" t="n"/>
+      <c r="K92" s="40" t="n"/>
+    </row>
+    <row r="93" ht="15" customHeight="1" s="20">
+      <c r="A93" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sunday Coffee — Per-person Spend</t>
         </is>
       </c>
-      <c r="B81" s="36" t="n">
+      <c r="B93" s="52" t="n">
         <v>8</v>
       </c>
-    </row>
-    <row r="82" ht="15" customHeight="1" s="20">
-      <c r="A82" s="24" t="inlineStr">
+      <c r="C93" s="53" t="n"/>
+      <c r="D93" s="53" t="n"/>
+      <c r="E93" s="53" t="n"/>
+      <c r="F93" s="53" t="n"/>
+      <c r="G93" s="53" t="n"/>
+      <c r="H93" s="53" t="n"/>
+      <c r="I93" s="53" t="n"/>
+      <c r="J93" s="53" t="n"/>
+      <c r="K93" s="53" t="n"/>
+    </row>
+    <row r="94" ht="15" customHeight="1" s="20">
+      <c r="A94" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sunday Coffee — Share Rate</t>
         </is>
       </c>
-      <c r="B82" s="34" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" ht="15" customHeight="1" s="20">
-      <c r="A83" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sunday Coffee — Revenue (fixed, no growth)</t>
-        </is>
-      </c>
-      <c r="B83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="C83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="D83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="E83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="F83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="G83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="H83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="I83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="J83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-      <c r="K83" s="29">
-        <f>$B$80*$B$81*$B$82</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84"/>
-    <row r="85" ht="15" customHeight="1" s="20">
-      <c r="A85" s="26" t="inlineStr">
+      <c r="B94" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" s="47" t="n"/>
+      <c r="D94" s="47" t="n"/>
+      <c r="E94" s="47" t="n"/>
+      <c r="F94" s="47" t="n"/>
+      <c r="G94" s="47" t="n"/>
+      <c r="H94" s="47" t="n"/>
+      <c r="I94" s="47" t="n"/>
+      <c r="J94" s="47" t="n"/>
+      <c r="K94" s="47" t="n"/>
+    </row>
+    <row r="95" ht="15" customHeight="1" s="20">
+      <c r="A95" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sunday Coffee — Est. Total Sales (reference)</t>
+        </is>
+      </c>
+      <c r="B95" s="42">
+        <f>B92*B93</f>
+        <v/>
+      </c>
+      <c r="C95" s="42">
+        <f>B95*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="D95" s="42">
+        <f>C95*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="E95" s="42">
+        <f>D95*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="F95" s="42">
+        <f>E95*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="G95" s="42">
+        <f>F95*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="H95" s="42">
+        <f>G95*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="I95" s="42">
+        <f>H95*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="J95" s="42">
+        <f>I95*(1+$B$9)</f>
+        <v/>
+      </c>
+      <c r="K95" s="42">
+        <f>J95*(1+$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sunday Coffee — Aura Revenue</t>
+        </is>
+      </c>
+      <c r="B96" s="42">
+        <f>B95*$B94</f>
+        <v/>
+      </c>
+      <c r="C96" s="42">
+        <f>C95*$B94</f>
+        <v/>
+      </c>
+      <c r="D96" s="42">
+        <f>D95*$B94</f>
+        <v/>
+      </c>
+      <c r="E96" s="42">
+        <f>E95*$B94</f>
+        <v/>
+      </c>
+      <c r="F96" s="42">
+        <f>F95*$B94</f>
+        <v/>
+      </c>
+      <c r="G96" s="42">
+        <f>G95*$B94</f>
+        <v/>
+      </c>
+      <c r="H96" s="42">
+        <f>H95*$B94</f>
+        <v/>
+      </c>
+      <c r="I96" s="42">
+        <f>I95*$B94</f>
+        <v/>
+      </c>
+      <c r="J96" s="42">
+        <f>J95*$B94</f>
+        <v/>
+      </c>
+      <c r="K96" s="42">
+        <f>K95*$B94</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" ht="15" customHeight="1" s="20">
+      <c r="A97" s="40" t="n"/>
+      <c r="B97" s="40" t="n"/>
+      <c r="C97" s="40" t="n"/>
+      <c r="D97" s="40" t="n"/>
+      <c r="E97" s="40" t="n"/>
+      <c r="F97" s="40" t="n"/>
+      <c r="G97" s="40" t="n"/>
+      <c r="H97" s="40" t="n"/>
+      <c r="I97" s="40" t="n"/>
+      <c r="J97" s="40" t="n"/>
+      <c r="K97" s="40" t="n"/>
+    </row>
+    <row r="98" ht="15" customHeight="1" s="20">
+      <c r="A98" s="54" t="inlineStr">
         <is>
           <t>Bar/F&amp;B Total</t>
         </is>
       </c>
-      <c r="B85" s="31">
-        <f>B72+B78+B83</f>
-        <v/>
-      </c>
-      <c r="C85" s="31">
-        <f>C72+C78+C83</f>
-        <v/>
-      </c>
-      <c r="D85" s="31">
-        <f>D72+D78+D83</f>
-        <v/>
-      </c>
-      <c r="E85" s="31">
-        <f>E72+E78+E83</f>
-        <v/>
-      </c>
-      <c r="F85" s="31">
-        <f>F72+F78+F83</f>
-        <v/>
-      </c>
-      <c r="G85" s="31">
-        <f>G72+G78+G83</f>
-        <v/>
-      </c>
-      <c r="H85" s="31">
-        <f>H72+H78+H83</f>
-        <v/>
-      </c>
-      <c r="I85" s="31">
-        <f>I72+I78+I83</f>
-        <v/>
-      </c>
-      <c r="J85" s="31">
-        <f>J72+J78+J83</f>
-        <v/>
-      </c>
-      <c r="K85" s="31">
-        <f>K72+K78+K83</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86"/>
-    <row r="87" ht="15" customHeight="1" s="20">
-      <c r="A87" s="22" t="inlineStr">
+      <c r="B98" s="53">
+        <f>B72+B78+B84+B90+B96</f>
+        <v/>
+      </c>
+      <c r="C98" s="53">
+        <f>C72+C78+C84+C90+C96</f>
+        <v/>
+      </c>
+      <c r="D98" s="53">
+        <f>D72+D78+D84+D90+D96</f>
+        <v/>
+      </c>
+      <c r="E98" s="53">
+        <f>E72+E78+E84+E90+E96</f>
+        <v/>
+      </c>
+      <c r="F98" s="53">
+        <f>F72+F78+F84+F90+F96</f>
+        <v/>
+      </c>
+      <c r="G98" s="53">
+        <f>G72+G78+G84+G90+G96</f>
+        <v/>
+      </c>
+      <c r="H98" s="53">
+        <f>H72+H78+H84+H90+H96</f>
+        <v/>
+      </c>
+      <c r="I98" s="53">
+        <f>I72+I78+I84+I90+I96</f>
+        <v/>
+      </c>
+      <c r="J98" s="53">
+        <f>J72+J78+J84+J90+J96</f>
+        <v/>
+      </c>
+      <c r="K98" s="53">
+        <f>K72+K78+K84+K90+K96</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99" ht="15" customHeight="1" s="20">
+      <c r="A99" s="40" t="n"/>
+      <c r="B99" s="49" t="n"/>
+      <c r="C99" s="49" t="n"/>
+      <c r="D99" s="49" t="n"/>
+      <c r="E99" s="49" t="n"/>
+      <c r="F99" s="49" t="n"/>
+      <c r="G99" s="49" t="n"/>
+      <c r="H99" s="49" t="n"/>
+      <c r="I99" s="49" t="n"/>
+      <c r="J99" s="49" t="n"/>
+      <c r="K99" s="49" t="n"/>
+    </row>
+    <row r="100" ht="15" customHeight="1" s="20">
+      <c r="A100" s="39" t="inlineStr">
         <is>
           <t>SECTION 5: DINNER REVENUE</t>
         </is>
       </c>
-      <c r="B87" s="22" t="n"/>
-      <c r="C87" s="22" t="n"/>
-      <c r="D87" s="22" t="n"/>
-      <c r="E87" s="22" t="n"/>
-      <c r="F87" s="22" t="n"/>
-      <c r="G87" s="22" t="n"/>
-      <c r="H87" s="22" t="n"/>
-      <c r="I87" s="22" t="n"/>
-      <c r="J87" s="22" t="n"/>
-      <c r="K87" s="22" t="n"/>
-    </row>
-    <row r="88" ht="15" customHeight="1" s="20">
-      <c r="A88" s="27" t="n"/>
-      <c r="B88" s="28" t="n">
+      <c r="B100" s="47" t="n"/>
+      <c r="C100" s="47" t="n"/>
+      <c r="D100" s="47" t="n"/>
+      <c r="E100" s="47" t="n"/>
+      <c r="F100" s="47" t="n"/>
+      <c r="G100" s="47" t="n"/>
+      <c r="H100" s="47" t="n"/>
+      <c r="I100" s="47" t="n"/>
+      <c r="J100" s="47" t="n"/>
+      <c r="K100" s="47" t="n"/>
+    </row>
+    <row r="101" ht="15" customHeight="1" s="20">
+      <c r="A101" s="40" t="n"/>
+      <c r="B101" s="55" t="n">
         <v>2027</v>
       </c>
-      <c r="C88" s="28" t="n">
+      <c r="C101" s="55" t="n">
         <v>2028</v>
       </c>
-      <c r="D88" s="28" t="n">
+      <c r="D101" s="55" t="n">
         <v>2029</v>
       </c>
-      <c r="E88" s="28" t="n">
+      <c r="E101" s="55" t="n">
         <v>2030</v>
       </c>
-      <c r="F88" s="28" t="n">
+      <c r="F101" s="55" t="n">
         <v>2031</v>
       </c>
-      <c r="G88" s="28" t="n">
+      <c r="G101" s="55" t="n">
         <v>2032</v>
       </c>
-      <c r="H88" s="28" t="n">
+      <c r="H101" s="55" t="n">
         <v>2033</v>
       </c>
-      <c r="I88" s="28" t="n">
+      <c r="I101" s="55" t="n">
         <v>2034</v>
       </c>
-      <c r="J88" s="28" t="n">
+      <c r="J101" s="55" t="n">
         <v>2035</v>
       </c>
-      <c r="K88" s="28" t="n">
+      <c r="K101" s="55" t="n">
         <v>2036</v>
       </c>
     </row>
-    <row r="89" ht="15" customHeight="1" s="20">
-      <c r="A89" s="26" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="48" t="inlineStr">
         <is>
           <t>Dinner Revenue (manual input)</t>
         </is>
       </c>
-      <c r="B89" s="36" t="n">
+      <c r="B102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="C89" s="36" t="n">
+      <c r="C102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="D89" s="36" t="n">
+      <c r="D102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="E89" s="36" t="n">
+      <c r="E102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="F89" s="36" t="n">
+      <c r="F102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="G89" s="36" t="n">
+      <c r="G102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="H89" s="36" t="n">
+      <c r="H102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="I89" s="36" t="n">
+      <c r="I102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="J89" s="36" t="n">
+      <c r="J102" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="K89" s="36" t="n">
+      <c r="K102" s="56" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="90" ht="15" customHeight="1" s="20">
-      <c r="A90" s="33" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  BP: 'Dinner is invite-only, sponsor-funded, never sold.' If a dinner-specific sponsor appears, it goes under Partnerships.</t>
         </is>
       </c>
     </row>
-    <row r="91"/>
-    <row r="92" ht="15" customHeight="1" s="20">
-      <c r="A92" s="22" t="inlineStr">
+    <row r="104"/>
+    <row r="105">
+      <c r="A105" s="58" t="inlineStr">
         <is>
           <t>SECTION 6: OTHER REVENUE</t>
         </is>
       </c>
-      <c r="B92" s="22" t="n"/>
-      <c r="C92" s="22" t="n"/>
-      <c r="D92" s="22" t="n"/>
-      <c r="E92" s="22" t="n"/>
-      <c r="F92" s="22" t="n"/>
-      <c r="G92" s="22" t="n"/>
-      <c r="H92" s="22" t="n"/>
-      <c r="I92" s="22" t="n"/>
-      <c r="J92" s="22" t="n"/>
-      <c r="K92" s="22" t="n"/>
-    </row>
-    <row r="93" ht="15" customHeight="1" s="20">
-      <c r="A93" s="27" t="n"/>
-      <c r="B93" s="28" t="n">
+    </row>
+    <row r="106">
+      <c r="B106" s="59" t="n">
         <v>2027</v>
       </c>
-      <c r="C93" s="28" t="n">
+      <c r="C106" s="59" t="n">
         <v>2028</v>
       </c>
-      <c r="D93" s="28" t="n">
+      <c r="D106" s="59" t="n">
         <v>2029</v>
       </c>
-      <c r="E93" s="28" t="n">
+      <c r="E106" s="59" t="n">
         <v>2030</v>
       </c>
-      <c r="F93" s="28" t="n">
+      <c r="F106" s="59" t="n">
         <v>2031</v>
       </c>
-      <c r="G93" s="28" t="n">
+      <c r="G106" s="59" t="n">
         <v>2032</v>
       </c>
-      <c r="H93" s="28" t="n">
+      <c r="H106" s="59" t="n">
         <v>2033</v>
       </c>
-      <c r="I93" s="28" t="n">
+      <c r="I106" s="59" t="n">
         <v>2034</v>
       </c>
-      <c r="J93" s="28" t="n">
+      <c r="J106" s="59" t="n">
         <v>2035</v>
       </c>
-      <c r="K93" s="28" t="n">
+      <c r="K106" s="59" t="n">
         <v>2036</v>
       </c>
     </row>
-    <row r="94" ht="15" customHeight="1" s="20">
-      <c r="A94" s="26" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="48" t="inlineStr">
         <is>
           <t>Other Revenue</t>
         </is>
       </c>
-      <c r="B94" s="36" t="n">
+      <c r="B107" s="56" t="n">
         <v>2000</v>
       </c>
-      <c r="C94" s="29">
-        <f>B94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="D94" s="29">
-        <f>C94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="E94" s="29">
-        <f>D94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="F94" s="29">
-        <f>E94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="G94" s="29">
-        <f>F94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="H94" s="29">
-        <f>G94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="I94" s="29">
-        <f>H94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="J94" s="29">
-        <f>I94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-      <c r="K94" s="29">
-        <f>J94*(1+'P&amp;L'!$B$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95" ht="15" customHeight="1" s="20">
-      <c r="A95" s="33" t="inlineStr">
+      <c r="C107">
+        <f>B107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="D107">
+        <f>C107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="E107">
+        <f>D107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="F107">
+        <f>E107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="G107">
+        <f>F107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="H107">
+        <f>G107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="I107">
+        <f>H107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="J107">
+        <f>I107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+      <c r="K107">
+        <f>J107*(1+'P&amp;L'!$B$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  Other Revenue grows with General Inflation Rate (P&amp;L sheet). Contents: add-ons, upselling, merchandise.</t>
         </is>
       </c>
     </row>
-    <row r="96"/>
-    <row r="97" ht="15" customHeight="1" s="20">
-      <c r="A97" s="22" t="inlineStr">
+    <row r="109"/>
+    <row r="110">
+      <c r="A110" s="58" t="inlineStr">
         <is>
           <t>REVENUE TOTALS</t>
         </is>
       </c>
-      <c r="B97" s="22" t="n"/>
-      <c r="C97" s="22" t="n"/>
-      <c r="D97" s="22" t="n"/>
-      <c r="E97" s="22" t="n"/>
-      <c r="F97" s="22" t="n"/>
-      <c r="G97" s="22" t="n"/>
-      <c r="H97" s="22" t="n"/>
-      <c r="I97" s="22" t="n"/>
-      <c r="J97" s="22" t="n"/>
-      <c r="K97" s="22" t="n"/>
-    </row>
-    <row r="98" ht="15" customHeight="1" s="20">
-      <c r="A98" s="27" t="n"/>
-      <c r="B98" s="28" t="n">
+    </row>
+    <row r="111">
+      <c r="B111" s="59" t="n">
         <v>2027</v>
       </c>
-      <c r="C98" s="28" t="n">
+      <c r="C111" s="59" t="n">
         <v>2028</v>
       </c>
-      <c r="D98" s="28" t="n">
+      <c r="D111" s="59" t="n">
         <v>2029</v>
       </c>
-      <c r="E98" s="28" t="n">
+      <c r="E111" s="59" t="n">
         <v>2030</v>
       </c>
-      <c r="F98" s="28" t="n">
+      <c r="F111" s="59" t="n">
         <v>2031</v>
       </c>
-      <c r="G98" s="28" t="n">
+      <c r="G111" s="59" t="n">
         <v>2032</v>
       </c>
-      <c r="H98" s="28" t="n">
+      <c r="H111" s="59" t="n">
         <v>2033</v>
       </c>
-      <c r="I98" s="28" t="n">
+      <c r="I111" s="59" t="n">
         <v>2034</v>
       </c>
-      <c r="J98" s="28" t="n">
+      <c r="J111" s="59" t="n">
         <v>2035</v>
       </c>
-      <c r="K98" s="28" t="n">
+      <c r="K111" s="59" t="n">
         <v>2036</v>
       </c>
     </row>
-    <row r="99" ht="15" customHeight="1" s="20">
-      <c r="A99" s="26" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="59" t="inlineStr">
         <is>
           <t>TOTAL WINTER REVENUE</t>
         </is>
       </c>
-      <c r="B99" s="31">
-        <f>B40+B56+B61+B85+B89+B94</f>
-        <v/>
-      </c>
-      <c r="C99" s="31">
-        <f>C40+C56+C61+C85+C89+C94</f>
-        <v/>
-      </c>
-      <c r="D99" s="31">
-        <f>D40+D56+D61+D85+D89+D94</f>
-        <v/>
-      </c>
-      <c r="E99" s="31">
-        <f>E40+E56+E61+E85+E89+E94</f>
-        <v/>
-      </c>
-      <c r="F99" s="31">
-        <f>F40+F56+F61+F85+F89+F94</f>
-        <v/>
-      </c>
-      <c r="G99" s="31">
-        <f>G40+G56+G61+G85+G89+G94</f>
-        <v/>
-      </c>
-      <c r="H99" s="31">
-        <f>H40+H56+H61+H85+H89+H94</f>
-        <v/>
-      </c>
-      <c r="I99" s="31">
-        <f>I40+I56+I61+I85+I89+I94</f>
-        <v/>
-      </c>
-      <c r="J99" s="31">
-        <f>J40+J56+J61+J85+J89+J94</f>
-        <v/>
-      </c>
-      <c r="K99" s="31">
-        <f>K40+K56+K61+K85+K89+K94</f>
-        <v/>
-      </c>
-    </row>
-    <row r="100" ht="15" customHeight="1" s="20">
-      <c r="A100" s="24" t="inlineStr">
+      <c r="B112">
+        <f>B40+B56+B61+B98+B102+B107</f>
+        <v/>
+      </c>
+      <c r="C112">
+        <f>C40+C56+C61+C98+C102+C107</f>
+        <v/>
+      </c>
+      <c r="D112">
+        <f>D40+D56+D61+D98+D102+D107</f>
+        <v/>
+      </c>
+      <c r="E112">
+        <f>E40+E56+E61+E98+E102+E107</f>
+        <v/>
+      </c>
+      <c r="F112">
+        <f>F40+F56+F61+F98+F102+F107</f>
+        <v/>
+      </c>
+      <c r="G112">
+        <f>G40+G56+G61+G98+G102+G107</f>
+        <v/>
+      </c>
+      <c r="H112">
+        <f>H40+H56+H61+H98+H102+H107</f>
+        <v/>
+      </c>
+      <c r="I112">
+        <f>I40+I56+I61+I98+I102+I107</f>
+        <v/>
+      </c>
+      <c r="J112">
+        <f>J40+J56+J61+J98+J102+J107</f>
+        <v/>
+      </c>
+      <c r="K112">
+        <f>K40+K56+K61+K98+K102+K107</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="59" t="inlineStr">
         <is>
           <t>Summer Revenue</t>
         </is>
       </c>
-      <c r="B100" s="29">
-        <f>IF(2027&gt;=$B$13,B99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="C100" s="29">
-        <f>IF(2028&gt;=$B$13,C99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="D100" s="29">
-        <f>IF(2029&gt;=$B$13,D99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="E100" s="29">
-        <f>IF(2030&gt;=$B$13,E99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="F100" s="29">
-        <f>IF(2031&gt;=$B$13,F99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="G100" s="29">
-        <f>IF(2032&gt;=$B$13,G99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="H100" s="29">
-        <f>IF(2033&gt;=$B$13,H99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="I100" s="29">
-        <f>IF(2034&gt;=$B$13,I99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="J100" s="29">
-        <f>IF(2035&gt;=$B$13,J99*$B$11,0)</f>
-        <v/>
-      </c>
-      <c r="K100" s="29">
-        <f>IF(2036&gt;=$B$13,K99*$B$11,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="101" ht="15" customHeight="1" s="20">
-      <c r="A101" s="26" t="inlineStr">
+      <c r="B113">
+        <f>IF(2027&gt;=$B$13,B112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="C113">
+        <f>IF(2028&gt;=$B$13,C112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="D113">
+        <f>IF(2029&gt;=$B$13,D112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="E113">
+        <f>IF(2030&gt;=$B$13,E112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="F113">
+        <f>IF(2031&gt;=$B$13,F112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="G113">
+        <f>IF(2032&gt;=$B$13,G112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="H113">
+        <f>IF(2033&gt;=$B$13,H112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="I113">
+        <f>IF(2034&gt;=$B$13,I112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="J113">
+        <f>IF(2035&gt;=$B$13,J112*$B$11,0)</f>
+        <v/>
+      </c>
+      <c r="K113">
+        <f>IF(2036&gt;=$B$13,K112*$B$11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="59" t="inlineStr">
         <is>
           <t>TOTAL ANNUAL REVENUE</t>
         </is>
       </c>
-      <c r="B101" s="31">
-        <f>B99+B100</f>
-        <v/>
-      </c>
-      <c r="C101" s="31">
-        <f>C99+C100</f>
-        <v/>
-      </c>
-      <c r="D101" s="31">
-        <f>D99+D100</f>
-        <v/>
-      </c>
-      <c r="E101" s="31">
-        <f>E99+E100</f>
-        <v/>
-      </c>
-      <c r="F101" s="31">
-        <f>F99+F100</f>
-        <v/>
-      </c>
-      <c r="G101" s="31">
-        <f>G99+G100</f>
-        <v/>
-      </c>
-      <c r="H101" s="31">
-        <f>H99+H100</f>
-        <v/>
-      </c>
-      <c r="I101" s="31">
-        <f>I99+I100</f>
-        <v/>
-      </c>
-      <c r="J101" s="31">
-        <f>J99+J100</f>
-        <v/>
-      </c>
-      <c r="K101" s="31">
-        <f>K99+K100</f>
+      <c r="B114">
+        <f>B112+B113</f>
+        <v/>
+      </c>
+      <c r="C114">
+        <f>C112+C113</f>
+        <v/>
+      </c>
+      <c r="D114">
+        <f>D112+D113</f>
+        <v/>
+      </c>
+      <c r="E114">
+        <f>E112+E113</f>
+        <v/>
+      </c>
+      <c r="F114">
+        <f>F112+F113</f>
+        <v/>
+      </c>
+      <c r="G114">
+        <f>G112+G113</f>
+        <v/>
+      </c>
+      <c r="H114">
+        <f>H112+H113</f>
+        <v/>
+      </c>
+      <c r="I114">
+        <f>I112+I113</f>
+        <v/>
+      </c>
+      <c r="J114">
+        <f>J112+J113</f>
+        <v/>
+      </c>
+      <c r="K114">
+        <f>K112+K113</f>
         <v/>
       </c>
     </row>
@@ -4853,7 +5465,7 @@
           <t>Initial Capital (GmbH paid-in)</t>
         </is>
       </c>
-      <c r="B6" s="36" t="n">
+      <c r="B6" s="37" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -5056,43 +5668,43 @@
         </is>
       </c>
       <c r="B13" s="29">
-        <f>Revenue!B85</f>
+        <f>Revenue!B98</f>
         <v/>
       </c>
       <c r="C13" s="29">
-        <f>Revenue!C85</f>
+        <f>Revenue!C98</f>
         <v/>
       </c>
       <c r="D13" s="29">
-        <f>Revenue!D85</f>
+        <f>Revenue!D98</f>
         <v/>
       </c>
       <c r="E13" s="29">
-        <f>Revenue!E85</f>
+        <f>Revenue!E98</f>
         <v/>
       </c>
       <c r="F13" s="29">
-        <f>Revenue!F85</f>
+        <f>Revenue!F98</f>
         <v/>
       </c>
       <c r="G13" s="29">
-        <f>Revenue!G85</f>
+        <f>Revenue!G98</f>
         <v/>
       </c>
       <c r="H13" s="29">
-        <f>Revenue!H85</f>
+        <f>Revenue!H98</f>
         <v/>
       </c>
       <c r="I13" s="29">
-        <f>Revenue!I85</f>
+        <f>Revenue!I98</f>
         <v/>
       </c>
       <c r="J13" s="29">
-        <f>Revenue!J85</f>
+        <f>Revenue!J98</f>
         <v/>
       </c>
       <c r="K13" s="29">
-        <f>Revenue!K85</f>
+        <f>Revenue!K98</f>
         <v/>
       </c>
     </row>
@@ -5103,43 +5715,43 @@
         </is>
       </c>
       <c r="B14" s="29">
-        <f>Revenue!B89</f>
+        <f>Revenue!B102</f>
         <v/>
       </c>
       <c r="C14" s="29">
-        <f>Revenue!C89</f>
+        <f>Revenue!C102</f>
         <v/>
       </c>
       <c r="D14" s="29">
-        <f>Revenue!D89</f>
+        <f>Revenue!D102</f>
         <v/>
       </c>
       <c r="E14" s="29">
-        <f>Revenue!E89</f>
+        <f>Revenue!E102</f>
         <v/>
       </c>
       <c r="F14" s="29">
-        <f>Revenue!F89</f>
+        <f>Revenue!F102</f>
         <v/>
       </c>
       <c r="G14" s="29">
-        <f>Revenue!G89</f>
+        <f>Revenue!G102</f>
         <v/>
       </c>
       <c r="H14" s="29">
-        <f>Revenue!H89</f>
+        <f>Revenue!H102</f>
         <v/>
       </c>
       <c r="I14" s="29">
-        <f>Revenue!I89</f>
+        <f>Revenue!I102</f>
         <v/>
       </c>
       <c r="J14" s="29">
-        <f>Revenue!J89</f>
+        <f>Revenue!J102</f>
         <v/>
       </c>
       <c r="K14" s="29">
-        <f>Revenue!K89</f>
+        <f>Revenue!K102</f>
         <v/>
       </c>
     </row>
@@ -5150,43 +5762,43 @@
         </is>
       </c>
       <c r="B15" s="29">
-        <f>Revenue!B94</f>
+        <f>Revenue!B107</f>
         <v/>
       </c>
       <c r="C15" s="29">
-        <f>Revenue!C94</f>
+        <f>Revenue!C107</f>
         <v/>
       </c>
       <c r="D15" s="29">
-        <f>Revenue!D94</f>
+        <f>Revenue!D107</f>
         <v/>
       </c>
       <c r="E15" s="29">
-        <f>Revenue!E94</f>
+        <f>Revenue!E107</f>
         <v/>
       </c>
       <c r="F15" s="29">
-        <f>Revenue!F94</f>
+        <f>Revenue!F107</f>
         <v/>
       </c>
       <c r="G15" s="29">
-        <f>Revenue!G94</f>
+        <f>Revenue!G107</f>
         <v/>
       </c>
       <c r="H15" s="29">
-        <f>Revenue!H94</f>
+        <f>Revenue!H107</f>
         <v/>
       </c>
       <c r="I15" s="29">
-        <f>Revenue!I94</f>
+        <f>Revenue!I107</f>
         <v/>
       </c>
       <c r="J15" s="29">
-        <f>Revenue!J94</f>
+        <f>Revenue!J107</f>
         <v/>
       </c>
       <c r="K15" s="29">
-        <f>Revenue!K94</f>
+        <f>Revenue!K107</f>
         <v/>
       </c>
     </row>
@@ -5198,43 +5810,43 @@
         </is>
       </c>
       <c r="B17" s="31">
-        <f>Revenue!B101</f>
+        <f>Revenue!B114</f>
         <v/>
       </c>
       <c r="C17" s="31">
-        <f>Revenue!C101</f>
+        <f>Revenue!C114</f>
         <v/>
       </c>
       <c r="D17" s="31">
-        <f>Revenue!D101</f>
+        <f>Revenue!D114</f>
         <v/>
       </c>
       <c r="E17" s="31">
-        <f>Revenue!E101</f>
+        <f>Revenue!E114</f>
         <v/>
       </c>
       <c r="F17" s="31">
-        <f>Revenue!F101</f>
+        <f>Revenue!F114</f>
         <v/>
       </c>
       <c r="G17" s="31">
-        <f>Revenue!G101</f>
+        <f>Revenue!G114</f>
         <v/>
       </c>
       <c r="H17" s="31">
-        <f>Revenue!H101</f>
+        <f>Revenue!H114</f>
         <v/>
       </c>
       <c r="I17" s="31">
-        <f>Revenue!I101</f>
+        <f>Revenue!I114</f>
         <v/>
       </c>
       <c r="J17" s="31">
-        <f>Revenue!J101</f>
+        <f>Revenue!J114</f>
         <v/>
       </c>
       <c r="K17" s="31">
-        <f>Revenue!K101</f>
+        <f>Revenue!K114</f>
         <v/>
       </c>
     </row>
@@ -5245,16 +5857,16 @@
           <t>Costs</t>
         </is>
       </c>
-      <c r="B19" s="38" t="n"/>
-      <c r="C19" s="38" t="n"/>
-      <c r="D19" s="38" t="n"/>
-      <c r="E19" s="38" t="n"/>
-      <c r="F19" s="38" t="n"/>
-      <c r="G19" s="38" t="n"/>
-      <c r="H19" s="38" t="n"/>
-      <c r="I19" s="38" t="n"/>
-      <c r="J19" s="38" t="n"/>
-      <c r="K19" s="38" t="n"/>
+      <c r="B19" s="60" t="n"/>
+      <c r="C19" s="60" t="n"/>
+      <c r="D19" s="60" t="n"/>
+      <c r="E19" s="60" t="n"/>
+      <c r="F19" s="60" t="n"/>
+      <c r="G19" s="60" t="n"/>
+      <c r="H19" s="60" t="n"/>
+      <c r="I19" s="60" t="n"/>
+      <c r="J19" s="60" t="n"/>
+      <c r="K19" s="60" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="20">
       <c r="A20" s="24" t="inlineStr">
@@ -5820,7 +6432,7 @@
           <t xml:space="preserve">  Venue (Swiss House)</t>
         </is>
       </c>
-      <c r="B16" s="36" t="n">
+      <c r="B16" s="37" t="n">
         <v>27951</v>
       </c>
       <c r="C16" s="29">
@@ -5866,7 +6478,7 @@
           <t xml:space="preserve">  F&amp;B Credit (guest spend vs minimums)</t>
         </is>
       </c>
-      <c r="B17" s="36" t="n">
+      <c r="B17" s="37" t="n">
         <v>-9000</v>
       </c>
       <c r="C17" s="29">
@@ -5912,7 +6524,7 @@
           <t xml:space="preserve">  Insurance / Permits / Ticketing</t>
         </is>
       </c>
-      <c r="B18" s="36" t="n">
+      <c r="B18" s="37" t="n">
         <v>2500</v>
       </c>
       <c r="C18" s="29">
@@ -5958,7 +6570,7 @@
           <t xml:space="preserve">  Transport</t>
         </is>
       </c>
-      <c r="B19" s="36" t="n">
+      <c r="B19" s="37" t="n">
         <v>2500</v>
       </c>
       <c r="C19" s="29">
@@ -6004,7 +6616,7 @@
           <t xml:space="preserve">  Sunday Program (incl. GRÜEZI coffee costs)</t>
         </is>
       </c>
-      <c r="B20" s="36" t="n">
+      <c r="B20" s="37" t="n">
         <v>1000</v>
       </c>
       <c r="C20" s="29">
@@ -6149,7 +6761,7 @@
           <t xml:space="preserve">  Welcome Drinks (Ticket Count × 2 × CHF 9)</t>
         </is>
       </c>
-      <c r="B26" s="36" t="n">
+      <c r="B26" s="37" t="n">
         <v>4500</v>
       </c>
       <c r="C26" s="29">
@@ -6195,7 +6807,7 @@
           <t xml:space="preserve">  Security</t>
         </is>
       </c>
-      <c r="B27" s="36" t="n">
+      <c r="B27" s="37" t="n">
         <v>4500</v>
       </c>
       <c r="C27" s="29">
@@ -6340,7 +6952,7 @@
           <t xml:space="preserve">  Talent (DJs / Artists)</t>
         </is>
       </c>
-      <c r="B33" s="36" t="n">
+      <c r="B33" s="37" t="n">
         <v>18000</v>
       </c>
       <c r="C33" s="29">
@@ -6386,7 +6998,7 @@
           <t xml:space="preserve">  Production (Sound / Lighting)</t>
         </is>
       </c>
-      <c r="B34" s="36" t="n">
+      <c r="B34" s="37" t="n">
         <v>12000</v>
       </c>
       <c r="C34" s="29">
@@ -6432,7 +7044,7 @@
           <t xml:space="preserve">  Decor / Branding</t>
         </is>
       </c>
-      <c r="B35" s="36" t="n">
+      <c r="B35" s="37" t="n">
         <v>3500</v>
       </c>
       <c r="C35" s="29">
@@ -6478,7 +7090,7 @@
           <t xml:space="preserve">  Photo / Video</t>
         </is>
       </c>
-      <c r="B36" s="36" t="n">
+      <c r="B36" s="37" t="n">
         <v>5000</v>
       </c>
       <c r="C36" s="29">
@@ -6524,7 +7136,7 @@
           <t xml:space="preserve">  Marketing / Print</t>
         </is>
       </c>
-      <c r="B37" s="36" t="n">
+      <c r="B37" s="37" t="n">
         <v>2000</v>
       </c>
       <c r="C37" s="29">
@@ -6570,7 +7182,7 @@
           <t xml:space="preserve">  Operating Partner</t>
         </is>
       </c>
-      <c r="B38" s="36" t="n">
+      <c r="B38" s="37" t="n">
         <v>6000</v>
       </c>
       <c r="C38" s="29">
@@ -6616,7 +7228,7 @@
           <t xml:space="preserve">  Chedi Winter Garden (Friday)</t>
         </is>
       </c>
-      <c r="B39" s="36" t="n">
+      <c r="B39" s="37" t="n">
         <v>2500</v>
       </c>
       <c r="C39" s="29">
@@ -7047,34 +7659,34 @@
           <t>Overhead (manual input)</t>
         </is>
       </c>
-      <c r="B53" s="36" t="n">
+      <c r="B53" s="37" t="n">
         <v>8000</v>
       </c>
-      <c r="C53" s="36" t="n">
+      <c r="C53" s="37" t="n">
         <v>8000</v>
       </c>
-      <c r="D53" s="36" t="n">
+      <c r="D53" s="37" t="n">
         <v>8000</v>
       </c>
-      <c r="E53" s="36" t="n">
+      <c r="E53" s="37" t="n">
         <v>39000</v>
       </c>
-      <c r="F53" s="36" t="n">
+      <c r="F53" s="37" t="n">
         <v>39000</v>
       </c>
-      <c r="G53" s="36" t="n">
+      <c r="G53" s="37" t="n">
         <v>39000</v>
       </c>
-      <c r="H53" s="36" t="n">
+      <c r="H53" s="37" t="n">
         <v>55000</v>
       </c>
-      <c r="I53" s="36" t="n">
+      <c r="I53" s="37" t="n">
         <v>56000</v>
       </c>
-      <c r="J53" s="36" t="n">
+      <c r="J53" s="37" t="n">
         <v>58000</v>
       </c>
-      <c r="K53" s="36" t="n">
+      <c r="K53" s="37" t="n">
         <v>60000</v>
       </c>
     </row>
@@ -7091,19 +7703,19 @@
           <t>Founder Pay (2027-2031: manual / 2032+: auto +4%/yr)</t>
         </is>
       </c>
-      <c r="B55" s="36" t="n">
+      <c r="B55" s="37" t="n">
         <v>10000</v>
       </c>
-      <c r="C55" s="36" t="n">
+      <c r="C55" s="37" t="n">
         <v>20000</v>
       </c>
-      <c r="D55" s="36" t="n">
+      <c r="D55" s="37" t="n">
         <v>30000</v>
       </c>
-      <c r="E55" s="36" t="n">
+      <c r="E55" s="37" t="n">
         <v>50000</v>
       </c>
-      <c r="F55" s="36" t="n">
+      <c r="F55" s="37" t="n">
         <v>70000</v>
       </c>
       <c r="G55" s="29">

</xml_diff>

<commit_message>
Cost sheet: rename header to MODEL ASSUMPTIONS, add TOTAL COST row
- Rename "GLOBAL COST VARIABLES" to "MODEL ASSUMPTIONS" with same
  visual style as Revenue sheet (gray background + navy text)
- Add TOTAL COST row (row 57) = Direct Cost + Overhead + Founder Pay
  with section header styling
- F&B Credit keeps 3% venue contract escalation rate

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -6277,7 +6277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="42" customWidth="1" style="19" min="1" max="1"/>
@@ -6293,9 +6293,9 @@
     </row>
     <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="20">
-      <c r="A3" s="22" t="inlineStr">
-        <is>
-          <t>GLOBAL COST VARIABLES</t>
+      <c r="A3" s="36" t="inlineStr">
+        <is>
+          <t>MODEL ASSUMPTIONS</t>
         </is>
       </c>
       <c r="B3" s="22" t="n"/>
@@ -7739,6 +7739,54 @@
         <v/>
       </c>
     </row>
+    <row r="56"/>
+    <row r="57">
+      <c r="A57" s="58" t="inlineStr">
+        <is>
+          <t>TOTAL COST</t>
+        </is>
+      </c>
+      <c r="B57">
+        <f>B49+B53+B55</f>
+        <v/>
+      </c>
+      <c r="C57">
+        <f>C49+C53+C55</f>
+        <v/>
+      </c>
+      <c r="D57">
+        <f>D49+D53+D55</f>
+        <v/>
+      </c>
+      <c r="E57">
+        <f>E49+E53+E55</f>
+        <v/>
+      </c>
+      <c r="F57">
+        <f>F49+F53+F55</f>
+        <v/>
+      </c>
+      <c r="G57">
+        <f>G49+G53+G55</f>
+        <v/>
+      </c>
+      <c r="H57">
+        <f>H49+H53+H55</f>
+        <v/>
+      </c>
+      <c r="I57">
+        <f>I49+I53+I55</f>
+        <v/>
+      </c>
+      <c r="J57">
+        <f>J49+J53+J55</f>
+        <v/>
+      </c>
+      <c r="K57">
+        <f>K49+K53+K55</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CC0B"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Add comment to F&B Credit explaining 9,000 CHF treatment
BP lists 'Bar/F&B (net) = 9,000' as revenue, but per Rox confirmation
Aura receives no bar/food sales share. The 9,000 is a deposit-style
credit on the cost side, not revenue. Excel comment on Cost!A17 explains.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -916,6 +916,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Unknown Author</author>
+    <author>Model Note</author>
   </authors>
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0">
@@ -936,6 +937,11 @@
     <comment ref="B16" authorId="0" shapeId="0">
       <text>
         <t>BP assumption table says '27,550 + VAT' but detailed calculation shows 27,951 incl. VAT. Only Gütsch (4,950) is quoted excl. VAT; other venues are F&amp;B minimums incl. VAT.</t>
+      </text>
+    </comment>
+    <comment ref="A17" authorId="1" shapeId="0">
+      <text>
+        <t>BP shows 'Bar/F&amp;B (net) = 9,000 CHF' as revenue, but per Rox confirmation, Aura receives no share of bar/food sales. This 9,000 is a deposit-style credit: guests are expected to spend more than 9,000 at the venue, so the excess offsets venue costs. It is correctly recorded here as a cost reduction, not as revenue.</t>
       </text>
     </comment>
     <comment ref="B17" authorId="0" shapeId="0">

</xml_diff>

<commit_message>
Implement new 6-factor scenario model in Dashboard
Replace the old 3-factor model (Ticket Occ / Partnership / Cost Overrun)
with 6 granular factors aligned to the Business Plan:
- Ticket Occupancy, Ticket Price Factor, Partnership Factor, ASA Factor
- Summer Start Year (per scenario), Founder Pay Factor

Downside: 85% occ, 90% price, 60% partnership, 75% ASA, summer 2029, 50% founder pay
Base: all 1.0, summer 2027
Upside: 110% price, 140% partnership, 125% ASA, summer 2027

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -126,6 +126,11 @@
     <font>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -191,7 +196,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -286,13 +291,42 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -300,10 +334,7 @@
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -311,39 +342,24 @@
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
     <xf numFmtId="3" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="3" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -356,16 +372,12 @@
     <xf numFmtId="1" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
     <xf numFmtId="3" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1201,7 +1213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="35" customWidth="1" style="19" min="1" max="1"/>
@@ -1356,43 +1368,43 @@
         </is>
       </c>
       <c r="B12" s="29">
-        <f>'P&amp;L'!B10*$C$60</f>
+        <f>'P&amp;L'!B10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="C12" s="29">
-        <f>'P&amp;L'!C10*$C$60</f>
+        <f>'P&amp;L'!C10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="D12" s="29">
-        <f>'P&amp;L'!D10*$C$60</f>
+        <f>'P&amp;L'!D10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="E12" s="29">
-        <f>'P&amp;L'!E10*$C$60</f>
+        <f>'P&amp;L'!E10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="F12" s="29">
-        <f>'P&amp;L'!F10*$C$60</f>
+        <f>'P&amp;L'!F10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="G12" s="29">
-        <f>'P&amp;L'!G10*$C$60</f>
+        <f>'P&amp;L'!G10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="H12" s="29">
-        <f>'P&amp;L'!H10*$C$60</f>
+        <f>'P&amp;L'!H10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="I12" s="29">
-        <f>'P&amp;L'!I10*$C$60</f>
+        <f>'P&amp;L'!I10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="J12" s="29">
-        <f>'P&amp;L'!J10*$C$60</f>
+        <f>'P&amp;L'!J10*$C$60*$C$61</f>
         <v/>
       </c>
       <c r="K12" s="29">
-        <f>'P&amp;L'!K10*$C$60</f>
+        <f>'P&amp;L'!K10*$C$60*$C$61</f>
         <v/>
       </c>
     </row>
@@ -1403,43 +1415,43 @@
         </is>
       </c>
       <c r="B13" s="29">
-        <f>'P&amp;L'!B11*$C$61</f>
+        <f>'P&amp;L'!B11*$C$62</f>
         <v/>
       </c>
       <c r="C13" s="29">
-        <f>'P&amp;L'!C11*$C$61</f>
+        <f>'P&amp;L'!C11*$C$62</f>
         <v/>
       </c>
       <c r="D13" s="29">
-        <f>'P&amp;L'!D11*$C$61</f>
+        <f>'P&amp;L'!D11*$C$62</f>
         <v/>
       </c>
       <c r="E13" s="29">
-        <f>'P&amp;L'!E11*$C$61</f>
+        <f>'P&amp;L'!E11*$C$62</f>
         <v/>
       </c>
       <c r="F13" s="29">
-        <f>'P&amp;L'!F11*$C$61</f>
+        <f>'P&amp;L'!F11*$C$62</f>
         <v/>
       </c>
       <c r="G13" s="29">
-        <f>'P&amp;L'!G11*$C$61</f>
+        <f>'P&amp;L'!G11*$C$62</f>
         <v/>
       </c>
       <c r="H13" s="29">
-        <f>'P&amp;L'!H11*$C$61</f>
+        <f>'P&amp;L'!H11*$C$62</f>
         <v/>
       </c>
       <c r="I13" s="29">
-        <f>'P&amp;L'!I11*$C$61</f>
+        <f>'P&amp;L'!I11*$C$62</f>
         <v/>
       </c>
       <c r="J13" s="29">
-        <f>'P&amp;L'!J11*$C$61</f>
+        <f>'P&amp;L'!J11*$C$62</f>
         <v/>
       </c>
       <c r="K13" s="29">
-        <f>'P&amp;L'!K11*$C$61</f>
+        <f>'P&amp;L'!K11*$C$62</f>
         <v/>
       </c>
     </row>
@@ -1450,43 +1462,43 @@
         </is>
       </c>
       <c r="B14" s="29">
-        <f>'P&amp;L'!B12+'P&amp;L'!B13+'P&amp;L'!B14+'P&amp;L'!B15</f>
+        <f>'P&amp;L'!B12*$C$63+'P&amp;L'!B13+'P&amp;L'!B14+'P&amp;L'!B15</f>
         <v/>
       </c>
       <c r="C14" s="29">
-        <f>'P&amp;L'!C12+'P&amp;L'!C13+'P&amp;L'!C14+'P&amp;L'!C15</f>
+        <f>'P&amp;L'!C12*$C$63+'P&amp;L'!C13+'P&amp;L'!C14+'P&amp;L'!C15</f>
         <v/>
       </c>
       <c r="D14" s="29">
-        <f>'P&amp;L'!D12+'P&amp;L'!D13+'P&amp;L'!D14+'P&amp;L'!D15</f>
+        <f>'P&amp;L'!D12*$C$63+'P&amp;L'!D13+'P&amp;L'!D14+'P&amp;L'!D15</f>
         <v/>
       </c>
       <c r="E14" s="29">
-        <f>'P&amp;L'!E12+'P&amp;L'!E13+'P&amp;L'!E14+'P&amp;L'!E15</f>
+        <f>'P&amp;L'!E12*$C$63+'P&amp;L'!E13+'P&amp;L'!E14+'P&amp;L'!E15</f>
         <v/>
       </c>
       <c r="F14" s="29">
-        <f>'P&amp;L'!F12+'P&amp;L'!F13+'P&amp;L'!F14+'P&amp;L'!F15</f>
+        <f>'P&amp;L'!F12*$C$63+'P&amp;L'!F13+'P&amp;L'!F14+'P&amp;L'!F15</f>
         <v/>
       </c>
       <c r="G14" s="29">
-        <f>'P&amp;L'!G12+'P&amp;L'!G13+'P&amp;L'!G14+'P&amp;L'!G15</f>
+        <f>'P&amp;L'!G12*$C$63+'P&amp;L'!G13+'P&amp;L'!G14+'P&amp;L'!G15</f>
         <v/>
       </c>
       <c r="H14" s="29">
-        <f>'P&amp;L'!H12+'P&amp;L'!H13+'P&amp;L'!H14+'P&amp;L'!H15</f>
+        <f>'P&amp;L'!H12*$C$63+'P&amp;L'!H13+'P&amp;L'!H14+'P&amp;L'!H15</f>
         <v/>
       </c>
       <c r="I14" s="29">
-        <f>'P&amp;L'!I12+'P&amp;L'!I13+'P&amp;L'!I14+'P&amp;L'!I15</f>
+        <f>'P&amp;L'!I12*$C$63+'P&amp;L'!I13+'P&amp;L'!I14+'P&amp;L'!I15</f>
         <v/>
       </c>
       <c r="J14" s="29">
-        <f>'P&amp;L'!J12+'P&amp;L'!J13+'P&amp;L'!J14+'P&amp;L'!J15</f>
+        <f>'P&amp;L'!J12*$C$63+'P&amp;L'!J13+'P&amp;L'!J14+'P&amp;L'!J15</f>
         <v/>
       </c>
       <c r="K14" s="29">
-        <f>'P&amp;L'!K12+'P&amp;L'!K13+'P&amp;L'!K14+'P&amp;L'!K15</f>
+        <f>'P&amp;L'!K12*$C$63+'P&amp;L'!K13+'P&amp;L'!K14+'P&amp;L'!K15</f>
         <v/>
       </c>
     </row>
@@ -1497,43 +1509,43 @@
         </is>
       </c>
       <c r="B15" s="25">
-        <f>(B12+B13+B14)*(1+IF(2027&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(B12+B13+B14)*(1+IF(2027&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="C15" s="25">
-        <f>(C12+C13+C14)*(1+IF(2028&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(C12+C13+C14)*(1+IF(2028&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="D15" s="25">
-        <f>(D12+D13+D14)*(1+IF(2029&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(D12+D13+D14)*(1+IF(2029&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="E15" s="25">
-        <f>(E12+E13+E14)*(1+IF(2030&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(E12+E13+E14)*(1+IF(2030&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="F15" s="25">
-        <f>(F12+F13+F14)*(1+IF(2031&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(F12+F13+F14)*(1+IF(2031&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="G15" s="25">
-        <f>(G12+G13+G14)*(1+IF(2032&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(G12+G13+G14)*(1+IF(2032&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="H15" s="25">
-        <f>(H12+H13+H14)*(1+IF(2033&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(H12+H13+H14)*(1+IF(2033&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="I15" s="25">
-        <f>(I12+I13+I14)*(1+IF(2034&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(I12+I13+I14)*(1+IF(2034&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="J15" s="25">
-        <f>(J12+J13+J14)*(1+IF(2035&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(J12+J13+J14)*(1+IF(2035&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="K15" s="25">
-        <f>(K12+K13+K14)*(1+IF(2036&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(K12+K13+K14)*(1+IF(2036&gt;=$C$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
     </row>
@@ -1544,43 +1556,43 @@
         </is>
       </c>
       <c r="B16" s="29">
-        <f>'P&amp;L'!B24*$C$62</f>
+        <f>'P&amp;L'!B20+'P&amp;L'!B21+'P&amp;L'!B22*$C$67</f>
         <v/>
       </c>
       <c r="C16" s="29">
-        <f>'P&amp;L'!C24*$C$62</f>
+        <f>'P&amp;L'!C20+'P&amp;L'!C21+'P&amp;L'!C22*$C$67</f>
         <v/>
       </c>
       <c r="D16" s="29">
-        <f>'P&amp;L'!D24*$C$62</f>
+        <f>'P&amp;L'!D20+'P&amp;L'!D21+'P&amp;L'!D22*$C$67</f>
         <v/>
       </c>
       <c r="E16" s="29">
-        <f>'P&amp;L'!E24*$C$62</f>
+        <f>'P&amp;L'!E20+'P&amp;L'!E21+'P&amp;L'!E22*$C$67</f>
         <v/>
       </c>
       <c r="F16" s="29">
-        <f>'P&amp;L'!F24*$C$62</f>
+        <f>'P&amp;L'!F20+'P&amp;L'!F21+'P&amp;L'!F22*$C$67</f>
         <v/>
       </c>
       <c r="G16" s="29">
-        <f>'P&amp;L'!G24*$C$62</f>
+        <f>'P&amp;L'!G20+'P&amp;L'!G21+'P&amp;L'!G22*$C$67</f>
         <v/>
       </c>
       <c r="H16" s="29">
-        <f>'P&amp;L'!H24*$C$62</f>
+        <f>'P&amp;L'!H20+'P&amp;L'!H21+'P&amp;L'!H22*$C$67</f>
         <v/>
       </c>
       <c r="I16" s="29">
-        <f>'P&amp;L'!I24*$C$62</f>
+        <f>'P&amp;L'!I20+'P&amp;L'!I21+'P&amp;L'!I22*$C$67</f>
         <v/>
       </c>
       <c r="J16" s="29">
-        <f>'P&amp;L'!J24*$C$62</f>
+        <f>'P&amp;L'!J20+'P&amp;L'!J21+'P&amp;L'!J22*$C$67</f>
         <v/>
       </c>
       <c r="K16" s="29">
-        <f>'P&amp;L'!K24*$C$62</f>
+        <f>'P&amp;L'!K20+'P&amp;L'!K21+'P&amp;L'!K22*$C$67</f>
         <v/>
       </c>
     </row>
@@ -1820,43 +1832,43 @@
         </is>
       </c>
       <c r="B24" s="29">
-        <f>'P&amp;L'!B10*$B$60</f>
+        <f>'P&amp;L'!B10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="C24" s="29">
-        <f>'P&amp;L'!C10*$B$60</f>
+        <f>'P&amp;L'!C10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="D24" s="29">
-        <f>'P&amp;L'!D10*$B$60</f>
+        <f>'P&amp;L'!D10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="E24" s="29">
-        <f>'P&amp;L'!E10*$B$60</f>
+        <f>'P&amp;L'!E10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="F24" s="29">
-        <f>'P&amp;L'!F10*$B$60</f>
+        <f>'P&amp;L'!F10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="G24" s="29">
-        <f>'P&amp;L'!G10*$B$60</f>
+        <f>'P&amp;L'!G10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="H24" s="29">
-        <f>'P&amp;L'!H10*$B$60</f>
+        <f>'P&amp;L'!H10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="I24" s="29">
-        <f>'P&amp;L'!I10*$B$60</f>
+        <f>'P&amp;L'!I10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="J24" s="29">
-        <f>'P&amp;L'!J10*$B$60</f>
+        <f>'P&amp;L'!J10*$B$60*$B$61</f>
         <v/>
       </c>
       <c r="K24" s="29">
-        <f>'P&amp;L'!K10*$B$60</f>
+        <f>'P&amp;L'!K10*$B$60*$B$61</f>
         <v/>
       </c>
     </row>
@@ -1867,90 +1879,90 @@
         </is>
       </c>
       <c r="B25" s="29">
-        <f>'P&amp;L'!B11*$B$61</f>
+        <f>'P&amp;L'!B11*$B$62</f>
         <v/>
       </c>
       <c r="C25" s="29">
-        <f>'P&amp;L'!C11*$B$61</f>
+        <f>'P&amp;L'!C11*$B$62</f>
         <v/>
       </c>
       <c r="D25" s="29">
-        <f>'P&amp;L'!D11*$B$61</f>
+        <f>'P&amp;L'!D11*$B$62</f>
         <v/>
       </c>
       <c r="E25" s="29">
-        <f>'P&amp;L'!E11*$B$61</f>
+        <f>'P&amp;L'!E11*$B$62</f>
         <v/>
       </c>
       <c r="F25" s="29">
-        <f>'P&amp;L'!F11*$B$61</f>
+        <f>'P&amp;L'!F11*$B$62</f>
         <v/>
       </c>
       <c r="G25" s="29">
-        <f>'P&amp;L'!G11*$B$61</f>
+        <f>'P&amp;L'!G11*$B$62</f>
         <v/>
       </c>
       <c r="H25" s="29">
-        <f>'P&amp;L'!H11*$B$61</f>
+        <f>'P&amp;L'!H11*$B$62</f>
         <v/>
       </c>
       <c r="I25" s="29">
-        <f>'P&amp;L'!I11*$B$61</f>
+        <f>'P&amp;L'!I11*$B$62</f>
         <v/>
       </c>
       <c r="J25" s="29">
-        <f>'P&amp;L'!J11*$B$61</f>
+        <f>'P&amp;L'!J11*$B$62</f>
         <v/>
       </c>
       <c r="K25" s="29">
-        <f>'P&amp;L'!K11*$B$61</f>
+        <f>'P&amp;L'!K11*$B$62</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="20">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Other Revenue (ASA + F&amp;B + Dinner + Other)</t>
+          <t xml:space="preserve">    Other Revenue (ASA+F&amp;B+Dinner+Other) (adj.)</t>
         </is>
       </c>
       <c r="B26" s="29">
-        <f>'P&amp;L'!B12+'P&amp;L'!B13+'P&amp;L'!B14+'P&amp;L'!B15</f>
+        <f>'P&amp;L'!B12*$B$63+'P&amp;L'!B13+'P&amp;L'!B14+'P&amp;L'!B15</f>
         <v/>
       </c>
       <c r="C26" s="29">
-        <f>'P&amp;L'!C12+'P&amp;L'!C13+'P&amp;L'!C14+'P&amp;L'!C15</f>
+        <f>'P&amp;L'!C12*$B$63+'P&amp;L'!C13+'P&amp;L'!C14+'P&amp;L'!C15</f>
         <v/>
       </c>
       <c r="D26" s="29">
-        <f>'P&amp;L'!D12+'P&amp;L'!D13+'P&amp;L'!D14+'P&amp;L'!D15</f>
+        <f>'P&amp;L'!D12*$B$63+'P&amp;L'!D13+'P&amp;L'!D14+'P&amp;L'!D15</f>
         <v/>
       </c>
       <c r="E26" s="29">
-        <f>'P&amp;L'!E12+'P&amp;L'!E13+'P&amp;L'!E14+'P&amp;L'!E15</f>
+        <f>'P&amp;L'!E12*$B$63+'P&amp;L'!E13+'P&amp;L'!E14+'P&amp;L'!E15</f>
         <v/>
       </c>
       <c r="F26" s="29">
-        <f>'P&amp;L'!F12+'P&amp;L'!F13+'P&amp;L'!F14+'P&amp;L'!F15</f>
+        <f>'P&amp;L'!F12*$B$63+'P&amp;L'!F13+'P&amp;L'!F14+'P&amp;L'!F15</f>
         <v/>
       </c>
       <c r="G26" s="29">
-        <f>'P&amp;L'!G12+'P&amp;L'!G13+'P&amp;L'!G14+'P&amp;L'!G15</f>
+        <f>'P&amp;L'!G12*$B$63+'P&amp;L'!G13+'P&amp;L'!G14+'P&amp;L'!G15</f>
         <v/>
       </c>
       <c r="H26" s="29">
-        <f>'P&amp;L'!H12+'P&amp;L'!H13+'P&amp;L'!H14+'P&amp;L'!H15</f>
+        <f>'P&amp;L'!H12*$B$63+'P&amp;L'!H13+'P&amp;L'!H14+'P&amp;L'!H15</f>
         <v/>
       </c>
       <c r="I26" s="29">
-        <f>'P&amp;L'!I12+'P&amp;L'!I13+'P&amp;L'!I14+'P&amp;L'!I15</f>
+        <f>'P&amp;L'!I12*$B$63+'P&amp;L'!I13+'P&amp;L'!I14+'P&amp;L'!I15</f>
         <v/>
       </c>
       <c r="J26" s="29">
-        <f>'P&amp;L'!J12+'P&amp;L'!J13+'P&amp;L'!J14+'P&amp;L'!J15</f>
+        <f>'P&amp;L'!J12*$B$63+'P&amp;L'!J13+'P&amp;L'!J14+'P&amp;L'!J15</f>
         <v/>
       </c>
       <c r="K26" s="29">
-        <f>'P&amp;L'!K12+'P&amp;L'!K13+'P&amp;L'!K14+'P&amp;L'!K15</f>
+        <f>'P&amp;L'!K12*$B$63+'P&amp;L'!K13+'P&amp;L'!K14+'P&amp;L'!K15</f>
         <v/>
       </c>
     </row>
@@ -1961,43 +1973,43 @@
         </is>
       </c>
       <c r="B27" s="25">
-        <f>(B24+B25+B26)*(1+IF(2027&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(B24+B25+B26)*(1+IF(2027&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="C27" s="25">
-        <f>(C24+C25+C26)*(1+IF(2028&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(C24+C25+C26)*(1+IF(2028&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="D27" s="25">
-        <f>(D24+D25+D26)*(1+IF(2029&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(D24+D25+D26)*(1+IF(2029&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="E27" s="25">
-        <f>(E24+E25+E26)*(1+IF(2030&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(E24+E25+E26)*(1+IF(2030&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="F27" s="25">
-        <f>(F24+F25+F26)*(1+IF(2031&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(F24+F25+F26)*(1+IF(2031&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="G27" s="25">
-        <f>(G24+G25+G26)*(1+IF(2032&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(G24+G25+G26)*(1+IF(2032&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="H27" s="25">
-        <f>(H24+H25+H26)*(1+IF(2033&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(H24+H25+H26)*(1+IF(2033&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="I27" s="25">
-        <f>(I24+I25+I26)*(1+IF(2034&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(I24+I25+I26)*(1+IF(2034&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="J27" s="25">
-        <f>(J24+J25+J26)*(1+IF(2035&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(J24+J25+J26)*(1+IF(2035&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="K27" s="25">
-        <f>(K24+K25+K26)*(1+IF(2036&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(K24+K25+K26)*(1+IF(2036&gt;=$B$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
     </row>
@@ -2008,43 +2020,43 @@
         </is>
       </c>
       <c r="B28" s="29">
-        <f>'P&amp;L'!B24*$B$62</f>
+        <f>'P&amp;L'!B20+'P&amp;L'!B21+'P&amp;L'!B22*$B$67</f>
         <v/>
       </c>
       <c r="C28" s="29">
-        <f>'P&amp;L'!C24*$B$62</f>
+        <f>'P&amp;L'!C20+'P&amp;L'!C21+'P&amp;L'!C22*$B$67</f>
         <v/>
       </c>
       <c r="D28" s="29">
-        <f>'P&amp;L'!D24*$B$62</f>
+        <f>'P&amp;L'!D20+'P&amp;L'!D21+'P&amp;L'!D22*$B$67</f>
         <v/>
       </c>
       <c r="E28" s="29">
-        <f>'P&amp;L'!E24*$B$62</f>
+        <f>'P&amp;L'!E20+'P&amp;L'!E21+'P&amp;L'!E22*$B$67</f>
         <v/>
       </c>
       <c r="F28" s="29">
-        <f>'P&amp;L'!F24*$B$62</f>
+        <f>'P&amp;L'!F20+'P&amp;L'!F21+'P&amp;L'!F22*$B$67</f>
         <v/>
       </c>
       <c r="G28" s="29">
-        <f>'P&amp;L'!G24*$B$62</f>
+        <f>'P&amp;L'!G20+'P&amp;L'!G21+'P&amp;L'!G22*$B$67</f>
         <v/>
       </c>
       <c r="H28" s="29">
-        <f>'P&amp;L'!H24*$B$62</f>
+        <f>'P&amp;L'!H20+'P&amp;L'!H21+'P&amp;L'!H22*$B$67</f>
         <v/>
       </c>
       <c r="I28" s="29">
-        <f>'P&amp;L'!I24*$B$62</f>
+        <f>'P&amp;L'!I20+'P&amp;L'!I21+'P&amp;L'!I22*$B$67</f>
         <v/>
       </c>
       <c r="J28" s="29">
-        <f>'P&amp;L'!J24*$B$62</f>
+        <f>'P&amp;L'!J20+'P&amp;L'!J21+'P&amp;L'!J22*$B$67</f>
         <v/>
       </c>
       <c r="K28" s="29">
-        <f>'P&amp;L'!K24*$B$62</f>
+        <f>'P&amp;L'!K20+'P&amp;L'!K21+'P&amp;L'!K22*$B$67</f>
         <v/>
       </c>
     </row>
@@ -2284,43 +2296,43 @@
         </is>
       </c>
       <c r="B36" s="29">
-        <f>'P&amp;L'!B10*$D$60</f>
+        <f>'P&amp;L'!B10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="C36" s="29">
-        <f>'P&amp;L'!C10*$D$60</f>
+        <f>'P&amp;L'!C10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="D36" s="29">
-        <f>'P&amp;L'!D10*$D$60</f>
+        <f>'P&amp;L'!D10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="E36" s="29">
-        <f>'P&amp;L'!E10*$D$60</f>
+        <f>'P&amp;L'!E10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="F36" s="29">
-        <f>'P&amp;L'!F10*$D$60</f>
+        <f>'P&amp;L'!F10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="G36" s="29">
-        <f>'P&amp;L'!G10*$D$60</f>
+        <f>'P&amp;L'!G10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="H36" s="29">
-        <f>'P&amp;L'!H10*$D$60</f>
+        <f>'P&amp;L'!H10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="I36" s="29">
-        <f>'P&amp;L'!I10*$D$60</f>
+        <f>'P&amp;L'!I10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="J36" s="29">
-        <f>'P&amp;L'!J10*$D$60</f>
+        <f>'P&amp;L'!J10*$D$60*$D$61</f>
         <v/>
       </c>
       <c r="K36" s="29">
-        <f>'P&amp;L'!K10*$D$60</f>
+        <f>'P&amp;L'!K10*$D$60*$D$61</f>
         <v/>
       </c>
     </row>
@@ -2331,90 +2343,90 @@
         </is>
       </c>
       <c r="B37" s="29">
-        <f>'P&amp;L'!B11*$D$61</f>
+        <f>'P&amp;L'!B11*$D$62</f>
         <v/>
       </c>
       <c r="C37" s="29">
-        <f>'P&amp;L'!C11*$D$61</f>
+        <f>'P&amp;L'!C11*$D$62</f>
         <v/>
       </c>
       <c r="D37" s="29">
-        <f>'P&amp;L'!D11*$D$61</f>
+        <f>'P&amp;L'!D11*$D$62</f>
         <v/>
       </c>
       <c r="E37" s="29">
-        <f>'P&amp;L'!E11*$D$61</f>
+        <f>'P&amp;L'!E11*$D$62</f>
         <v/>
       </c>
       <c r="F37" s="29">
-        <f>'P&amp;L'!F11*$D$61</f>
+        <f>'P&amp;L'!F11*$D$62</f>
         <v/>
       </c>
       <c r="G37" s="29">
-        <f>'P&amp;L'!G11*$D$61</f>
+        <f>'P&amp;L'!G11*$D$62</f>
         <v/>
       </c>
       <c r="H37" s="29">
-        <f>'P&amp;L'!H11*$D$61</f>
+        <f>'P&amp;L'!H11*$D$62</f>
         <v/>
       </c>
       <c r="I37" s="29">
-        <f>'P&amp;L'!I11*$D$61</f>
+        <f>'P&amp;L'!I11*$D$62</f>
         <v/>
       </c>
       <c r="J37" s="29">
-        <f>'P&amp;L'!J11*$D$61</f>
+        <f>'P&amp;L'!J11*$D$62</f>
         <v/>
       </c>
       <c r="K37" s="29">
-        <f>'P&amp;L'!K11*$D$61</f>
+        <f>'P&amp;L'!K11*$D$62</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="20">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Other Revenue (ASA + F&amp;B + Dinner + Other)</t>
+          <t xml:space="preserve">    Other Revenue (ASA+F&amp;B+Dinner+Other) (adj.)</t>
         </is>
       </c>
       <c r="B38" s="29">
-        <f>'P&amp;L'!B12+'P&amp;L'!B13+'P&amp;L'!B14+'P&amp;L'!B15</f>
+        <f>'P&amp;L'!B12*$D$63+'P&amp;L'!B13+'P&amp;L'!B14+'P&amp;L'!B15</f>
         <v/>
       </c>
       <c r="C38" s="29">
-        <f>'P&amp;L'!C12+'P&amp;L'!C13+'P&amp;L'!C14+'P&amp;L'!C15</f>
+        <f>'P&amp;L'!C12*$D$63+'P&amp;L'!C13+'P&amp;L'!C14+'P&amp;L'!C15</f>
         <v/>
       </c>
       <c r="D38" s="29">
-        <f>'P&amp;L'!D12+'P&amp;L'!D13+'P&amp;L'!D14+'P&amp;L'!D15</f>
+        <f>'P&amp;L'!D12*$D$63+'P&amp;L'!D13+'P&amp;L'!D14+'P&amp;L'!D15</f>
         <v/>
       </c>
       <c r="E38" s="29">
-        <f>'P&amp;L'!E12+'P&amp;L'!E13+'P&amp;L'!E14+'P&amp;L'!E15</f>
+        <f>'P&amp;L'!E12*$D$63+'P&amp;L'!E13+'P&amp;L'!E14+'P&amp;L'!E15</f>
         <v/>
       </c>
       <c r="F38" s="29">
-        <f>'P&amp;L'!F12+'P&amp;L'!F13+'P&amp;L'!F14+'P&amp;L'!F15</f>
+        <f>'P&amp;L'!F12*$D$63+'P&amp;L'!F13+'P&amp;L'!F14+'P&amp;L'!F15</f>
         <v/>
       </c>
       <c r="G38" s="29">
-        <f>'P&amp;L'!G12+'P&amp;L'!G13+'P&amp;L'!G14+'P&amp;L'!G15</f>
+        <f>'P&amp;L'!G12*$D$63+'P&amp;L'!G13+'P&amp;L'!G14+'P&amp;L'!G15</f>
         <v/>
       </c>
       <c r="H38" s="29">
-        <f>'P&amp;L'!H12+'P&amp;L'!H13+'P&amp;L'!H14+'P&amp;L'!H15</f>
+        <f>'P&amp;L'!H12*$D$63+'P&amp;L'!H13+'P&amp;L'!H14+'P&amp;L'!H15</f>
         <v/>
       </c>
       <c r="I38" s="29">
-        <f>'P&amp;L'!I12+'P&amp;L'!I13+'P&amp;L'!I14+'P&amp;L'!I15</f>
+        <f>'P&amp;L'!I12*$D$63+'P&amp;L'!I13+'P&amp;L'!I14+'P&amp;L'!I15</f>
         <v/>
       </c>
       <c r="J38" s="29">
-        <f>'P&amp;L'!J12+'P&amp;L'!J13+'P&amp;L'!J14+'P&amp;L'!J15</f>
+        <f>'P&amp;L'!J12*$D$63+'P&amp;L'!J13+'P&amp;L'!J14+'P&amp;L'!J15</f>
         <v/>
       </c>
       <c r="K38" s="29">
-        <f>'P&amp;L'!K12+'P&amp;L'!K13+'P&amp;L'!K14+'P&amp;L'!K15</f>
+        <f>'P&amp;L'!K12*$D$63+'P&amp;L'!K13+'P&amp;L'!K14+'P&amp;L'!K15</f>
         <v/>
       </c>
     </row>
@@ -2425,43 +2437,43 @@
         </is>
       </c>
       <c r="B39" s="25">
-        <f>(B36+B37+B38)*(1+IF(2027&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(B36+B37+B38)*(1+IF(2027&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="C39" s="25">
-        <f>(C36+C37+C38)*(1+IF(2028&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(C36+C37+C38)*(1+IF(2028&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="D39" s="25">
-        <f>(D36+D37+D38)*(1+IF(2029&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(D36+D37+D38)*(1+IF(2029&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="E39" s="25">
-        <f>(E36+E37+E38)*(1+IF(2030&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(E36+E37+E38)*(1+IF(2030&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="F39" s="25">
-        <f>(F36+F37+F38)*(1+IF(2031&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(F36+F37+F38)*(1+IF(2031&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="G39" s="25">
-        <f>(G36+G37+G38)*(1+IF(2032&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(G36+G37+G38)*(1+IF(2032&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="H39" s="25">
-        <f>(H36+H37+H38)*(1+IF(2033&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(H36+H37+H38)*(1+IF(2033&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="I39" s="25">
-        <f>(I36+I37+I38)*(1+IF(2034&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(I36+I37+I38)*(1+IF(2034&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="J39" s="25">
-        <f>(J36+J37+J38)*(1+IF(2035&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(J36+J37+J38)*(1+IF(2035&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="K39" s="25">
-        <f>(K36+K37+K38)*(1+IF(2036&gt;=Revenue!$B$13,Revenue!$B$11,0))</f>
+        <f>(K36+K37+K38)*(1+IF(2036&gt;=$D$66,Revenue!$B$11,0))</f>
         <v/>
       </c>
     </row>
@@ -2472,43 +2484,43 @@
         </is>
       </c>
       <c r="B40" s="29">
-        <f>'P&amp;L'!B24*$D$62</f>
+        <f>'P&amp;L'!B20+'P&amp;L'!B21+'P&amp;L'!B22*$D$67</f>
         <v/>
       </c>
       <c r="C40" s="29">
-        <f>'P&amp;L'!C24*$D$62</f>
+        <f>'P&amp;L'!C20+'P&amp;L'!C21+'P&amp;L'!C22*$D$67</f>
         <v/>
       </c>
       <c r="D40" s="29">
-        <f>'P&amp;L'!D24*$D$62</f>
+        <f>'P&amp;L'!D20+'P&amp;L'!D21+'P&amp;L'!D22*$D$67</f>
         <v/>
       </c>
       <c r="E40" s="29">
-        <f>'P&amp;L'!E24*$D$62</f>
+        <f>'P&amp;L'!E20+'P&amp;L'!E21+'P&amp;L'!E22*$D$67</f>
         <v/>
       </c>
       <c r="F40" s="29">
-        <f>'P&amp;L'!F24*$D$62</f>
+        <f>'P&amp;L'!F20+'P&amp;L'!F21+'P&amp;L'!F22*$D$67</f>
         <v/>
       </c>
       <c r="G40" s="29">
-        <f>'P&amp;L'!G24*$D$62</f>
+        <f>'P&amp;L'!G20+'P&amp;L'!G21+'P&amp;L'!G22*$D$67</f>
         <v/>
       </c>
       <c r="H40" s="29">
-        <f>'P&amp;L'!H24*$D$62</f>
+        <f>'P&amp;L'!H20+'P&amp;L'!H21+'P&amp;L'!H22*$D$67</f>
         <v/>
       </c>
       <c r="I40" s="29">
-        <f>'P&amp;L'!I24*$D$62</f>
+        <f>'P&amp;L'!I20+'P&amp;L'!I21+'P&amp;L'!I22*$D$67</f>
         <v/>
       </c>
       <c r="J40" s="29">
-        <f>'P&amp;L'!J24*$D$62</f>
+        <f>'P&amp;L'!J20+'P&amp;L'!J21+'P&amp;L'!J22*$D$67</f>
         <v/>
       </c>
       <c r="K40" s="29">
-        <f>'P&amp;L'!K24*$D$62</f>
+        <f>'P&amp;L'!K20+'P&amp;L'!K21+'P&amp;L'!K22*$D$67</f>
         <v/>
       </c>
     </row>
@@ -2711,147 +2723,342 @@
     <row r="53"/>
     <row r="54"/>
     <row r="55" ht="15" customHeight="1" s="20">
-      <c r="A55" s="22" t="inlineStr">
+      <c r="A55" s="32" t="inlineStr">
         <is>
           <t>SCENARIO ADJUSTMENTS (change values below to adjust scenarios)</t>
         </is>
       </c>
-      <c r="B55" s="22" t="n"/>
-      <c r="C55" s="22" t="n"/>
-      <c r="D55" s="22" t="n"/>
-      <c r="E55" s="22" t="n"/>
-      <c r="F55" s="22" t="n"/>
-      <c r="G55" s="22" t="n"/>
-      <c r="H55" s="22" t="n"/>
-      <c r="I55" s="22" t="n"/>
-      <c r="J55" s="22" t="n"/>
-      <c r="K55" s="22" t="n"/>
+      <c r="B55" s="33" t="n"/>
+      <c r="C55" s="33" t="n"/>
+      <c r="D55" s="33" t="n"/>
+      <c r="E55" s="33" t="n"/>
+      <c r="F55" s="33" t="n"/>
+      <c r="G55" s="33" t="n"/>
+      <c r="H55" s="33" t="n"/>
+      <c r="I55" s="33" t="n"/>
+      <c r="J55" s="33" t="n"/>
+      <c r="K55" s="33" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="20">
-      <c r="B56" s="32" t="inlineStr">
+      <c r="A56" s="34" t="n"/>
+      <c r="B56" s="35" t="inlineStr">
         <is>
           <t>Downside</t>
         </is>
       </c>
-      <c r="C56" s="32" t="inlineStr">
+      <c r="C56" s="35" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="D56" s="32" t="inlineStr">
+      <c r="D56" s="35" t="inlineStr">
         <is>
           <t>Upside</t>
         </is>
       </c>
-    </row>
-    <row r="57"/>
+      <c r="E56" s="34" t="n"/>
+      <c r="F56" s="34" t="n"/>
+      <c r="G56" s="34" t="n"/>
+      <c r="H56" s="34" t="n"/>
+      <c r="I56" s="34" t="n"/>
+      <c r="J56" s="34" t="n"/>
+      <c r="K56" s="34" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="34" t="n"/>
+      <c r="B57" s="34" t="n"/>
+      <c r="C57" s="34" t="n"/>
+      <c r="D57" s="34" t="n"/>
+      <c r="E57" s="34" t="n"/>
+      <c r="F57" s="34" t="n"/>
+      <c r="G57" s="34" t="n"/>
+      <c r="H57" s="34" t="n"/>
+      <c r="I57" s="34" t="n"/>
+      <c r="J57" s="34" t="n"/>
+      <c r="K57" s="34" t="n"/>
+    </row>
     <row r="58" ht="15" customHeight="1" s="20">
-      <c r="A58" s="26" t="inlineStr">
-        <is>
-          <t>■ FIRST EDITION FACTORS</t>
-        </is>
-      </c>
+      <c r="A58" s="36" t="inlineStr">
+        <is>
+          <t>■ REVENUE FACTORS</t>
+        </is>
+      </c>
+      <c r="B58" s="34" t="n"/>
+      <c r="C58" s="34" t="n"/>
+      <c r="D58" s="34" t="n"/>
+      <c r="E58" s="34" t="n"/>
+      <c r="F58" s="34" t="n"/>
+      <c r="G58" s="34" t="n"/>
+      <c r="H58" s="34" t="n"/>
+      <c r="I58" s="34" t="n"/>
+      <c r="J58" s="34" t="n"/>
+      <c r="K58" s="34" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="20">
-      <c r="A59" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  These multiply each year's revenue/cost directly.</t>
-        </is>
-      </c>
+      <c r="A59" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  These multiply each year's revenue line directly.</t>
+        </is>
+      </c>
+      <c r="B59" s="34" t="n"/>
+      <c r="C59" s="34" t="n"/>
+      <c r="D59" s="34" t="n"/>
+      <c r="E59" s="34" t="n"/>
+      <c r="F59" s="34" t="n"/>
+      <c r="G59" s="34" t="n"/>
+      <c r="H59" s="34" t="n"/>
+      <c r="I59" s="34" t="n"/>
+      <c r="J59" s="34" t="n"/>
+      <c r="K59" s="34" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" s="20">
-      <c r="A60" s="24" t="inlineStr">
+      <c r="A60" s="38" t="inlineStr">
         <is>
           <t>Ticket Occupancy</t>
         </is>
       </c>
-      <c r="B60" s="34" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="C60" s="34" t="n">
+      <c r="B60" s="39" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C60" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="D60" s="34" t="n">
+      <c r="D60" s="39" t="n">
         <v>1</v>
       </c>
+      <c r="E60" s="34" t="n"/>
+      <c r="F60" s="34" t="n"/>
+      <c r="G60" s="34" t="n"/>
+      <c r="H60" s="34" t="n"/>
+      <c r="I60" s="34" t="n"/>
+      <c r="J60" s="34" t="n"/>
+      <c r="K60" s="34" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="20">
-      <c r="A61" s="24" t="inlineStr">
+      <c r="A61" s="38" t="inlineStr">
+        <is>
+          <t>Ticket Price Factor</t>
+        </is>
+      </c>
+      <c r="B61" s="40" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C61" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="40" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E61" s="34" t="n"/>
+      <c r="F61" s="34" t="n"/>
+      <c r="G61" s="34" t="n"/>
+      <c r="H61" s="34" t="n"/>
+      <c r="I61" s="34" t="n"/>
+      <c r="J61" s="34" t="n"/>
+      <c r="K61" s="34" t="n"/>
+    </row>
+    <row r="62" ht="15" customHeight="1" s="20">
+      <c r="A62" s="38" t="inlineStr">
         <is>
           <t>Partnership Factor</t>
         </is>
       </c>
-      <c r="B61" s="35" t="n">
+      <c r="B62" s="40" t="n">
         <v>0.6</v>
       </c>
-      <c r="C61" s="35" t="n">
+      <c r="C62" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="D61" s="35" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="62" ht="15" customHeight="1" s="20">
-      <c r="A62" s="24" t="inlineStr">
-        <is>
-          <t>Cost Overrun Factor</t>
-        </is>
-      </c>
-      <c r="B62" s="35" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="C62" s="35" t="n">
+      <c r="D62" s="40" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E62" s="34" t="n"/>
+      <c r="F62" s="34" t="n"/>
+      <c r="G62" s="34" t="n"/>
+      <c r="H62" s="34" t="n"/>
+      <c r="I62" s="34" t="n"/>
+      <c r="J62" s="34" t="n"/>
+      <c r="K62" s="34" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="41" t="inlineStr">
+        <is>
+          <t>ASA Factor</t>
+        </is>
+      </c>
+      <c r="B63" s="42" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C63" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="D62" s="35" t="n">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="63"/>
+      <c r="D63" s="42" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E63" s="34" t="n"/>
+      <c r="F63" s="34" t="n"/>
+      <c r="G63" s="34" t="n"/>
+      <c r="H63" s="34" t="n"/>
+      <c r="I63" s="34" t="n"/>
+      <c r="J63" s="34" t="n"/>
+      <c r="K63" s="34" t="n"/>
+    </row>
     <row r="64" ht="15" customHeight="1" s="20">
-      <c r="A64" s="33" t="inlineStr">
-        <is>
-          <t>SCENARIO EXPLANATIONS:</t>
-        </is>
-      </c>
+      <c r="A64" s="33" t="n"/>
+      <c r="B64" s="34" t="n"/>
+      <c r="C64" s="34" t="n"/>
+      <c r="D64" s="34" t="n"/>
+      <c r="E64" s="34" t="n"/>
+      <c r="F64" s="34" t="n"/>
+      <c r="G64" s="34" t="n"/>
+      <c r="H64" s="34" t="n"/>
+      <c r="I64" s="34" t="n"/>
+      <c r="J64" s="34" t="n"/>
+      <c r="K64" s="34" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="20">
-      <c r="A65" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ticket Occupancy: % of tickets sold (e.g., 80% = 200 of 250 tickets). Upside cannot exceed 100% due to venue cap.</t>
-        </is>
-      </c>
+      <c r="A65" s="36" t="inlineStr">
+        <is>
+          <t>■ STRUCTURAL FACTORS</t>
+        </is>
+      </c>
+      <c r="B65" s="34" t="n"/>
+      <c r="C65" s="34" t="n"/>
+      <c r="D65" s="34" t="n"/>
+      <c r="E65" s="34" t="n"/>
+      <c r="F65" s="34" t="n"/>
+      <c r="G65" s="34" t="n"/>
+      <c r="H65" s="34" t="n"/>
+      <c r="I65" s="34" t="n"/>
+      <c r="J65" s="34" t="n"/>
+      <c r="K65" s="34" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="20">
-      <c r="A66" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Partnership Factor: Multiplier on total partnership revenue (e.g., ×0.6 = sponsors 40% fewer).</t>
-        </is>
-      </c>
+      <c r="A66" s="38" t="inlineStr">
+        <is>
+          <t>Summer Start Year</t>
+        </is>
+      </c>
+      <c r="B66" s="42" t="n">
+        <v>2029</v>
+      </c>
+      <c r="C66" s="42" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D66" s="42" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E66" s="34" t="n"/>
+      <c r="F66" s="34" t="n"/>
+      <c r="G66" s="34" t="n"/>
+      <c r="H66" s="34" t="n"/>
+      <c r="I66" s="34" t="n"/>
+      <c r="J66" s="34" t="n"/>
+      <c r="K66" s="34" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="20">
-      <c r="A67" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cost Overrun Factor: Multiplier on total direct costs (e.g., ×1.15 = costs 15% over budget).</t>
-        </is>
-      </c>
+      <c r="A67" s="38" t="inlineStr">
+        <is>
+          <t>Founder Pay Factor</t>
+        </is>
+      </c>
+      <c r="B67" s="42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C67" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="34" t="n"/>
+      <c r="F67" s="34" t="n"/>
+      <c r="G67" s="34" t="n"/>
+      <c r="H67" s="34" t="n"/>
+      <c r="I67" s="34" t="n"/>
+      <c r="J67" s="34" t="n"/>
+      <c r="K67" s="34" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="20">
       <c r="A68" s="33" t="n"/>
+      <c r="B68" s="34" t="n"/>
+      <c r="C68" s="34" t="n"/>
+      <c r="D68" s="34" t="n"/>
+      <c r="E68" s="34" t="n"/>
+      <c r="F68" s="34" t="n"/>
+      <c r="G68" s="34" t="n"/>
+      <c r="H68" s="34" t="n"/>
+      <c r="I68" s="34" t="n"/>
+      <c r="J68" s="34" t="n"/>
+      <c r="K68" s="34" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="20">
-      <c r="A69" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Downside = worst case (all factors negative simultaneously). Base = as entered in Revenue/Cost sheets. Upside = best case.</t>
-        </is>
-      </c>
+      <c r="A69" s="43" t="inlineStr">
+        <is>
+          <t>SCENARIO DEFINITIONS:</t>
+        </is>
+      </c>
+      <c r="B69" s="34" t="n"/>
+      <c r="C69" s="34" t="n"/>
+      <c r="D69" s="34" t="n"/>
+      <c r="E69" s="34" t="n"/>
+      <c r="F69" s="34" t="n"/>
+      <c r="G69" s="34" t="n"/>
+      <c r="H69" s="34" t="n"/>
+      <c r="I69" s="34" t="n"/>
+      <c r="J69" s="34" t="n"/>
+      <c r="K69" s="34" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="20">
-      <c r="A70" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  To test individual growth rates or prices, change the yellow cells in Revenue/Cost sheets directly.</t>
-        </is>
-      </c>
+      <c r="A70" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Downside: Tickets 15% below plan, prices 10% lower, partnerships 40% lower, ASA 25% lower, summer from 2029, founder pay halved.</t>
+        </is>
+      </c>
+      <c r="B70" s="34" t="n"/>
+      <c r="C70" s="34" t="n"/>
+      <c r="D70" s="34" t="n"/>
+      <c r="E70" s="34" t="n"/>
+      <c r="F70" s="34" t="n"/>
+      <c r="G70" s="34" t="n"/>
+      <c r="H70" s="34" t="n"/>
+      <c r="I70" s="34" t="n"/>
+      <c r="J70" s="34" t="n"/>
+      <c r="K70" s="34" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Base: All factors at 1.0 — as entered in Revenue/Cost sheets. Summer from 2027.</t>
+        </is>
+      </c>
+      <c r="B71" s="34" t="n"/>
+      <c r="C71" s="34" t="n"/>
+      <c r="D71" s="34" t="n"/>
+      <c r="E71" s="34" t="n"/>
+      <c r="F71" s="34" t="n"/>
+      <c r="G71" s="34" t="n"/>
+      <c r="H71" s="34" t="n"/>
+      <c r="I71" s="34" t="n"/>
+      <c r="J71" s="34" t="n"/>
+      <c r="K71" s="34" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upside: Prices 10% higher, partnerships 40% higher, ASA +25%. Summer from 2027.</t>
+        </is>
+      </c>
+      <c r="B72" s="34" t="n"/>
+      <c r="C72" s="34" t="n"/>
+      <c r="D72" s="34" t="n"/>
+      <c r="E72" s="34" t="n"/>
+      <c r="F72" s="34" t="n"/>
+      <c r="G72" s="34" t="n"/>
+      <c r="H72" s="34" t="n"/>
+      <c r="I72" s="34" t="n"/>
+      <c r="J72" s="34" t="n"/>
+      <c r="K72" s="34" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CC0B"/>
@@ -2884,7 +3091,7 @@
     </row>
     <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="20">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>MODEL ASSUMPTIONS</t>
         </is>
@@ -2906,7 +3113,7 @@
           <t>Total Guest Count</t>
         </is>
       </c>
-      <c r="B4" s="37" t="n">
+      <c r="B4" s="45" t="n">
         <v>280</v>
       </c>
     </row>
@@ -2916,7 +3123,7 @@
           <t>Total Ticket Count</t>
         </is>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="45" t="n">
         <v>250</v>
       </c>
     </row>
@@ -2926,7 +3133,7 @@
           <t>Net Factor (VAT + platform fees)</t>
         </is>
       </c>
-      <c r="B6" s="35" t="n">
+      <c r="B6" s="46" t="n">
         <v>0.89</v>
       </c>
     </row>
@@ -2936,7 +3143,7 @@
           <t>Ticket Price Growth Rate (to 2030)</t>
         </is>
       </c>
-      <c r="B7" s="34" t="n">
+      <c r="B7" s="47" t="n">
         <v>0.08</v>
       </c>
     </row>
@@ -2946,7 +3153,7 @@
           <t>Ticket Price Growth Rate (2031+)</t>
         </is>
       </c>
-      <c r="B8" s="34" t="n">
+      <c r="B8" s="47" t="n">
         <v>0.04</v>
       </c>
     </row>
@@ -2956,7 +3163,7 @@
           <t>F&amp;B Growth Rate</t>
         </is>
       </c>
-      <c r="B9" s="34" t="n">
+      <c r="B9" s="47" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -2966,7 +3173,7 @@
           <t>Partnership Growth Rate (2032+)</t>
         </is>
       </c>
-      <c r="B10" s="34" t="n">
+      <c r="B10" s="47" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -2976,7 +3183,7 @@
           <t>Summer Revenue Multiplier</t>
         </is>
       </c>
-      <c r="B11" s="35" t="n">
+      <c r="B11" s="46" t="n">
         <v>0.55</v>
       </c>
     </row>
@@ -2986,7 +3193,7 @@
           <t>Summer Cost Multiplier</t>
         </is>
       </c>
-      <c r="B12" s="35" t="n">
+      <c r="B12" s="46" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -2996,7 +3203,7 @@
           <t>Summer Start Year</t>
         </is>
       </c>
-      <c r="B13" s="38" t="n">
+      <c r="B13" s="48" t="n">
         <v>2027</v>
       </c>
     </row>
@@ -3031,7 +3238,7 @@
           <t xml:space="preserve">  Drop 1 Allocation %</t>
         </is>
       </c>
-      <c r="B17" s="34" t="n">
+      <c r="B17" s="47" t="n">
         <v>0.28</v>
       </c>
     </row>
@@ -3041,7 +3248,7 @@
           <t xml:space="preserve">  Drop 2 Allocation %</t>
         </is>
       </c>
-      <c r="B18" s="34" t="n">
+      <c r="B18" s="47" t="n">
         <v>0.44</v>
       </c>
     </row>
@@ -3051,7 +3258,7 @@
           <t xml:space="preserve">  Drop 3 Allocation %</t>
         </is>
       </c>
-      <c r="B19" s="34" t="n">
+      <c r="B19" s="47" t="n">
         <v>0.28</v>
       </c>
     </row>
@@ -3069,7 +3276,7 @@
           <t xml:space="preserve">  Drop 1 Unit Price</t>
         </is>
       </c>
-      <c r="B22" s="37" t="n">
+      <c r="B22" s="45" t="n">
         <v>210</v>
       </c>
     </row>
@@ -3079,7 +3286,7 @@
           <t xml:space="preserve">  Drop 2 Unit Price</t>
         </is>
       </c>
-      <c r="B23" s="37" t="n">
+      <c r="B23" s="45" t="n">
         <v>250</v>
       </c>
     </row>
@@ -3089,7 +3296,7 @@
           <t xml:space="preserve">  Drop 3 Unit Price</t>
         </is>
       </c>
-      <c r="B24" s="37" t="n">
+      <c r="B24" s="45" t="n">
         <v>290</v>
       </c>
     </row>
@@ -3710,19 +3917,19 @@
           <t xml:space="preserve">  Presenting Partner — Price</t>
         </is>
       </c>
-      <c r="B44" s="37" t="n">
+      <c r="B44" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="C44" s="37" t="n">
+      <c r="C44" s="45" t="n">
         <v>50000</v>
       </c>
-      <c r="D44" s="37" t="n">
+      <c r="D44" s="45" t="n">
         <v>50000</v>
       </c>
-      <c r="E44" s="37" t="n">
+      <c r="E44" s="45" t="n">
         <v>50000</v>
       </c>
-      <c r="F44" s="37" t="n">
+      <c r="F44" s="45" t="n">
         <v>50000</v>
       </c>
     </row>
@@ -3732,19 +3939,19 @@
           <t xml:space="preserve">  Presenting Partner — Count</t>
         </is>
       </c>
-      <c r="B45" s="37" t="n">
+      <c r="B45" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="C45" s="37" t="n">
+      <c r="C45" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="37" t="n">
+      <c r="D45" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="E45" s="37" t="n">
+      <c r="E45" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="F45" s="37" t="n">
+      <c r="F45" s="45" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3782,19 +3989,19 @@
           <t xml:space="preserve">  Partner — Price</t>
         </is>
       </c>
-      <c r="B48" s="37" t="n">
+      <c r="B48" s="45" t="n">
         <v>15000</v>
       </c>
-      <c r="C48" s="37" t="n">
+      <c r="C48" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D48" s="37" t="n">
+      <c r="D48" s="45" t="n">
         <v>15000</v>
       </c>
-      <c r="E48" s="37" t="n">
+      <c r="E48" s="45" t="n">
         <v>15000</v>
       </c>
-      <c r="F48" s="37" t="n">
+      <c r="F48" s="45" t="n">
         <v>15000</v>
       </c>
     </row>
@@ -3804,19 +4011,19 @@
           <t xml:space="preserve">  Partner — Count</t>
         </is>
       </c>
-      <c r="B49" s="37" t="n">
+      <c r="B49" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="C49" s="37" t="n">
+      <c r="C49" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="D49" s="37" t="n">
+      <c r="D49" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="E49" s="37" t="n">
+      <c r="E49" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="F49" s="37" t="n">
+      <c r="F49" s="45" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3854,19 +4061,19 @@
           <t xml:space="preserve">  Supporting Partner — Price</t>
         </is>
       </c>
-      <c r="B52" s="37" t="n">
+      <c r="B52" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="C52" s="37" t="n">
+      <c r="C52" s="45" t="n">
         <v>5000</v>
       </c>
-      <c r="D52" s="37" t="n">
+      <c r="D52" s="45" t="n">
         <v>5000</v>
       </c>
-      <c r="E52" s="37" t="n">
+      <c r="E52" s="45" t="n">
         <v>5000</v>
       </c>
-      <c r="F52" s="37" t="n">
+      <c r="F52" s="45" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -3876,19 +4083,19 @@
           <t xml:space="preserve">  Supporting Partner — Count</t>
         </is>
       </c>
-      <c r="B53" s="37" t="n">
+      <c r="B53" s="45" t="n">
         <v>0</v>
       </c>
-      <c r="C53" s="37" t="n">
+      <c r="C53" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="D53" s="37" t="n">
+      <c r="D53" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="E53" s="37" t="n">
+      <c r="E53" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="F53" s="37" t="n">
+      <c r="F53" s="45" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3968,7 +4175,7 @@
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="20">
-      <c r="A57" s="33" t="inlineStr">
+      <c r="A57" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  2027-2031: Tier breakdown (editable). 2032-2036: Auto-calculated from 2031 total at Partnership Growth Rate.</t>
         </is>
@@ -4031,39 +4238,39 @@
           <t>ASA Contribution (manual input)</t>
         </is>
       </c>
-      <c r="B61" s="37" t="n">
+      <c r="B61" s="45" t="n">
         <v>10000</v>
       </c>
-      <c r="C61" s="37" t="n">
+      <c r="C61" s="45" t="n">
         <v>12500</v>
       </c>
-      <c r="D61" s="37" t="n">
+      <c r="D61" s="45" t="n">
         <v>15000</v>
       </c>
-      <c r="E61" s="37" t="n">
+      <c r="E61" s="45" t="n">
         <v>20000</v>
       </c>
-      <c r="F61" s="37" t="n">
+      <c r="F61" s="45" t="n">
         <v>25000</v>
       </c>
-      <c r="G61" s="37" t="n">
+      <c r="G61" s="45" t="n">
         <v>30000</v>
       </c>
-      <c r="H61" s="37" t="n">
+      <c r="H61" s="45" t="n">
         <v>30000</v>
       </c>
-      <c r="I61" s="37" t="n">
+      <c r="I61" s="45" t="n">
         <v>35000</v>
       </c>
-      <c r="J61" s="37" t="n">
+      <c r="J61" s="45" t="n">
         <v>40000</v>
       </c>
-      <c r="K61" s="37" t="n">
+      <c r="K61" s="45" t="n">
         <v>45000</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="20">
-      <c r="A62" s="33" t="inlineStr">
+      <c r="A62" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  ASA partnership contribution follows a 3-phase negotiation schedule (Build / Grow / Anchor). Values are irregular and entered manually per year.</t>
         </is>
@@ -4071,1054 +4278,1054 @@
     </row>
     <row r="63"/>
     <row r="64" ht="15" customHeight="1" s="20">
-      <c r="A64" s="39" t="inlineStr">
+      <c r="A64" s="50" t="inlineStr">
         <is>
           <t>SECTION 4: BAR / F&amp;B REVENUE</t>
         </is>
       </c>
-      <c r="B64" s="40" t="n"/>
-      <c r="C64" s="40" t="n"/>
-      <c r="D64" s="40" t="n"/>
-      <c r="E64" s="40" t="n"/>
-      <c r="F64" s="40" t="n"/>
-      <c r="G64" s="40" t="n"/>
-      <c r="H64" s="40" t="n"/>
-      <c r="I64" s="40" t="n"/>
-      <c r="J64" s="40" t="n"/>
-      <c r="K64" s="40" t="n"/>
+      <c r="B64" s="33" t="n"/>
+      <c r="C64" s="33" t="n"/>
+      <c r="D64" s="33" t="n"/>
+      <c r="E64" s="33" t="n"/>
+      <c r="F64" s="33" t="n"/>
+      <c r="G64" s="33" t="n"/>
+      <c r="H64" s="33" t="n"/>
+      <c r="I64" s="33" t="n"/>
+      <c r="J64" s="33" t="n"/>
+      <c r="K64" s="33" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="20">
-      <c r="A65" s="41" t="inlineStr">
+      <c r="A65" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  Share rates are currently set to 0%. Aura does not take a share of bar/food revenue. If a share agreement is negotiated, change the share rate.</t>
         </is>
       </c>
-      <c r="B65" s="42" t="n"/>
-      <c r="C65" s="42" t="n"/>
-      <c r="D65" s="42" t="n"/>
-      <c r="E65" s="42" t="n"/>
-      <c r="F65" s="42" t="n"/>
-      <c r="G65" s="42" t="n"/>
-      <c r="H65" s="42" t="n"/>
-      <c r="I65" s="42" t="n"/>
-      <c r="J65" s="42" t="n"/>
-      <c r="K65" s="42" t="n"/>
+      <c r="B65" s="34" t="n"/>
+      <c r="C65" s="34" t="n"/>
+      <c r="D65" s="34" t="n"/>
+      <c r="E65" s="34" t="n"/>
+      <c r="F65" s="34" t="n"/>
+      <c r="G65" s="34" t="n"/>
+      <c r="H65" s="34" t="n"/>
+      <c r="I65" s="34" t="n"/>
+      <c r="J65" s="34" t="n"/>
+      <c r="K65" s="34" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="42" t="n"/>
-      <c r="B66" s="42" t="n"/>
-      <c r="C66" s="42" t="n"/>
-      <c r="D66" s="42" t="n"/>
-      <c r="E66" s="42" t="n"/>
-      <c r="F66" s="42" t="n"/>
-      <c r="G66" s="42" t="n"/>
-      <c r="H66" s="42" t="n"/>
-      <c r="I66" s="42" t="n"/>
-      <c r="J66" s="42" t="n"/>
-      <c r="K66" s="42" t="n"/>
+      <c r="A66" s="34" t="n"/>
+      <c r="B66" s="34" t="n"/>
+      <c r="C66" s="34" t="n"/>
+      <c r="D66" s="34" t="n"/>
+      <c r="E66" s="34" t="n"/>
+      <c r="F66" s="34" t="n"/>
+      <c r="G66" s="34" t="n"/>
+      <c r="H66" s="34" t="n"/>
+      <c r="I66" s="34" t="n"/>
+      <c r="J66" s="34" t="n"/>
+      <c r="K66" s="34" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="20">
-      <c r="A67" s="40" t="n"/>
-      <c r="B67" s="43" t="n">
+      <c r="A67" s="33" t="n"/>
+      <c r="B67" s="51" t="n">
         <v>2027</v>
       </c>
-      <c r="C67" s="43" t="n">
+      <c r="C67" s="51" t="n">
         <v>2028</v>
       </c>
-      <c r="D67" s="43" t="n">
+      <c r="D67" s="51" t="n">
         <v>2029</v>
       </c>
-      <c r="E67" s="43" t="n">
+      <c r="E67" s="51" t="n">
         <v>2030</v>
       </c>
-      <c r="F67" s="43" t="n">
+      <c r="F67" s="51" t="n">
         <v>2031</v>
       </c>
-      <c r="G67" s="43" t="n">
+      <c r="G67" s="51" t="n">
         <v>2032</v>
       </c>
-      <c r="H67" s="43" t="n">
+      <c r="H67" s="51" t="n">
         <v>2033</v>
       </c>
-      <c r="I67" s="43" t="n">
+      <c r="I67" s="51" t="n">
         <v>2034</v>
       </c>
-      <c r="J67" s="43" t="n">
+      <c r="J67" s="51" t="n">
         <v>2035</v>
       </c>
-      <c r="K67" s="43" t="n">
+      <c r="K67" s="51" t="n">
         <v>2036</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="20">
-      <c r="A68" s="44" t="inlineStr">
+      <c r="A68" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Friday Night: Coffee + Drinks — Guest Count</t>
         </is>
       </c>
-      <c r="B68" s="45" t="n">
+      <c r="B68" s="52" t="n">
         <v>150</v>
       </c>
-      <c r="C68" s="42" t="n"/>
-      <c r="D68" s="42" t="n"/>
-      <c r="E68" s="42" t="n"/>
-      <c r="F68" s="42" t="n"/>
-      <c r="G68" s="42" t="n"/>
-      <c r="H68" s="42" t="n"/>
-      <c r="I68" s="42" t="n"/>
-      <c r="J68" s="42" t="n"/>
-      <c r="K68" s="42" t="n"/>
+      <c r="C68" s="34" t="n"/>
+      <c r="D68" s="34" t="n"/>
+      <c r="E68" s="34" t="n"/>
+      <c r="F68" s="34" t="n"/>
+      <c r="G68" s="34" t="n"/>
+      <c r="H68" s="34" t="n"/>
+      <c r="I68" s="34" t="n"/>
+      <c r="J68" s="34" t="n"/>
+      <c r="K68" s="34" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="20">
-      <c r="A69" s="44" t="inlineStr">
+      <c r="A69" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Friday Night: Coffee + Drinks — Per-person Spend</t>
         </is>
       </c>
-      <c r="B69" s="45" t="n">
+      <c r="B69" s="52" t="n">
         <v>50</v>
       </c>
-      <c r="C69" s="42" t="n"/>
-      <c r="D69" s="42" t="n"/>
-      <c r="E69" s="42" t="n"/>
-      <c r="F69" s="42" t="n"/>
-      <c r="G69" s="42" t="n"/>
-      <c r="H69" s="42" t="n"/>
-      <c r="I69" s="42" t="n"/>
-      <c r="J69" s="42" t="n"/>
-      <c r="K69" s="42" t="n"/>
+      <c r="C69" s="34" t="n"/>
+      <c r="D69" s="34" t="n"/>
+      <c r="E69" s="34" t="n"/>
+      <c r="F69" s="34" t="n"/>
+      <c r="G69" s="34" t="n"/>
+      <c r="H69" s="34" t="n"/>
+      <c r="I69" s="34" t="n"/>
+      <c r="J69" s="34" t="n"/>
+      <c r="K69" s="34" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="20">
-      <c r="A70" s="44" t="inlineStr">
+      <c r="A70" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Friday Night: Coffee + Drinks — Share Rate</t>
         </is>
       </c>
-      <c r="B70" s="46" t="n">
+      <c r="B70" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C70" s="42" t="n"/>
-      <c r="D70" s="42" t="n"/>
-      <c r="E70" s="42" t="n"/>
-      <c r="F70" s="42" t="n"/>
-      <c r="G70" s="42" t="n"/>
-      <c r="H70" s="42" t="n"/>
-      <c r="I70" s="42" t="n"/>
-      <c r="J70" s="42" t="n"/>
-      <c r="K70" s="42" t="n"/>
+      <c r="C70" s="34" t="n"/>
+      <c r="D70" s="34" t="n"/>
+      <c r="E70" s="34" t="n"/>
+      <c r="F70" s="34" t="n"/>
+      <c r="G70" s="34" t="n"/>
+      <c r="H70" s="34" t="n"/>
+      <c r="I70" s="34" t="n"/>
+      <c r="J70" s="34" t="n"/>
+      <c r="K70" s="34" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" s="20">
-      <c r="A71" s="44" t="inlineStr">
+      <c r="A71" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Friday Night: Coffee + Drinks — Est. Total Sales (reference)</t>
         </is>
       </c>
-      <c r="B71" s="47">
+      <c r="B71" s="53">
         <f>B68*B69</f>
         <v/>
       </c>
-      <c r="C71" s="47">
+      <c r="C71" s="53">
         <f>B71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="D71" s="47">
+      <c r="D71" s="53">
         <f>C71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="E71" s="47">
+      <c r="E71" s="53">
         <f>D71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="F71" s="47">
+      <c r="F71" s="53">
         <f>E71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="G71" s="47">
+      <c r="G71" s="53">
         <f>F71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="H71" s="47">
+      <c r="H71" s="53">
         <f>G71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="I71" s="47">
+      <c r="I71" s="53">
         <f>H71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="J71" s="47">
+      <c r="J71" s="53">
         <f>I71*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="K71" s="47">
+      <c r="K71" s="53">
         <f>J71*(1+$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="20">
-      <c r="A72" s="44" t="inlineStr">
+      <c r="A72" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Friday Night: Coffee + Drinks — Aura Revenue</t>
         </is>
       </c>
-      <c r="B72" s="47">
+      <c r="B72" s="53">
         <f>B71*$B70</f>
         <v/>
       </c>
-      <c r="C72" s="47">
+      <c r="C72" s="53">
         <f>C71*$B70</f>
         <v/>
       </c>
-      <c r="D72" s="47">
+      <c r="D72" s="53">
         <f>D71*$B70</f>
         <v/>
       </c>
-      <c r="E72" s="47">
+      <c r="E72" s="53">
         <f>E71*$B70</f>
         <v/>
       </c>
-      <c r="F72" s="47">
+      <c r="F72" s="53">
         <f>F71*$B70</f>
         <v/>
       </c>
-      <c r="G72" s="47">
+      <c r="G72" s="53">
         <f>G71*$B70</f>
         <v/>
       </c>
-      <c r="H72" s="47">
+      <c r="H72" s="53">
         <f>H71*$B70</f>
         <v/>
       </c>
-      <c r="I72" s="47">
+      <c r="I72" s="53">
         <f>I71*$B70</f>
         <v/>
       </c>
-      <c r="J72" s="47">
+      <c r="J72" s="53">
         <f>J71*$B70</f>
         <v/>
       </c>
-      <c r="K72" s="47">
+      <c r="K72" s="53">
         <f>K71*$B70</f>
         <v/>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="42" t="n"/>
-      <c r="B73" s="42" t="n"/>
-      <c r="C73" s="42" t="n"/>
-      <c r="D73" s="42" t="n"/>
-      <c r="E73" s="42" t="n"/>
-      <c r="F73" s="42" t="n"/>
-      <c r="G73" s="42" t="n"/>
-      <c r="H73" s="42" t="n"/>
-      <c r="I73" s="42" t="n"/>
-      <c r="J73" s="42" t="n"/>
-      <c r="K73" s="42" t="n"/>
+      <c r="A73" s="34" t="n"/>
+      <c r="B73" s="34" t="n"/>
+      <c r="C73" s="34" t="n"/>
+      <c r="D73" s="34" t="n"/>
+      <c r="E73" s="34" t="n"/>
+      <c r="F73" s="34" t="n"/>
+      <c r="G73" s="34" t="n"/>
+      <c r="H73" s="34" t="n"/>
+      <c r="I73" s="34" t="n"/>
+      <c r="J73" s="34" t="n"/>
+      <c r="K73" s="34" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" s="20">
-      <c r="A74" s="44" t="inlineStr">
+      <c r="A74" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Drinks — Guest Count</t>
         </is>
       </c>
-      <c r="B74" s="45" t="n">
+      <c r="B74" s="52" t="n">
         <v>280</v>
       </c>
-      <c r="C74" s="42" t="n"/>
-      <c r="D74" s="42" t="n"/>
-      <c r="E74" s="42" t="n"/>
-      <c r="F74" s="42" t="n"/>
-      <c r="G74" s="42" t="n"/>
-      <c r="H74" s="42" t="n"/>
-      <c r="I74" s="42" t="n"/>
-      <c r="J74" s="42" t="n"/>
-      <c r="K74" s="42" t="n"/>
+      <c r="C74" s="34" t="n"/>
+      <c r="D74" s="34" t="n"/>
+      <c r="E74" s="34" t="n"/>
+      <c r="F74" s="34" t="n"/>
+      <c r="G74" s="34" t="n"/>
+      <c r="H74" s="34" t="n"/>
+      <c r="I74" s="34" t="n"/>
+      <c r="J74" s="34" t="n"/>
+      <c r="K74" s="34" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" s="20">
-      <c r="A75" s="44" t="inlineStr">
+      <c r="A75" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Drinks — Per-person Spend</t>
         </is>
       </c>
-      <c r="B75" s="45" t="n">
+      <c r="B75" s="52" t="n">
         <v>20</v>
       </c>
-      <c r="C75" s="42" t="n"/>
-      <c r="D75" s="42" t="n"/>
-      <c r="E75" s="42" t="n"/>
-      <c r="F75" s="42" t="n"/>
-      <c r="G75" s="42" t="n"/>
-      <c r="H75" s="42" t="n"/>
-      <c r="I75" s="42" t="n"/>
-      <c r="J75" s="42" t="n"/>
-      <c r="K75" s="42" t="n"/>
+      <c r="C75" s="34" t="n"/>
+      <c r="D75" s="34" t="n"/>
+      <c r="E75" s="34" t="n"/>
+      <c r="F75" s="34" t="n"/>
+      <c r="G75" s="34" t="n"/>
+      <c r="H75" s="34" t="n"/>
+      <c r="I75" s="34" t="n"/>
+      <c r="J75" s="34" t="n"/>
+      <c r="K75" s="34" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1" s="20">
-      <c r="A76" s="44" t="inlineStr">
+      <c r="A76" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Drinks — Share Rate</t>
         </is>
       </c>
-      <c r="B76" s="46" t="n">
+      <c r="B76" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C76" s="42" t="n"/>
-      <c r="D76" s="42" t="n"/>
-      <c r="E76" s="42" t="n"/>
-      <c r="F76" s="42" t="n"/>
-      <c r="G76" s="42" t="n"/>
-      <c r="H76" s="42" t="n"/>
-      <c r="I76" s="42" t="n"/>
-      <c r="J76" s="42" t="n"/>
-      <c r="K76" s="42" t="n"/>
+      <c r="C76" s="34" t="n"/>
+      <c r="D76" s="34" t="n"/>
+      <c r="E76" s="34" t="n"/>
+      <c r="F76" s="34" t="n"/>
+      <c r="G76" s="34" t="n"/>
+      <c r="H76" s="34" t="n"/>
+      <c r="I76" s="34" t="n"/>
+      <c r="J76" s="34" t="n"/>
+      <c r="K76" s="34" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" s="20">
-      <c r="A77" s="44" t="inlineStr">
+      <c r="A77" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Drinks — Est. Total Sales (reference)</t>
         </is>
       </c>
-      <c r="B77" s="47">
+      <c r="B77" s="53">
         <f>B74*B75</f>
         <v/>
       </c>
-      <c r="C77" s="47">
+      <c r="C77" s="53">
         <f>B77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="D77" s="47">
+      <c r="D77" s="53">
         <f>C77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="E77" s="47">
+      <c r="E77" s="53">
         <f>D77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="F77" s="47">
+      <c r="F77" s="53">
         <f>E77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="G77" s="47">
+      <c r="G77" s="53">
         <f>F77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="H77" s="47">
+      <c r="H77" s="53">
         <f>G77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="I77" s="47">
+      <c r="I77" s="53">
         <f>H77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="J77" s="47">
+      <c r="J77" s="53">
         <f>I77*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="K77" s="47">
+      <c r="K77" s="53">
         <f>J77*(1+$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="20">
-      <c r="A78" s="44" t="inlineStr">
+      <c r="A78" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Drinks — Aura Revenue</t>
         </is>
       </c>
-      <c r="B78" s="47">
+      <c r="B78" s="53">
         <f>B77*$B76</f>
         <v/>
       </c>
-      <c r="C78" s="47">
+      <c r="C78" s="53">
         <f>C77*$B76</f>
         <v/>
       </c>
-      <c r="D78" s="47">
+      <c r="D78" s="53">
         <f>D77*$B76</f>
         <v/>
       </c>
-      <c r="E78" s="47">
+      <c r="E78" s="53">
         <f>E77*$B76</f>
         <v/>
       </c>
-      <c r="F78" s="47">
+      <c r="F78" s="53">
         <f>F77*$B76</f>
         <v/>
       </c>
-      <c r="G78" s="47">
+      <c r="G78" s="53">
         <f>G77*$B76</f>
         <v/>
       </c>
-      <c r="H78" s="47">
+      <c r="H78" s="53">
         <f>H77*$B76</f>
         <v/>
       </c>
-      <c r="I78" s="47">
+      <c r="I78" s="53">
         <f>I77*$B76</f>
         <v/>
       </c>
-      <c r="J78" s="47">
+      <c r="J78" s="53">
         <f>J77*$B76</f>
         <v/>
       </c>
-      <c r="K78" s="47">
+      <c r="K78" s="53">
         <f>K77*$B76</f>
         <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="42" t="n"/>
-      <c r="B79" s="42" t="n"/>
-      <c r="C79" s="42" t="n"/>
-      <c r="D79" s="42" t="n"/>
-      <c r="E79" s="42" t="n"/>
-      <c r="F79" s="42" t="n"/>
-      <c r="G79" s="42" t="n"/>
-      <c r="H79" s="42" t="n"/>
-      <c r="I79" s="42" t="n"/>
-      <c r="J79" s="42" t="n"/>
-      <c r="K79" s="42" t="n"/>
+      <c r="A79" s="34" t="n"/>
+      <c r="B79" s="34" t="n"/>
+      <c r="C79" s="34" t="n"/>
+      <c r="D79" s="34" t="n"/>
+      <c r="E79" s="34" t="n"/>
+      <c r="F79" s="34" t="n"/>
+      <c r="G79" s="34" t="n"/>
+      <c r="H79" s="34" t="n"/>
+      <c r="I79" s="34" t="n"/>
+      <c r="J79" s="34" t="n"/>
+      <c r="K79" s="34" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1" s="20">
-      <c r="A80" s="44" t="inlineStr">
+      <c r="A80" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Food — Guest Count</t>
         </is>
       </c>
-      <c r="B80" s="45" t="n">
+      <c r="B80" s="52" t="n">
         <v>280</v>
       </c>
-      <c r="C80" s="42" t="n"/>
-      <c r="D80" s="42" t="n"/>
-      <c r="E80" s="42" t="n"/>
-      <c r="F80" s="42" t="n"/>
-      <c r="G80" s="42" t="n"/>
-      <c r="H80" s="42" t="n"/>
-      <c r="I80" s="42" t="n"/>
-      <c r="J80" s="42" t="n"/>
-      <c r="K80" s="42" t="n"/>
+      <c r="C80" s="34" t="n"/>
+      <c r="D80" s="34" t="n"/>
+      <c r="E80" s="34" t="n"/>
+      <c r="F80" s="34" t="n"/>
+      <c r="G80" s="34" t="n"/>
+      <c r="H80" s="34" t="n"/>
+      <c r="I80" s="34" t="n"/>
+      <c r="J80" s="34" t="n"/>
+      <c r="K80" s="34" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1" s="20">
-      <c r="A81" s="44" t="inlineStr">
+      <c r="A81" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Food — Per-person Spend</t>
         </is>
       </c>
-      <c r="B81" s="45" t="n">
+      <c r="B81" s="52" t="n">
         <v>50</v>
       </c>
-      <c r="C81" s="42" t="n"/>
-      <c r="D81" s="42" t="n"/>
-      <c r="E81" s="42" t="n"/>
-      <c r="F81" s="42" t="n"/>
-      <c r="G81" s="42" t="n"/>
-      <c r="H81" s="42" t="n"/>
-      <c r="I81" s="42" t="n"/>
-      <c r="J81" s="42" t="n"/>
-      <c r="K81" s="42" t="n"/>
+      <c r="C81" s="34" t="n"/>
+      <c r="D81" s="34" t="n"/>
+      <c r="E81" s="34" t="n"/>
+      <c r="F81" s="34" t="n"/>
+      <c r="G81" s="34" t="n"/>
+      <c r="H81" s="34" t="n"/>
+      <c r="I81" s="34" t="n"/>
+      <c r="J81" s="34" t="n"/>
+      <c r="K81" s="34" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1" s="20">
-      <c r="A82" s="44" t="inlineStr">
+      <c r="A82" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Food — Share Rate</t>
         </is>
       </c>
-      <c r="B82" s="46" t="n">
+      <c r="B82" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C82" s="42" t="n"/>
-      <c r="D82" s="42" t="n"/>
-      <c r="E82" s="42" t="n"/>
-      <c r="F82" s="42" t="n"/>
-      <c r="G82" s="42" t="n"/>
-      <c r="H82" s="42" t="n"/>
-      <c r="I82" s="42" t="n"/>
-      <c r="J82" s="42" t="n"/>
-      <c r="K82" s="42" t="n"/>
+      <c r="C82" s="34" t="n"/>
+      <c r="D82" s="34" t="n"/>
+      <c r="E82" s="34" t="n"/>
+      <c r="F82" s="34" t="n"/>
+      <c r="G82" s="34" t="n"/>
+      <c r="H82" s="34" t="n"/>
+      <c r="I82" s="34" t="n"/>
+      <c r="J82" s="34" t="n"/>
+      <c r="K82" s="34" t="n"/>
     </row>
     <row r="83" ht="15" customHeight="1" s="20">
-      <c r="A83" s="44" t="inlineStr">
+      <c r="A83" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Food — Est. Total Sales (reference)</t>
         </is>
       </c>
-      <c r="B83" s="47">
+      <c r="B83" s="53">
         <f>B80*B81</f>
         <v/>
       </c>
-      <c r="C83" s="47">
+      <c r="C83" s="53">
         <f>B83*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="D83" s="47">
+      <c r="D83" s="53">
         <f>C83*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="E83" s="47">
+      <c r="E83" s="53">
         <f>D83*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="F83" s="47">
+      <c r="F83" s="53">
         <f>E83*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="G83" s="47">
+      <c r="G83" s="53">
         <f>F83*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="H83" s="47">
+      <c r="H83" s="53">
         <f>G83*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="I83" s="47">
+      <c r="I83" s="53">
         <f>H83*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="J83" s="47">
+      <c r="J83" s="53">
         <f>I83*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="K83" s="47">
+      <c r="K83" s="53">
         <f>J83*(1+$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="48" t="inlineStr">
+      <c r="A84" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Day: Food — Aura Revenue</t>
         </is>
       </c>
-      <c r="B84" s="42">
+      <c r="B84" s="34">
         <f>B83*$B82</f>
         <v/>
       </c>
-      <c r="C84" s="42">
+      <c r="C84" s="34">
         <f>C83*$B82</f>
         <v/>
       </c>
-      <c r="D84" s="42">
+      <c r="D84" s="34">
         <f>D83*$B82</f>
         <v/>
       </c>
-      <c r="E84" s="42">
+      <c r="E84" s="34">
         <f>E83*$B82</f>
         <v/>
       </c>
-      <c r="F84" s="42">
+      <c r="F84" s="34">
         <f>F83*$B82</f>
         <v/>
       </c>
-      <c r="G84" s="42">
+      <c r="G84" s="34">
         <f>G83*$B82</f>
         <v/>
       </c>
-      <c r="H84" s="42">
+      <c r="H84" s="34">
         <f>H83*$B82</f>
         <v/>
       </c>
-      <c r="I84" s="42">
+      <c r="I84" s="34">
         <f>I83*$B82</f>
         <v/>
       </c>
-      <c r="J84" s="42">
+      <c r="J84" s="34">
         <f>J83*$B82</f>
         <v/>
       </c>
-      <c r="K84" s="42">
+      <c r="K84" s="34">
         <f>K83*$B82</f>
         <v/>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="20">
-      <c r="A85" s="40" t="n"/>
-      <c r="B85" s="49" t="n"/>
-      <c r="C85" s="49" t="n"/>
-      <c r="D85" s="49" t="n"/>
-      <c r="E85" s="49" t="n"/>
-      <c r="F85" s="49" t="n"/>
-      <c r="G85" s="49" t="n"/>
-      <c r="H85" s="49" t="n"/>
-      <c r="I85" s="49" t="n"/>
-      <c r="J85" s="49" t="n"/>
-      <c r="K85" s="49" t="n"/>
+      <c r="A85" s="33" t="n"/>
+      <c r="B85" s="54" t="n"/>
+      <c r="C85" s="54" t="n"/>
+      <c r="D85" s="54" t="n"/>
+      <c r="E85" s="54" t="n"/>
+      <c r="F85" s="54" t="n"/>
+      <c r="G85" s="54" t="n"/>
+      <c r="H85" s="54" t="n"/>
+      <c r="I85" s="54" t="n"/>
+      <c r="J85" s="54" t="n"/>
+      <c r="K85" s="54" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="48" t="inlineStr">
+      <c r="A86" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Night: Drinks — Guest Count</t>
         </is>
       </c>
-      <c r="B86" s="50" t="n">
+      <c r="B86" s="42" t="n">
         <v>150</v>
       </c>
-      <c r="C86" s="42" t="n"/>
-      <c r="D86" s="42" t="n"/>
-      <c r="E86" s="42" t="n"/>
-      <c r="F86" s="42" t="n"/>
-      <c r="G86" s="42" t="n"/>
-      <c r="H86" s="42" t="n"/>
-      <c r="I86" s="42" t="n"/>
-      <c r="J86" s="42" t="n"/>
-      <c r="K86" s="42" t="n"/>
+      <c r="C86" s="34" t="n"/>
+      <c r="D86" s="34" t="n"/>
+      <c r="E86" s="34" t="n"/>
+      <c r="F86" s="34" t="n"/>
+      <c r="G86" s="34" t="n"/>
+      <c r="H86" s="34" t="n"/>
+      <c r="I86" s="34" t="n"/>
+      <c r="J86" s="34" t="n"/>
+      <c r="K86" s="34" t="n"/>
     </row>
     <row r="87" ht="15" customHeight="1" s="20">
-      <c r="A87" s="44" t="inlineStr">
+      <c r="A87" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Night: Drinks — Per-person Spend</t>
         </is>
       </c>
-      <c r="B87" s="51" t="n">
+      <c r="B87" s="55" t="n">
         <v>50</v>
       </c>
-      <c r="C87" s="40" t="n"/>
-      <c r="D87" s="40" t="n"/>
-      <c r="E87" s="40" t="n"/>
-      <c r="F87" s="40" t="n"/>
-      <c r="G87" s="40" t="n"/>
-      <c r="H87" s="40" t="n"/>
-      <c r="I87" s="40" t="n"/>
-      <c r="J87" s="40" t="n"/>
-      <c r="K87" s="40" t="n"/>
+      <c r="C87" s="33" t="n"/>
+      <c r="D87" s="33" t="n"/>
+      <c r="E87" s="33" t="n"/>
+      <c r="F87" s="33" t="n"/>
+      <c r="G87" s="33" t="n"/>
+      <c r="H87" s="33" t="n"/>
+      <c r="I87" s="33" t="n"/>
+      <c r="J87" s="33" t="n"/>
+      <c r="K87" s="33" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1" s="20">
-      <c r="A88" s="44" t="inlineStr">
+      <c r="A88" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Night: Drinks — Share Rate</t>
         </is>
       </c>
-      <c r="B88" s="52" t="n">
+      <c r="B88" s="56" t="n">
         <v>0</v>
       </c>
-      <c r="C88" s="53" t="n"/>
-      <c r="D88" s="53" t="n"/>
-      <c r="E88" s="53" t="n"/>
-      <c r="F88" s="53" t="n"/>
-      <c r="G88" s="53" t="n"/>
-      <c r="H88" s="53" t="n"/>
-      <c r="I88" s="53" t="n"/>
-      <c r="J88" s="53" t="n"/>
-      <c r="K88" s="53" t="n"/>
+      <c r="C88" s="57" t="n"/>
+      <c r="D88" s="57" t="n"/>
+      <c r="E88" s="57" t="n"/>
+      <c r="F88" s="57" t="n"/>
+      <c r="G88" s="57" t="n"/>
+      <c r="H88" s="57" t="n"/>
+      <c r="I88" s="57" t="n"/>
+      <c r="J88" s="57" t="n"/>
+      <c r="K88" s="57" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1" s="20">
-      <c r="A89" s="44" t="inlineStr">
+      <c r="A89" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Night: Drinks — Est. Total Sales (reference)</t>
         </is>
       </c>
-      <c r="B89" s="47">
+      <c r="B89" s="53">
         <f>B86*B87</f>
         <v/>
       </c>
-      <c r="C89" s="47">
+      <c r="C89" s="53">
         <f>B89*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="D89" s="47">
+      <c r="D89" s="53">
         <f>C89*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="E89" s="47">
+      <c r="E89" s="53">
         <f>D89*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="F89" s="47">
+      <c r="F89" s="53">
         <f>E89*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="G89" s="47">
+      <c r="G89" s="53">
         <f>F89*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="H89" s="47">
+      <c r="H89" s="53">
         <f>G89*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="I89" s="47">
+      <c r="I89" s="53">
         <f>H89*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="J89" s="47">
+      <c r="J89" s="53">
         <f>I89*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="K89" s="47">
+      <c r="K89" s="53">
         <f>J89*(1+$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="20">
-      <c r="A90" s="44" t="inlineStr">
+      <c r="A90" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Saturday Night: Drinks — Aura Revenue</t>
         </is>
       </c>
-      <c r="B90" s="42">
+      <c r="B90" s="34">
         <f>B89*$B88</f>
         <v/>
       </c>
-      <c r="C90" s="42">
+      <c r="C90" s="34">
         <f>C89*$B88</f>
         <v/>
       </c>
-      <c r="D90" s="42">
+      <c r="D90" s="34">
         <f>D89*$B88</f>
         <v/>
       </c>
-      <c r="E90" s="42">
+      <c r="E90" s="34">
         <f>E89*$B88</f>
         <v/>
       </c>
-      <c r="F90" s="42">
+      <c r="F90" s="34">
         <f>F89*$B88</f>
         <v/>
       </c>
-      <c r="G90" s="42">
+      <c r="G90" s="34">
         <f>G89*$B88</f>
         <v/>
       </c>
-      <c r="H90" s="42">
+      <c r="H90" s="34">
         <f>H89*$B88</f>
         <v/>
       </c>
-      <c r="I90" s="42">
+      <c r="I90" s="34">
         <f>I89*$B88</f>
         <v/>
       </c>
-      <c r="J90" s="42">
+      <c r="J90" s="34">
         <f>J89*$B88</f>
         <v/>
       </c>
-      <c r="K90" s="42">
+      <c r="K90" s="34">
         <f>K89*$B88</f>
         <v/>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="42" t="n"/>
-      <c r="B91" s="42" t="n"/>
-      <c r="C91" s="42" t="n"/>
-      <c r="D91" s="42" t="n"/>
-      <c r="E91" s="42" t="n"/>
-      <c r="F91" s="42" t="n"/>
-      <c r="G91" s="42" t="n"/>
-      <c r="H91" s="42" t="n"/>
-      <c r="I91" s="42" t="n"/>
-      <c r="J91" s="42" t="n"/>
-      <c r="K91" s="42" t="n"/>
+      <c r="A91" s="34" t="n"/>
+      <c r="B91" s="34" t="n"/>
+      <c r="C91" s="34" t="n"/>
+      <c r="D91" s="34" t="n"/>
+      <c r="E91" s="34" t="n"/>
+      <c r="F91" s="34" t="n"/>
+      <c r="G91" s="34" t="n"/>
+      <c r="H91" s="34" t="n"/>
+      <c r="I91" s="34" t="n"/>
+      <c r="J91" s="34" t="n"/>
+      <c r="K91" s="34" t="n"/>
     </row>
     <row r="92" ht="15" customHeight="1" s="20">
-      <c r="A92" s="44" t="inlineStr">
+      <c r="A92" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sunday Coffee — Guest Count</t>
         </is>
       </c>
-      <c r="B92" s="51" t="n">
+      <c r="B92" s="55" t="n">
         <v>80</v>
       </c>
-      <c r="C92" s="40" t="n"/>
-      <c r="D92" s="40" t="n"/>
-      <c r="E92" s="40" t="n"/>
-      <c r="F92" s="40" t="n"/>
-      <c r="G92" s="40" t="n"/>
-      <c r="H92" s="40" t="n"/>
-      <c r="I92" s="40" t="n"/>
-      <c r="J92" s="40" t="n"/>
-      <c r="K92" s="40" t="n"/>
+      <c r="C92" s="33" t="n"/>
+      <c r="D92" s="33" t="n"/>
+      <c r="E92" s="33" t="n"/>
+      <c r="F92" s="33" t="n"/>
+      <c r="G92" s="33" t="n"/>
+      <c r="H92" s="33" t="n"/>
+      <c r="I92" s="33" t="n"/>
+      <c r="J92" s="33" t="n"/>
+      <c r="K92" s="33" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1" s="20">
-      <c r="A93" s="44" t="inlineStr">
+      <c r="A93" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sunday Coffee — Per-person Spend</t>
         </is>
       </c>
-      <c r="B93" s="52" t="n">
+      <c r="B93" s="56" t="n">
         <v>8</v>
       </c>
-      <c r="C93" s="53" t="n"/>
-      <c r="D93" s="53" t="n"/>
-      <c r="E93" s="53" t="n"/>
-      <c r="F93" s="53" t="n"/>
-      <c r="G93" s="53" t="n"/>
-      <c r="H93" s="53" t="n"/>
-      <c r="I93" s="53" t="n"/>
-      <c r="J93" s="53" t="n"/>
-      <c r="K93" s="53" t="n"/>
+      <c r="C93" s="57" t="n"/>
+      <c r="D93" s="57" t="n"/>
+      <c r="E93" s="57" t="n"/>
+      <c r="F93" s="57" t="n"/>
+      <c r="G93" s="57" t="n"/>
+      <c r="H93" s="57" t="n"/>
+      <c r="I93" s="57" t="n"/>
+      <c r="J93" s="57" t="n"/>
+      <c r="K93" s="57" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1" s="20">
-      <c r="A94" s="44" t="inlineStr">
+      <c r="A94" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sunday Coffee — Share Rate</t>
         </is>
       </c>
-      <c r="B94" s="45" t="n">
+      <c r="B94" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="C94" s="47" t="n"/>
-      <c r="D94" s="47" t="n"/>
-      <c r="E94" s="47" t="n"/>
-      <c r="F94" s="47" t="n"/>
-      <c r="G94" s="47" t="n"/>
-      <c r="H94" s="47" t="n"/>
-      <c r="I94" s="47" t="n"/>
-      <c r="J94" s="47" t="n"/>
-      <c r="K94" s="47" t="n"/>
+      <c r="C94" s="53" t="n"/>
+      <c r="D94" s="53" t="n"/>
+      <c r="E94" s="53" t="n"/>
+      <c r="F94" s="53" t="n"/>
+      <c r="G94" s="53" t="n"/>
+      <c r="H94" s="53" t="n"/>
+      <c r="I94" s="53" t="n"/>
+      <c r="J94" s="53" t="n"/>
+      <c r="K94" s="53" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1" s="20">
-      <c r="A95" s="44" t="inlineStr">
+      <c r="A95" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sunday Coffee — Est. Total Sales (reference)</t>
         </is>
       </c>
-      <c r="B95" s="42">
+      <c r="B95" s="34">
         <f>B92*B93</f>
         <v/>
       </c>
-      <c r="C95" s="42">
+      <c r="C95" s="34">
         <f>B95*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="D95" s="42">
+      <c r="D95" s="34">
         <f>C95*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="E95" s="42">
+      <c r="E95" s="34">
         <f>D95*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="F95" s="42">
+      <c r="F95" s="34">
         <f>E95*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="G95" s="42">
+      <c r="G95" s="34">
         <f>F95*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="H95" s="42">
+      <c r="H95" s="34">
         <f>G95*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="I95" s="42">
+      <c r="I95" s="34">
         <f>H95*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="J95" s="42">
+      <c r="J95" s="34">
         <f>I95*(1+$B$9)</f>
         <v/>
       </c>
-      <c r="K95" s="42">
+      <c r="K95" s="34">
         <f>J95*(1+$B$9)</f>
         <v/>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="48" t="inlineStr">
+      <c r="A96" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sunday Coffee — Aura Revenue</t>
         </is>
       </c>
-      <c r="B96" s="42">
+      <c r="B96" s="34">
         <f>B95*$B94</f>
         <v/>
       </c>
-      <c r="C96" s="42">
+      <c r="C96" s="34">
         <f>C95*$B94</f>
         <v/>
       </c>
-      <c r="D96" s="42">
+      <c r="D96" s="34">
         <f>D95*$B94</f>
         <v/>
       </c>
-      <c r="E96" s="42">
+      <c r="E96" s="34">
         <f>E95*$B94</f>
         <v/>
       </c>
-      <c r="F96" s="42">
+      <c r="F96" s="34">
         <f>F95*$B94</f>
         <v/>
       </c>
-      <c r="G96" s="42">
+      <c r="G96" s="34">
         <f>G95*$B94</f>
         <v/>
       </c>
-      <c r="H96" s="42">
+      <c r="H96" s="34">
         <f>H95*$B94</f>
         <v/>
       </c>
-      <c r="I96" s="42">
+      <c r="I96" s="34">
         <f>I95*$B94</f>
         <v/>
       </c>
-      <c r="J96" s="42">
+      <c r="J96" s="34">
         <f>J95*$B94</f>
         <v/>
       </c>
-      <c r="K96" s="42">
+      <c r="K96" s="34">
         <f>K95*$B94</f>
         <v/>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="20">
-      <c r="A97" s="40" t="n"/>
-      <c r="B97" s="40" t="n"/>
-      <c r="C97" s="40" t="n"/>
-      <c r="D97" s="40" t="n"/>
-      <c r="E97" s="40" t="n"/>
-      <c r="F97" s="40" t="n"/>
-      <c r="G97" s="40" t="n"/>
-      <c r="H97" s="40" t="n"/>
-      <c r="I97" s="40" t="n"/>
-      <c r="J97" s="40" t="n"/>
-      <c r="K97" s="40" t="n"/>
+      <c r="A97" s="33" t="n"/>
+      <c r="B97" s="33" t="n"/>
+      <c r="C97" s="33" t="n"/>
+      <c r="D97" s="33" t="n"/>
+      <c r="E97" s="33" t="n"/>
+      <c r="F97" s="33" t="n"/>
+      <c r="G97" s="33" t="n"/>
+      <c r="H97" s="33" t="n"/>
+      <c r="I97" s="33" t="n"/>
+      <c r="J97" s="33" t="n"/>
+      <c r="K97" s="33" t="n"/>
     </row>
     <row r="98" ht="15" customHeight="1" s="20">
-      <c r="A98" s="54" t="inlineStr">
+      <c r="A98" s="36" t="inlineStr">
         <is>
           <t>Bar/F&amp;B Total</t>
         </is>
       </c>
-      <c r="B98" s="53">
+      <c r="B98" s="57">
         <f>B72+B78+B84+B90+B96</f>
         <v/>
       </c>
-      <c r="C98" s="53">
+      <c r="C98" s="57">
         <f>C72+C78+C84+C90+C96</f>
         <v/>
       </c>
-      <c r="D98" s="53">
+      <c r="D98" s="57">
         <f>D72+D78+D84+D90+D96</f>
         <v/>
       </c>
-      <c r="E98" s="53">
+      <c r="E98" s="57">
         <f>E72+E78+E84+E90+E96</f>
         <v/>
       </c>
-      <c r="F98" s="53">
+      <c r="F98" s="57">
         <f>F72+F78+F84+F90+F96</f>
         <v/>
       </c>
-      <c r="G98" s="53">
+      <c r="G98" s="57">
         <f>G72+G78+G84+G90+G96</f>
         <v/>
       </c>
-      <c r="H98" s="53">
+      <c r="H98" s="57">
         <f>H72+H78+H84+H90+H96</f>
         <v/>
       </c>
-      <c r="I98" s="53">
+      <c r="I98" s="57">
         <f>I72+I78+I84+I90+I96</f>
         <v/>
       </c>
-      <c r="J98" s="53">
+      <c r="J98" s="57">
         <f>J72+J78+J84+J90+J96</f>
         <v/>
       </c>
-      <c r="K98" s="53">
+      <c r="K98" s="57">
         <f>K72+K78+K84+K90+K96</f>
         <v/>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="20">
-      <c r="A99" s="40" t="n"/>
-      <c r="B99" s="49" t="n"/>
-      <c r="C99" s="49" t="n"/>
-      <c r="D99" s="49" t="n"/>
-      <c r="E99" s="49" t="n"/>
-      <c r="F99" s="49" t="n"/>
-      <c r="G99" s="49" t="n"/>
-      <c r="H99" s="49" t="n"/>
-      <c r="I99" s="49" t="n"/>
-      <c r="J99" s="49" t="n"/>
-      <c r="K99" s="49" t="n"/>
+      <c r="A99" s="33" t="n"/>
+      <c r="B99" s="54" t="n"/>
+      <c r="C99" s="54" t="n"/>
+      <c r="D99" s="54" t="n"/>
+      <c r="E99" s="54" t="n"/>
+      <c r="F99" s="54" t="n"/>
+      <c r="G99" s="54" t="n"/>
+      <c r="H99" s="54" t="n"/>
+      <c r="I99" s="54" t="n"/>
+      <c r="J99" s="54" t="n"/>
+      <c r="K99" s="54" t="n"/>
     </row>
     <row r="100" ht="15" customHeight="1" s="20">
-      <c r="A100" s="39" t="inlineStr">
+      <c r="A100" s="50" t="inlineStr">
         <is>
           <t>SECTION 5: DINNER REVENUE</t>
         </is>
       </c>
-      <c r="B100" s="47" t="n"/>
-      <c r="C100" s="47" t="n"/>
-      <c r="D100" s="47" t="n"/>
-      <c r="E100" s="47" t="n"/>
-      <c r="F100" s="47" t="n"/>
-      <c r="G100" s="47" t="n"/>
-      <c r="H100" s="47" t="n"/>
-      <c r="I100" s="47" t="n"/>
-      <c r="J100" s="47" t="n"/>
-      <c r="K100" s="47" t="n"/>
+      <c r="B100" s="53" t="n"/>
+      <c r="C100" s="53" t="n"/>
+      <c r="D100" s="53" t="n"/>
+      <c r="E100" s="53" t="n"/>
+      <c r="F100" s="53" t="n"/>
+      <c r="G100" s="53" t="n"/>
+      <c r="H100" s="53" t="n"/>
+      <c r="I100" s="53" t="n"/>
+      <c r="J100" s="53" t="n"/>
+      <c r="K100" s="53" t="n"/>
     </row>
     <row r="101" ht="15" customHeight="1" s="20">
-      <c r="A101" s="40" t="n"/>
-      <c r="B101" s="55" t="n">
+      <c r="A101" s="33" t="n"/>
+      <c r="B101" s="58" t="n">
         <v>2027</v>
       </c>
-      <c r="C101" s="55" t="n">
+      <c r="C101" s="58" t="n">
         <v>2028</v>
       </c>
-      <c r="D101" s="55" t="n">
+      <c r="D101" s="58" t="n">
         <v>2029</v>
       </c>
-      <c r="E101" s="55" t="n">
+      <c r="E101" s="58" t="n">
         <v>2030</v>
       </c>
-      <c r="F101" s="55" t="n">
+      <c r="F101" s="58" t="n">
         <v>2031</v>
       </c>
-      <c r="G101" s="55" t="n">
+      <c r="G101" s="58" t="n">
         <v>2032</v>
       </c>
-      <c r="H101" s="55" t="n">
+      <c r="H101" s="58" t="n">
         <v>2033</v>
       </c>
-      <c r="I101" s="55" t="n">
+      <c r="I101" s="58" t="n">
         <v>2034</v>
       </c>
-      <c r="J101" s="55" t="n">
+      <c r="J101" s="58" t="n">
         <v>2035</v>
       </c>
-      <c r="K101" s="55" t="n">
+      <c r="K101" s="58" t="n">
         <v>2036</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="48" t="inlineStr">
+      <c r="A102" s="41" t="inlineStr">
         <is>
           <t>Dinner Revenue (manual input)</t>
         </is>
       </c>
-      <c r="B102" s="56" t="n">
+      <c r="B102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="C102" s="56" t="n">
+      <c r="C102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="D102" s="56" t="n">
+      <c r="D102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="E102" s="56" t="n">
+      <c r="E102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="F102" s="56" t="n">
+      <c r="F102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G102" s="56" t="n">
+      <c r="G102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="H102" s="56" t="n">
+      <c r="H102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="I102" s="56" t="n">
+      <c r="I102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="J102" s="56" t="n">
+      <c r="J102" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="K102" s="56" t="n">
+      <c r="K102" s="59" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="57" t="inlineStr">
+      <c r="A103" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  BP: 'Dinner is invite-only, sponsor-funded, never sold.' If a dinner-specific sponsor appears, it goes under Partnerships.</t>
         </is>
@@ -5126,51 +5333,51 @@
     </row>
     <row r="104"/>
     <row r="105">
-      <c r="A105" s="58" t="inlineStr">
+      <c r="A105" s="60" t="inlineStr">
         <is>
           <t>SECTION 6: OTHER REVENUE</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="B106" s="59" t="n">
+      <c r="B106" s="61" t="n">
         <v>2027</v>
       </c>
-      <c r="C106" s="59" t="n">
+      <c r="C106" s="61" t="n">
         <v>2028</v>
       </c>
-      <c r="D106" s="59" t="n">
+      <c r="D106" s="61" t="n">
         <v>2029</v>
       </c>
-      <c r="E106" s="59" t="n">
+      <c r="E106" s="61" t="n">
         <v>2030</v>
       </c>
-      <c r="F106" s="59" t="n">
+      <c r="F106" s="61" t="n">
         <v>2031</v>
       </c>
-      <c r="G106" s="59" t="n">
+      <c r="G106" s="61" t="n">
         <v>2032</v>
       </c>
-      <c r="H106" s="59" t="n">
+      <c r="H106" s="61" t="n">
         <v>2033</v>
       </c>
-      <c r="I106" s="59" t="n">
+      <c r="I106" s="61" t="n">
         <v>2034</v>
       </c>
-      <c r="J106" s="59" t="n">
+      <c r="J106" s="61" t="n">
         <v>2035</v>
       </c>
-      <c r="K106" s="59" t="n">
+      <c r="K106" s="61" t="n">
         <v>2036</v>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="48" t="inlineStr">
+      <c r="A107" s="41" t="inlineStr">
         <is>
           <t>Other Revenue</t>
         </is>
       </c>
-      <c r="B107" s="56" t="n">
+      <c r="B107" s="59" t="n">
         <v>2000</v>
       </c>
       <c r="C107">
@@ -5211,7 +5418,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="57" t="inlineStr">
+      <c r="A108" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">  Other Revenue grows with General Inflation Rate (P&amp;L sheet). Contents: add-ons, upselling, merchandise.</t>
         </is>
@@ -5219,46 +5426,46 @@
     </row>
     <row r="109"/>
     <row r="110">
-      <c r="A110" s="58" t="inlineStr">
+      <c r="A110" s="60" t="inlineStr">
         <is>
           <t>REVENUE TOTALS</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="B111" s="59" t="n">
+      <c r="B111" s="61" t="n">
         <v>2027</v>
       </c>
-      <c r="C111" s="59" t="n">
+      <c r="C111" s="61" t="n">
         <v>2028</v>
       </c>
-      <c r="D111" s="59" t="n">
+      <c r="D111" s="61" t="n">
         <v>2029</v>
       </c>
-      <c r="E111" s="59" t="n">
+      <c r="E111" s="61" t="n">
         <v>2030</v>
       </c>
-      <c r="F111" s="59" t="n">
+      <c r="F111" s="61" t="n">
         <v>2031</v>
       </c>
-      <c r="G111" s="59" t="n">
+      <c r="G111" s="61" t="n">
         <v>2032</v>
       </c>
-      <c r="H111" s="59" t="n">
+      <c r="H111" s="61" t="n">
         <v>2033</v>
       </c>
-      <c r="I111" s="59" t="n">
+      <c r="I111" s="61" t="n">
         <v>2034</v>
       </c>
-      <c r="J111" s="59" t="n">
+      <c r="J111" s="61" t="n">
         <v>2035</v>
       </c>
-      <c r="K111" s="59" t="n">
+      <c r="K111" s="61" t="n">
         <v>2036</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="59" t="inlineStr">
+      <c r="A112" s="61" t="inlineStr">
         <is>
           <t>TOTAL WINTER REVENUE</t>
         </is>
@@ -5305,7 +5512,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="59" t="inlineStr">
+      <c r="A113" s="61" t="inlineStr">
         <is>
           <t>Summer Revenue</t>
         </is>
@@ -5352,7 +5559,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="59" t="inlineStr">
+      <c r="A114" s="61" t="inlineStr">
         <is>
           <t>TOTAL ANNUAL REVENUE</t>
         </is>
@@ -5451,7 +5658,7 @@
           <t>General Inflation Rate</t>
         </is>
       </c>
-      <c r="B4" s="34" t="n">
+      <c r="B4" s="47" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -5461,7 +5668,7 @@
           <t>Tax Rate (Uri canton combined)</t>
         </is>
       </c>
-      <c r="B5" s="34" t="n">
+      <c r="B5" s="47" t="n">
         <v>0.1264</v>
       </c>
     </row>
@@ -5471,7 +5678,7 @@
           <t>Initial Capital (GmbH paid-in)</t>
         </is>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="B6" s="45" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -5863,16 +6070,16 @@
           <t>Costs</t>
         </is>
       </c>
-      <c r="B19" s="60" t="n"/>
-      <c r="C19" s="60" t="n"/>
-      <c r="D19" s="60" t="n"/>
-      <c r="E19" s="60" t="n"/>
-      <c r="F19" s="60" t="n"/>
-      <c r="G19" s="60" t="n"/>
-      <c r="H19" s="60" t="n"/>
-      <c r="I19" s="60" t="n"/>
-      <c r="J19" s="60" t="n"/>
-      <c r="K19" s="60" t="n"/>
+      <c r="B19" s="62" t="n"/>
+      <c r="C19" s="62" t="n"/>
+      <c r="D19" s="62" t="n"/>
+      <c r="E19" s="62" t="n"/>
+      <c r="F19" s="62" t="n"/>
+      <c r="G19" s="62" t="n"/>
+      <c r="H19" s="62" t="n"/>
+      <c r="I19" s="62" t="n"/>
+      <c r="J19" s="62" t="n"/>
+      <c r="K19" s="62" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="20">
       <c r="A20" s="24" t="inlineStr">
@@ -6299,7 +6506,7 @@
     </row>
     <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="20">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>MODEL ASSUMPTIONS</t>
         </is>
@@ -6321,7 +6528,7 @@
           <t>Venue Contract Escalation Rate</t>
         </is>
       </c>
-      <c r="B4" s="34" t="n">
+      <c r="B4" s="47" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -6331,7 +6538,7 @@
           <t>Ambition Growth Rate (Category C)</t>
         </is>
       </c>
-      <c r="B5" s="34" t="n">
+      <c r="B5" s="47" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -6341,41 +6548,41 @@
           <t>Contingency %</t>
         </is>
       </c>
-      <c r="B6" s="34" t="n">
+      <c r="B6" s="47" t="n">
         <v>0.09</v>
       </c>
     </row>
     <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="20">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="49" t="inlineStr">
         <is>
           <t>COST CATEGORY DEFINITIONS:</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="20">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="A9" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Category A (Fixed/Contract): Costs driven by contracts or predictable obligations. Grow at contractual rate or general inflation.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="20">
-      <c r="A10" s="33" t="inlineStr">
+      <c r="A10" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Category B (Guest-linked): Costs that scale with the number of ticket holders. More tickets sold = higher cost.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="20">
-      <c r="A11" s="33" t="inlineStr">
+      <c r="A11" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Category C (Ambition-linked): Costs tied to the quality and ambition of the event. Default growth: Ambition Growth Rate above.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="20">
-      <c r="A12" s="33" t="inlineStr">
+      <c r="A12" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Contingency: A buffer calculated as % of total costs (A+B+C) for unexpected expenses.</t>
         </is>
@@ -6438,7 +6645,7 @@
           <t xml:space="preserve">  Venue (Swiss House)</t>
         </is>
       </c>
-      <c r="B16" s="37" t="n">
+      <c r="B16" s="45" t="n">
         <v>27951</v>
       </c>
       <c r="C16" s="29">
@@ -6484,7 +6691,7 @@
           <t xml:space="preserve">  F&amp;B Credit (guest spend vs minimums)</t>
         </is>
       </c>
-      <c r="B17" s="37" t="n">
+      <c r="B17" s="45" t="n">
         <v>-9000</v>
       </c>
       <c r="C17" s="29">
@@ -6530,7 +6737,7 @@
           <t xml:space="preserve">  Insurance / Permits / Ticketing</t>
         </is>
       </c>
-      <c r="B18" s="37" t="n">
+      <c r="B18" s="45" t="n">
         <v>2500</v>
       </c>
       <c r="C18" s="29">
@@ -6576,7 +6783,7 @@
           <t xml:space="preserve">  Transport</t>
         </is>
       </c>
-      <c r="B19" s="37" t="n">
+      <c r="B19" s="45" t="n">
         <v>2500</v>
       </c>
       <c r="C19" s="29">
@@ -6622,7 +6829,7 @@
           <t xml:space="preserve">  Sunday Program (incl. GRÜEZI coffee costs)</t>
         </is>
       </c>
-      <c r="B20" s="37" t="n">
+      <c r="B20" s="45" t="n">
         <v>1000</v>
       </c>
       <c r="C20" s="29">
@@ -6767,7 +6974,7 @@
           <t xml:space="preserve">  Welcome Drinks (Ticket Count × 2 × CHF 9)</t>
         </is>
       </c>
-      <c r="B26" s="37" t="n">
+      <c r="B26" s="45" t="n">
         <v>4500</v>
       </c>
       <c r="C26" s="29">
@@ -6813,7 +7020,7 @@
           <t xml:space="preserve">  Security</t>
         </is>
       </c>
-      <c r="B27" s="37" t="n">
+      <c r="B27" s="45" t="n">
         <v>4500</v>
       </c>
       <c r="C27" s="29">
@@ -6958,7 +7165,7 @@
           <t xml:space="preserve">  Talent (DJs / Artists)</t>
         </is>
       </c>
-      <c r="B33" s="37" t="n">
+      <c r="B33" s="45" t="n">
         <v>18000</v>
       </c>
       <c r="C33" s="29">
@@ -7004,7 +7211,7 @@
           <t xml:space="preserve">  Production (Sound / Lighting)</t>
         </is>
       </c>
-      <c r="B34" s="37" t="n">
+      <c r="B34" s="45" t="n">
         <v>12000</v>
       </c>
       <c r="C34" s="29">
@@ -7050,7 +7257,7 @@
           <t xml:space="preserve">  Decor / Branding</t>
         </is>
       </c>
-      <c r="B35" s="37" t="n">
+      <c r="B35" s="45" t="n">
         <v>3500</v>
       </c>
       <c r="C35" s="29">
@@ -7096,7 +7303,7 @@
           <t xml:space="preserve">  Photo / Video</t>
         </is>
       </c>
-      <c r="B36" s="37" t="n">
+      <c r="B36" s="45" t="n">
         <v>5000</v>
       </c>
       <c r="C36" s="29">
@@ -7142,7 +7349,7 @@
           <t xml:space="preserve">  Marketing / Print</t>
         </is>
       </c>
-      <c r="B37" s="37" t="n">
+      <c r="B37" s="45" t="n">
         <v>2000</v>
       </c>
       <c r="C37" s="29">
@@ -7188,7 +7395,7 @@
           <t xml:space="preserve">  Operating Partner</t>
         </is>
       </c>
-      <c r="B38" s="37" t="n">
+      <c r="B38" s="45" t="n">
         <v>6000</v>
       </c>
       <c r="C38" s="29">
@@ -7234,7 +7441,7 @@
           <t xml:space="preserve">  Chedi Winter Garden (Friday)</t>
         </is>
       </c>
-      <c r="B39" s="37" t="n">
+      <c r="B39" s="45" t="n">
         <v>2500</v>
       </c>
       <c r="C39" s="29">
@@ -7665,39 +7872,39 @@
           <t>Overhead (manual input)</t>
         </is>
       </c>
-      <c r="B53" s="37" t="n">
+      <c r="B53" s="45" t="n">
         <v>8000</v>
       </c>
-      <c r="C53" s="37" t="n">
+      <c r="C53" s="45" t="n">
         <v>8000</v>
       </c>
-      <c r="D53" s="37" t="n">
+      <c r="D53" s="45" t="n">
         <v>8000</v>
       </c>
-      <c r="E53" s="37" t="n">
+      <c r="E53" s="45" t="n">
         <v>39000</v>
       </c>
-      <c r="F53" s="37" t="n">
+      <c r="F53" s="45" t="n">
         <v>39000</v>
       </c>
-      <c r="G53" s="37" t="n">
+      <c r="G53" s="45" t="n">
         <v>39000</v>
       </c>
-      <c r="H53" s="37" t="n">
+      <c r="H53" s="45" t="n">
         <v>55000</v>
       </c>
-      <c r="I53" s="37" t="n">
+      <c r="I53" s="45" t="n">
         <v>56000</v>
       </c>
-      <c r="J53" s="37" t="n">
+      <c r="J53" s="45" t="n">
         <v>58000</v>
       </c>
-      <c r="K53" s="37" t="n">
+      <c r="K53" s="45" t="n">
         <v>60000</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="20">
-      <c r="A54" s="33" t="inlineStr">
+      <c r="A54" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  Overhead jumps when new hires are added (part-time producer in 2030, additional staff in 2033). Cannot be modeled with a growth rate.</t>
         </is>
@@ -7709,19 +7916,19 @@
           <t>Founder Pay (2027-2031: manual / 2032+: auto +4%/yr)</t>
         </is>
       </c>
-      <c r="B55" s="37" t="n">
+      <c r="B55" s="45" t="n">
         <v>10000</v>
       </c>
-      <c r="C55" s="37" t="n">
+      <c r="C55" s="45" t="n">
         <v>20000</v>
       </c>
-      <c r="D55" s="37" t="n">
+      <c r="D55" s="45" t="n">
         <v>30000</v>
       </c>
-      <c r="E55" s="37" t="n">
+      <c r="E55" s="45" t="n">
         <v>50000</v>
       </c>
-      <c r="F55" s="37" t="n">
+      <c r="F55" s="45" t="n">
         <v>70000</v>
       </c>
       <c r="G55" s="29">
@@ -7747,7 +7954,7 @@
     </row>
     <row r="56"/>
     <row r="57">
-      <c r="A57" s="58" t="inlineStr">
+      <c r="A57" s="60" t="inlineStr">
         <is>
           <t>TOTAL COST</t>
         </is>

</xml_diff>

<commit_message>
Add cost control factors to Downside scenario
Add Direct Cost Factor (DS=0.80), fixed Downside Overhead (8K CHF),
reflecting realistic cost management in a downside world — no new hires,
20% direct cost reduction. Downside now recovers to profitability by 2029
(summer edition start) with 10-year cumulative cash +169K CHF, vs the
previous -419K with uncontrolled costs.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -322,9 +322,7 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -1213,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:K76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="35" customWidth="1" style="19" min="1" max="1"/>
@@ -1509,43 +1507,43 @@
         </is>
       </c>
       <c r="B15" s="25">
-        <f>(B12+B13+B14)*(1+IF(2027&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(B12+B13+B14)*(1+IF(2027&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="C15" s="25">
-        <f>(C12+C13+C14)*(1+IF(2028&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(C12+C13+C14)*(1+IF(2028&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="D15" s="25">
-        <f>(D12+D13+D14)*(1+IF(2029&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(D12+D13+D14)*(1+IF(2029&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="E15" s="25">
-        <f>(E12+E13+E14)*(1+IF(2030&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(E12+E13+E14)*(1+IF(2030&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="F15" s="25">
-        <f>(F12+F13+F14)*(1+IF(2031&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(F12+F13+F14)*(1+IF(2031&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="G15" s="25">
-        <f>(G12+G13+G14)*(1+IF(2032&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(G12+G13+G14)*(1+IF(2032&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="H15" s="25">
-        <f>(H12+H13+H14)*(1+IF(2033&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(H12+H13+H14)*(1+IF(2033&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="I15" s="25">
-        <f>(I12+I13+I14)*(1+IF(2034&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(I12+I13+I14)*(1+IF(2034&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="J15" s="25">
-        <f>(J12+J13+J14)*(1+IF(2035&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(J12+J13+J14)*(1+IF(2035&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="K15" s="25">
-        <f>(K12+K13+K14)*(1+IF(2036&gt;=$C$66,Revenue!$B$11,0))</f>
+        <f>(K12+K13+K14)*(1+IF(2036&gt;=$C$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
     </row>
@@ -1556,43 +1554,43 @@
         </is>
       </c>
       <c r="B16" s="29">
-        <f>'P&amp;L'!B20+'P&amp;L'!B21+'P&amp;L'!B22*$C$67</f>
+        <f>'P&amp;L'!B20*$C$66+'P&amp;L'!B21+'P&amp;L'!B22*$C$67</f>
         <v/>
       </c>
       <c r="C16" s="29">
-        <f>'P&amp;L'!C20+'P&amp;L'!C21+'P&amp;L'!C22*$C$67</f>
+        <f>'P&amp;L'!C20*$C$66+'P&amp;L'!C21+'P&amp;L'!C22*$C$67</f>
         <v/>
       </c>
       <c r="D16" s="29">
-        <f>'P&amp;L'!D20+'P&amp;L'!D21+'P&amp;L'!D22*$C$67</f>
+        <f>'P&amp;L'!D20*$C$66+'P&amp;L'!D21+'P&amp;L'!D22*$C$67</f>
         <v/>
       </c>
       <c r="E16" s="29">
-        <f>'P&amp;L'!E20+'P&amp;L'!E21+'P&amp;L'!E22*$C$67</f>
+        <f>'P&amp;L'!E20*$C$66+'P&amp;L'!E21+'P&amp;L'!E22*$C$67</f>
         <v/>
       </c>
       <c r="F16" s="29">
-        <f>'P&amp;L'!F20+'P&amp;L'!F21+'P&amp;L'!F22*$C$67</f>
+        <f>'P&amp;L'!F20*$C$66+'P&amp;L'!F21+'P&amp;L'!F22*$C$67</f>
         <v/>
       </c>
       <c r="G16" s="29">
-        <f>'P&amp;L'!G20+'P&amp;L'!G21+'P&amp;L'!G22*$C$67</f>
+        <f>'P&amp;L'!G20*$C$66+'P&amp;L'!G21+'P&amp;L'!G22*$C$67</f>
         <v/>
       </c>
       <c r="H16" s="29">
-        <f>'P&amp;L'!H20+'P&amp;L'!H21+'P&amp;L'!H22*$C$67</f>
+        <f>'P&amp;L'!H20*$C$66+'P&amp;L'!H21+'P&amp;L'!H22*$C$67</f>
         <v/>
       </c>
       <c r="I16" s="29">
-        <f>'P&amp;L'!I20+'P&amp;L'!I21+'P&amp;L'!I22*$C$67</f>
+        <f>'P&amp;L'!I20*$C$66+'P&amp;L'!I21+'P&amp;L'!I22*$C$67</f>
         <v/>
       </c>
       <c r="J16" s="29">
-        <f>'P&amp;L'!J20+'P&amp;L'!J21+'P&amp;L'!J22*$C$67</f>
+        <f>'P&amp;L'!J20*$C$66+'P&amp;L'!J21+'P&amp;L'!J22*$C$67</f>
         <v/>
       </c>
       <c r="K16" s="29">
-        <f>'P&amp;L'!K20+'P&amp;L'!K21+'P&amp;L'!K22*$C$67</f>
+        <f>'P&amp;L'!K20*$C$66+'P&amp;L'!K21+'P&amp;L'!K22*$C$67</f>
         <v/>
       </c>
     </row>
@@ -1973,43 +1971,43 @@
         </is>
       </c>
       <c r="B27" s="25">
-        <f>(B24+B25+B26)*(1+IF(2027&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(B24+B25+B26)*(1+IF(2027&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="C27" s="25">
-        <f>(C24+C25+C26)*(1+IF(2028&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(C24+C25+C26)*(1+IF(2028&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="D27" s="25">
-        <f>(D24+D25+D26)*(1+IF(2029&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(D24+D25+D26)*(1+IF(2029&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="E27" s="25">
-        <f>(E24+E25+E26)*(1+IF(2030&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(E24+E25+E26)*(1+IF(2030&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="F27" s="25">
-        <f>(F24+F25+F26)*(1+IF(2031&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(F24+F25+F26)*(1+IF(2031&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="G27" s="25">
-        <f>(G24+G25+G26)*(1+IF(2032&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(G24+G25+G26)*(1+IF(2032&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="H27" s="25">
-        <f>(H24+H25+H26)*(1+IF(2033&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(H24+H25+H26)*(1+IF(2033&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="I27" s="25">
-        <f>(I24+I25+I26)*(1+IF(2034&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(I24+I25+I26)*(1+IF(2034&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="J27" s="25">
-        <f>(J24+J25+J26)*(1+IF(2035&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(J24+J25+J26)*(1+IF(2035&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="K27" s="25">
-        <f>(K24+K25+K26)*(1+IF(2036&gt;=$B$66,Revenue!$B$11,0))</f>
+        <f>(K24+K25+K26)*(1+IF(2036&gt;=$B$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
     </row>
@@ -2020,43 +2018,43 @@
         </is>
       </c>
       <c r="B28" s="29">
-        <f>'P&amp;L'!B20+'P&amp;L'!B21+'P&amp;L'!B22*$B$67</f>
+        <f>'P&amp;L'!B20*$B$66-$B$68+'P&amp;L'!B22*$B$67</f>
         <v/>
       </c>
       <c r="C28" s="29">
-        <f>'P&amp;L'!C20+'P&amp;L'!C21+'P&amp;L'!C22*$B$67</f>
+        <f>'P&amp;L'!C20*$B$66-$B$68+'P&amp;L'!C22*$B$67</f>
         <v/>
       </c>
       <c r="D28" s="29">
-        <f>'P&amp;L'!D20+'P&amp;L'!D21+'P&amp;L'!D22*$B$67</f>
+        <f>'P&amp;L'!D20*$B$66-$B$68+'P&amp;L'!D22*$B$67</f>
         <v/>
       </c>
       <c r="E28" s="29">
-        <f>'P&amp;L'!E20+'P&amp;L'!E21+'P&amp;L'!E22*$B$67</f>
+        <f>'P&amp;L'!E20*$B$66-$B$68+'P&amp;L'!E22*$B$67</f>
         <v/>
       </c>
       <c r="F28" s="29">
-        <f>'P&amp;L'!F20+'P&amp;L'!F21+'P&amp;L'!F22*$B$67</f>
+        <f>'P&amp;L'!F20*$B$66-$B$68+'P&amp;L'!F22*$B$67</f>
         <v/>
       </c>
       <c r="G28" s="29">
-        <f>'P&amp;L'!G20+'P&amp;L'!G21+'P&amp;L'!G22*$B$67</f>
+        <f>'P&amp;L'!G20*$B$66-$B$68+'P&amp;L'!G22*$B$67</f>
         <v/>
       </c>
       <c r="H28" s="29">
-        <f>'P&amp;L'!H20+'P&amp;L'!H21+'P&amp;L'!H22*$B$67</f>
+        <f>'P&amp;L'!H20*$B$66-$B$68+'P&amp;L'!H22*$B$67</f>
         <v/>
       </c>
       <c r="I28" s="29">
-        <f>'P&amp;L'!I20+'P&amp;L'!I21+'P&amp;L'!I22*$B$67</f>
+        <f>'P&amp;L'!I20*$B$66-$B$68+'P&amp;L'!I22*$B$67</f>
         <v/>
       </c>
       <c r="J28" s="29">
-        <f>'P&amp;L'!J20+'P&amp;L'!J21+'P&amp;L'!J22*$B$67</f>
+        <f>'P&amp;L'!J20*$B$66-$B$68+'P&amp;L'!J22*$B$67</f>
         <v/>
       </c>
       <c r="K28" s="29">
-        <f>'P&amp;L'!K20+'P&amp;L'!K21+'P&amp;L'!K22*$B$67</f>
+        <f>'P&amp;L'!K20*$B$66-$B$68+'P&amp;L'!K22*$B$67</f>
         <v/>
       </c>
     </row>
@@ -2437,43 +2435,43 @@
         </is>
       </c>
       <c r="B39" s="25">
-        <f>(B36+B37+B38)*(1+IF(2027&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(B36+B37+B38)*(1+IF(2027&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="C39" s="25">
-        <f>(C36+C37+C38)*(1+IF(2028&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(C36+C37+C38)*(1+IF(2028&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="D39" s="25">
-        <f>(D36+D37+D38)*(1+IF(2029&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(D36+D37+D38)*(1+IF(2029&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="E39" s="25">
-        <f>(E36+E37+E38)*(1+IF(2030&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(E36+E37+E38)*(1+IF(2030&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="F39" s="25">
-        <f>(F36+F37+F38)*(1+IF(2031&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(F36+F37+F38)*(1+IF(2031&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="G39" s="25">
-        <f>(G36+G37+G38)*(1+IF(2032&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(G36+G37+G38)*(1+IF(2032&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="H39" s="25">
-        <f>(H36+H37+H38)*(1+IF(2033&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(H36+H37+H38)*(1+IF(2033&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="I39" s="25">
-        <f>(I36+I37+I38)*(1+IF(2034&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(I36+I37+I38)*(1+IF(2034&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="J39" s="25">
-        <f>(J36+J37+J38)*(1+IF(2035&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(J36+J37+J38)*(1+IF(2035&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
       <c r="K39" s="25">
-        <f>(K36+K37+K38)*(1+IF(2036&gt;=$D$66,Revenue!$B$11,0))</f>
+        <f>(K36+K37+K38)*(1+IF(2036&gt;=$D$71,Revenue!$B$11,0))</f>
         <v/>
       </c>
     </row>
@@ -2484,43 +2482,43 @@
         </is>
       </c>
       <c r="B40" s="29">
-        <f>'P&amp;L'!B20+'P&amp;L'!B21+'P&amp;L'!B22*$D$67</f>
+        <f>'P&amp;L'!B20*$D$66+'P&amp;L'!B21+'P&amp;L'!B22*$D$67</f>
         <v/>
       </c>
       <c r="C40" s="29">
-        <f>'P&amp;L'!C20+'P&amp;L'!C21+'P&amp;L'!C22*$D$67</f>
+        <f>'P&amp;L'!C20*$D$66+'P&amp;L'!C21+'P&amp;L'!C22*$D$67</f>
         <v/>
       </c>
       <c r="D40" s="29">
-        <f>'P&amp;L'!D20+'P&amp;L'!D21+'P&amp;L'!D22*$D$67</f>
+        <f>'P&amp;L'!D20*$D$66+'P&amp;L'!D21+'P&amp;L'!D22*$D$67</f>
         <v/>
       </c>
       <c r="E40" s="29">
-        <f>'P&amp;L'!E20+'P&amp;L'!E21+'P&amp;L'!E22*$D$67</f>
+        <f>'P&amp;L'!E20*$D$66+'P&amp;L'!E21+'P&amp;L'!E22*$D$67</f>
         <v/>
       </c>
       <c r="F40" s="29">
-        <f>'P&amp;L'!F20+'P&amp;L'!F21+'P&amp;L'!F22*$D$67</f>
+        <f>'P&amp;L'!F20*$D$66+'P&amp;L'!F21+'P&amp;L'!F22*$D$67</f>
         <v/>
       </c>
       <c r="G40" s="29">
-        <f>'P&amp;L'!G20+'P&amp;L'!G21+'P&amp;L'!G22*$D$67</f>
+        <f>'P&amp;L'!G20*$D$66+'P&amp;L'!G21+'P&amp;L'!G22*$D$67</f>
         <v/>
       </c>
       <c r="H40" s="29">
-        <f>'P&amp;L'!H20+'P&amp;L'!H21+'P&amp;L'!H22*$D$67</f>
+        <f>'P&amp;L'!H20*$D$66+'P&amp;L'!H21+'P&amp;L'!H22*$D$67</f>
         <v/>
       </c>
       <c r="I40" s="29">
-        <f>'P&amp;L'!I20+'P&amp;L'!I21+'P&amp;L'!I22*$D$67</f>
+        <f>'P&amp;L'!I20*$D$66+'P&amp;L'!I21+'P&amp;L'!I22*$D$67</f>
         <v/>
       </c>
       <c r="J40" s="29">
-        <f>'P&amp;L'!J20+'P&amp;L'!J21+'P&amp;L'!J22*$D$67</f>
+        <f>'P&amp;L'!J20*$D$66+'P&amp;L'!J21+'P&amp;L'!J22*$D$67</f>
         <v/>
       </c>
       <c r="K40" s="29">
-        <f>'P&amp;L'!K20+'P&amp;L'!K21+'P&amp;L'!K22*$D$67</f>
+        <f>'P&amp;L'!K20*$D$66+'P&amp;L'!K21+'P&amp;L'!K22*$D$67</f>
         <v/>
       </c>
     </row>
@@ -2919,7 +2917,7 @@
     <row r="65" ht="15" customHeight="1" s="20">
       <c r="A65" s="36" t="inlineStr">
         <is>
-          <t>■ STRUCTURAL FACTORS</t>
+          <t>■ COST FACTORS</t>
         </is>
       </c>
       <c r="B65" s="34" t="n"/>
@@ -2936,17 +2934,17 @@
     <row r="66" ht="15" customHeight="1" s="20">
       <c r="A66" s="38" t="inlineStr">
         <is>
-          <t>Summer Start Year</t>
+          <t>Direct Cost Factor</t>
         </is>
       </c>
       <c r="B66" s="42" t="n">
-        <v>2029</v>
+        <v>0.8</v>
       </c>
       <c r="C66" s="42" t="n">
-        <v>2027</v>
+        <v>1</v>
       </c>
       <c r="D66" s="42" t="n">
-        <v>2027</v>
+        <v>1</v>
       </c>
       <c r="E66" s="34" t="n"/>
       <c r="F66" s="34" t="n"/>
@@ -2980,8 +2978,14 @@
       <c r="K67" s="34" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="20">
-      <c r="A68" s="33" t="n"/>
-      <c r="B68" s="34" t="n"/>
+      <c r="A68" s="38" t="inlineStr">
+        <is>
+          <t>Downside Overhead (CHF)</t>
+        </is>
+      </c>
+      <c r="B68" s="42" t="n">
+        <v>8000</v>
+      </c>
       <c r="C68" s="34" t="n"/>
       <c r="D68" s="34" t="n"/>
       <c r="E68" s="34" t="n"/>
@@ -2993,11 +2997,7 @@
       <c r="K68" s="34" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="20">
-      <c r="A69" s="43" t="inlineStr">
-        <is>
-          <t>SCENARIO DEFINITIONS:</t>
-        </is>
-      </c>
+      <c r="A69" s="33" t="n"/>
       <c r="B69" s="34" t="n"/>
       <c r="C69" s="34" t="n"/>
       <c r="D69" s="34" t="n"/>
@@ -3010,9 +3010,9 @@
       <c r="K69" s="34" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="20">
-      <c r="A70" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Downside: Tickets 15% below plan, prices 10% lower, partnerships 40% lower, ASA 25% lower, summer from 2029, founder pay halved.</t>
+      <c r="A70" s="36" t="inlineStr">
+        <is>
+          <t>■ STRUCTURAL FACTORS</t>
         </is>
       </c>
       <c r="B70" s="34" t="n"/>
@@ -3027,14 +3027,20 @@
       <c r="K70" s="34" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Base: All factors at 1.0 — as entered in Revenue/Cost sheets. Summer from 2027.</t>
-        </is>
-      </c>
-      <c r="B71" s="34" t="n"/>
-      <c r="C71" s="34" t="n"/>
-      <c r="D71" s="34" t="n"/>
+      <c r="A71" s="41" t="inlineStr">
+        <is>
+          <t>Summer Start Year</t>
+        </is>
+      </c>
+      <c r="B71" s="42" t="n">
+        <v>2029</v>
+      </c>
+      <c r="C71" s="42" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D71" s="42" t="n">
+        <v>2027</v>
+      </c>
       <c r="E71" s="34" t="n"/>
       <c r="F71" s="34" t="n"/>
       <c r="G71" s="34" t="n"/>
@@ -3044,11 +3050,7 @@
       <c r="K71" s="34" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Upside: Prices 10% higher, partnerships 40% higher, ASA +25%. Summer from 2027.</t>
-        </is>
-      </c>
+      <c r="A72" s="34" t="n"/>
       <c r="B72" s="34" t="n"/>
       <c r="C72" s="34" t="n"/>
       <c r="D72" s="34" t="n"/>
@@ -3059,6 +3061,74 @@
       <c r="I72" s="34" t="n"/>
       <c r="J72" s="34" t="n"/>
       <c r="K72" s="34" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="43" t="inlineStr">
+        <is>
+          <t>SCENARIO DEFINITIONS:</t>
+        </is>
+      </c>
+      <c r="B73" s="34" t="n"/>
+      <c r="C73" s="34" t="n"/>
+      <c r="D73" s="34" t="n"/>
+      <c r="E73" s="34" t="n"/>
+      <c r="F73" s="34" t="n"/>
+      <c r="G73" s="34" t="n"/>
+      <c r="H73" s="34" t="n"/>
+      <c r="I73" s="34" t="n"/>
+      <c r="J73" s="34" t="n"/>
+      <c r="K73" s="34" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Downside: Tickets -15%, prices -10%, partnerships -40%, ASA -25%, direct costs ×0.8, overhead fixed 8K, founder pay halved, summer from 2029.</t>
+        </is>
+      </c>
+      <c r="B74" s="34" t="n"/>
+      <c r="C74" s="34" t="n"/>
+      <c r="D74" s="34" t="n"/>
+      <c r="E74" s="34" t="n"/>
+      <c r="F74" s="34" t="n"/>
+      <c r="G74" s="34" t="n"/>
+      <c r="H74" s="34" t="n"/>
+      <c r="I74" s="34" t="n"/>
+      <c r="J74" s="34" t="n"/>
+      <c r="K74" s="34" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Base: All factors at 1.0 — as entered in Revenue/Cost sheets. Summer from 2027.</t>
+        </is>
+      </c>
+      <c r="B75" s="34" t="n"/>
+      <c r="C75" s="34" t="n"/>
+      <c r="D75" s="34" t="n"/>
+      <c r="E75" s="34" t="n"/>
+      <c r="F75" s="34" t="n"/>
+      <c r="G75" s="34" t="n"/>
+      <c r="H75" s="34" t="n"/>
+      <c r="I75" s="34" t="n"/>
+      <c r="J75" s="34" t="n"/>
+      <c r="K75" s="34" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Upside: Prices +10%, partnerships +40%, ASA +25%. Summer from 2027.</t>
+        </is>
+      </c>
+      <c r="B76" s="34" t="n"/>
+      <c r="C76" s="34" t="n"/>
+      <c r="D76" s="34" t="n"/>
+      <c r="E76" s="34" t="n"/>
+      <c r="F76" s="34" t="n"/>
+      <c r="G76" s="34" t="n"/>
+      <c r="H76" s="34" t="n"/>
+      <c r="I76" s="34" t="n"/>
+      <c r="J76" s="34" t="n"/>
+      <c r="K76" s="34" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CC0B"/>

</xml_diff>

<commit_message>
Adjust Direct Cost Factor from 0.80 to 0.90 for realism
A 10% cost reduction is more realistic than 20% given that venue
contracts and insurance are fixed obligations. Founder pay halved
remains at 0.50 as defined in the Business Plan. Downside now shows
break-even over 10 years (cumulative cash ~20K CHF = initial capital).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PC2eaRJ4nQmnEGC6euTDhq
</commit_message>
<xml_diff>
--- a/Aura_Andermatt_10Year_Model.xlsx
+++ b/Aura_Andermatt_10Year_Model.xlsx
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="B66" s="42" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="C66" s="42" t="n">
         <v>1</v>
@@ -3082,7 +3082,7 @@
     <row r="74">
       <c r="A74" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Downside: Tickets -15%, prices -10%, partnerships -40%, ASA -25%, direct costs ×0.8, overhead fixed 8K, founder pay halved, summer from 2029.</t>
+          <t xml:space="preserve">  Downside: Tickets -15%, prices -10%, partnerships -40%, ASA -25%, direct costs ×0.9, overhead fixed 8K, founder pay halved (BP), summer from 2029.</t>
         </is>
       </c>
       <c r="B74" s="34" t="n"/>

</xml_diff>